<commit_message>
Another refit to UNAIDS data, to show that model is capable to refit to unaids
- Refit to UNAIDS
</commit_message>
<xml_diff>
--- a/data/All_clinics_data.xlsx
+++ b/data/All_clinics_data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10608"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10713"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://unsw-my.sharepoint.com/personal/z5288872_ad_unsw_edu_au/Documents/Modelling HIV [Quang]/PNG-Transmission-Model/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1704" documentId="13_ncr:1_{B01AED12-C7E5-C04A-9CE5-A2F269A7A508}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0C58D92E-D31B-7943-8A5F-35DFA3947DEA}"/>
+  <xr:revisionPtr revIDLastSave="1706" documentId="13_ncr:1_{B01AED12-C7E5-C04A-9CE5-A2F269A7A508}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{632C31A9-A870-CA40-92BB-35D4F8CAFFCB}"/>
   <bookViews>
-    <workbookView xWindow="-32400" yWindow="500" windowWidth="30220" windowHeight="21100" activeTab="4" xr2:uid="{2E625105-1FFC-624E-9A6F-F385E9B192AB}"/>
+    <workbookView xWindow="-32400" yWindow="500" windowWidth="30220" windowHeight="21100" activeTab="1" xr2:uid="{2E625105-1FFC-624E-9A6F-F385E9B192AB}"/>
   </bookViews>
   <sheets>
     <sheet name="(Hidden) Estimates" sheetId="2" state="hidden" r:id="rId1"/>
@@ -3353,14 +3353,17 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
@@ -3368,7 +3371,31 @@
     <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="5" fillId="3" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="2" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="2" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="3" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="3" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="3" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="3" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="3" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="5" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -3380,28 +3407,7 @@
     <xf numFmtId="49" fontId="5" fillId="2" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="5" fillId="3" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="49" fontId="5" fillId="2" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="2" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="2" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="3" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="3" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="3" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="5" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -3413,43 +3419,40 @@
     <xf numFmtId="49" fontId="5" fillId="3" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="5" fillId="3" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="5" fillId="3" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="37" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="37" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="49" fontId="5" fillId="0" borderId="10" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="38" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="39" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="5" fillId="0" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="39" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="38" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="49" fontId="5" fillId="0" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="5" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -3459,9 +3462,6 @@
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="5" fillId="0" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="5" fillId="0" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -3500,34 +3500,16 @@
     <xf numFmtId="0" fontId="12" fillId="5" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="4" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="4" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="4" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="4" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="4" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="9" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="9" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="25" fillId="9" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="9" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="25" fillId="9" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="9" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="7" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="7" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="8" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -3539,10 +3521,13 @@
     <xf numFmtId="0" fontId="22" fillId="8" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="25" fillId="4" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="25" fillId="9" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="25" fillId="4" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="25" fillId="4" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="4" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="9" fontId="25" fillId="4" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -3551,11 +3536,26 @@
     <xf numFmtId="9" fontId="25" fillId="4" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="7" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="25" fillId="4" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="7" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="25" fillId="4" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="9" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="9" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="4" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="4" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="4" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -4467,86 +4467,86 @@
       <c r="AY4" s="23"/>
     </row>
     <row r="5" spans="1:54" s="7" customFormat="1" ht="39.5" customHeight="1">
-      <c r="D5" s="140" t="s">
+      <c r="D5" s="141" t="s">
         <v>27</v>
       </c>
-      <c r="E5" s="140"/>
-      <c r="F5" s="140"/>
-      <c r="G5" s="141" t="s">
+      <c r="E5" s="141"/>
+      <c r="F5" s="141"/>
+      <c r="G5" s="140" t="s">
         <v>28</v>
       </c>
-      <c r="H5" s="141"/>
-      <c r="I5" s="141"/>
-      <c r="J5" s="140" t="s">
+      <c r="H5" s="140"/>
+      <c r="I5" s="140"/>
+      <c r="J5" s="141" t="s">
         <v>29</v>
       </c>
-      <c r="K5" s="140"/>
-      <c r="L5" s="140"/>
-      <c r="M5" s="141" t="s">
+      <c r="K5" s="141"/>
+      <c r="L5" s="141"/>
+      <c r="M5" s="140" t="s">
         <v>30</v>
       </c>
-      <c r="N5" s="141"/>
-      <c r="O5" s="141"/>
-      <c r="P5" s="140" t="s">
+      <c r="N5" s="140"/>
+      <c r="O5" s="140"/>
+      <c r="P5" s="141" t="s">
         <v>31</v>
       </c>
-      <c r="Q5" s="140"/>
-      <c r="R5" s="140"/>
-      <c r="S5" s="141" t="s">
+      <c r="Q5" s="141"/>
+      <c r="R5" s="141"/>
+      <c r="S5" s="140" t="s">
         <v>32</v>
       </c>
-      <c r="T5" s="141"/>
-      <c r="U5" s="141"/>
-      <c r="V5" s="140" t="s">
+      <c r="T5" s="140"/>
+      <c r="U5" s="140"/>
+      <c r="V5" s="141" t="s">
         <v>33</v>
       </c>
-      <c r="W5" s="140"/>
-      <c r="X5" s="140"/>
-      <c r="Y5" s="141" t="s">
+      <c r="W5" s="141"/>
+      <c r="X5" s="141"/>
+      <c r="Y5" s="140" t="s">
         <v>34</v>
       </c>
-      <c r="Z5" s="141"/>
-      <c r="AA5" s="141"/>
-      <c r="AB5" s="140" t="s">
+      <c r="Z5" s="140"/>
+      <c r="AA5" s="140"/>
+      <c r="AB5" s="141" t="s">
         <v>35</v>
       </c>
-      <c r="AC5" s="140"/>
-      <c r="AD5" s="140"/>
-      <c r="AE5" s="141" t="s">
+      <c r="AC5" s="141"/>
+      <c r="AD5" s="141"/>
+      <c r="AE5" s="140" t="s">
         <v>36</v>
       </c>
-      <c r="AF5" s="141"/>
-      <c r="AG5" s="141"/>
-      <c r="AH5" s="140" t="s">
+      <c r="AF5" s="140"/>
+      <c r="AG5" s="140"/>
+      <c r="AH5" s="141" t="s">
         <v>37</v>
       </c>
-      <c r="AI5" s="140"/>
-      <c r="AJ5" s="140"/>
-      <c r="AK5" s="141" t="s">
+      <c r="AI5" s="141"/>
+      <c r="AJ5" s="141"/>
+      <c r="AK5" s="140" t="s">
         <v>38</v>
       </c>
-      <c r="AL5" s="141"/>
-      <c r="AM5" s="141"/>
-      <c r="AN5" s="140" t="s">
+      <c r="AL5" s="140"/>
+      <c r="AM5" s="140"/>
+      <c r="AN5" s="141" t="s">
         <v>11</v>
       </c>
-      <c r="AO5" s="140"/>
-      <c r="AP5" s="140"/>
-      <c r="AQ5" s="141" t="s">
+      <c r="AO5" s="141"/>
+      <c r="AP5" s="141"/>
+      <c r="AQ5" s="140" t="s">
         <v>39</v>
       </c>
-      <c r="AR5" s="141"/>
-      <c r="AS5" s="141"/>
-      <c r="AT5" s="140" t="s">
+      <c r="AR5" s="140"/>
+      <c r="AS5" s="140"/>
+      <c r="AT5" s="141" t="s">
         <v>40</v>
       </c>
-      <c r="AU5" s="140"/>
-      <c r="AV5" s="140"/>
-      <c r="AW5" s="141" t="s">
+      <c r="AU5" s="141"/>
+      <c r="AV5" s="141"/>
+      <c r="AW5" s="140" t="s">
         <v>41</v>
       </c>
-      <c r="AX5" s="141"/>
-      <c r="AY5" s="141"/>
+      <c r="AX5" s="140"/>
+      <c r="AY5" s="140"/>
       <c r="AZ5" s="142" t="s">
         <v>99</v>
       </c>
@@ -9515,6 +9515,11 @@
     </row>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="D5:F5"/>
+    <mergeCell ref="G5:I5"/>
+    <mergeCell ref="J5:L5"/>
+    <mergeCell ref="M5:O5"/>
+    <mergeCell ref="P5:R5"/>
     <mergeCell ref="AE5:AG5"/>
     <mergeCell ref="AH5:AJ5"/>
     <mergeCell ref="AK5:AM5"/>
@@ -9527,11 +9532,6 @@
     <mergeCell ref="V5:X5"/>
     <mergeCell ref="Y5:AA5"/>
     <mergeCell ref="AB5:AD5"/>
-    <mergeCell ref="D5:F5"/>
-    <mergeCell ref="G5:I5"/>
-    <mergeCell ref="J5:L5"/>
-    <mergeCell ref="M5:O5"/>
-    <mergeCell ref="P5:R5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -9539,14 +9539,14 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1B60185D-CC42-3A43-A0D3-7E0EEA9302F5}">
-  <dimension ref="A1:AI150"/>
+  <dimension ref="A1:AK150"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.1640625" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="43.83203125" customWidth="1"/>
     <col min="2" max="2" width="13" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:35" s="37" customFormat="1">
+    <row r="1" spans="1:37" s="37" customFormat="1">
       <c r="A1" s="35"/>
       <c r="B1" s="36"/>
       <c r="C1" s="36">
@@ -9648,8 +9648,14 @@
       <c r="AI1" s="37">
         <v>2022</v>
       </c>
-    </row>
-    <row r="2" spans="1:35">
+      <c r="AJ1" s="37">
+        <v>2023</v>
+      </c>
+      <c r="AK1" s="37">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="2" spans="1:37">
       <c r="A2" s="7"/>
       <c r="B2" s="7"/>
       <c r="C2" s="28" t="s">
@@ -9746,7 +9752,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="3" spans="1:35" ht="30">
+    <row r="3" spans="1:37" ht="30">
       <c r="A3" s="7"/>
       <c r="B3" s="7"/>
       <c r="C3" s="28" t="s">
@@ -9843,7 +9849,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="4" spans="1:35">
+    <row r="4" spans="1:37">
       <c r="A4" s="47" t="s">
         <v>101</v>
       </c>
@@ -9880,7 +9886,7 @@
       <c r="AF4" s="28"/>
       <c r="AG4" s="28"/>
     </row>
-    <row r="5" spans="1:35">
+    <row r="5" spans="1:37">
       <c r="A5" s="53" t="s">
         <v>232</v>
       </c>
@@ -9936,7 +9942,7 @@
         <v>0.85</v>
       </c>
     </row>
-    <row r="6" spans="1:35">
+    <row r="6" spans="1:37">
       <c r="A6" s="53"/>
       <c r="B6" s="46" t="s">
         <v>22</v>
@@ -9980,7 +9986,7 @@
       <c r="AE6" s="29"/>
       <c r="AG6" s="29"/>
     </row>
-    <row r="7" spans="1:35">
+    <row r="7" spans="1:37">
       <c r="A7" s="53"/>
       <c r="B7" s="46" t="s">
         <v>23</v>
@@ -10024,7 +10030,7 @@
       <c r="AE7" s="29"/>
       <c r="AG7" s="29"/>
     </row>
-    <row r="8" spans="1:35" s="37" customFormat="1">
+    <row r="8" spans="1:37" s="37" customFormat="1">
       <c r="A8" s="49" t="s">
         <v>377</v>
       </c>
@@ -10064,7 +10070,7 @@
       <c r="AE8" s="36"/>
       <c r="AG8" s="72"/>
     </row>
-    <row r="9" spans="1:35" s="37" customFormat="1">
+    <row r="9" spans="1:37" s="37" customFormat="1">
       <c r="A9" s="49" t="s">
         <v>378</v>
       </c>
@@ -10103,7 +10109,7 @@
       <c r="AE9" s="36"/>
       <c r="AG9" s="72"/>
     </row>
-    <row r="10" spans="1:35">
+    <row r="10" spans="1:37">
       <c r="A10" s="53" t="s">
         <v>379</v>
       </c>
@@ -10138,7 +10144,7 @@
       <c r="AE10" s="28"/>
       <c r="AG10" s="29"/>
     </row>
-    <row r="11" spans="1:35" ht="45">
+    <row r="11" spans="1:37" ht="45">
       <c r="A11" s="53" t="s">
         <v>388</v>
       </c>
@@ -10176,7 +10182,7 @@
       <c r="AE11" s="28"/>
       <c r="AG11" s="29"/>
     </row>
-    <row r="12" spans="1:35">
+    <row r="12" spans="1:37">
       <c r="A12" s="53" t="s">
         <v>380</v>
       </c>
@@ -10217,7 +10223,7 @@
       <c r="AE12" s="28"/>
       <c r="AG12" s="29"/>
     </row>
-    <row r="13" spans="1:35">
+    <row r="13" spans="1:37">
       <c r="A13" s="53" t="s">
         <v>381</v>
       </c>
@@ -10256,8 +10262,8 @@
       <c r="AE13" s="28"/>
       <c r="AG13" s="29"/>
     </row>
-    <row r="14" spans="1:35" s="37" customFormat="1" ht="17" customHeight="1">
-      <c r="A14" s="144" t="s">
+    <row r="14" spans="1:37" s="37" customFormat="1" ht="17" customHeight="1">
+      <c r="A14" s="145" t="s">
         <v>376</v>
       </c>
       <c r="B14" s="130" t="s">
@@ -10297,8 +10303,8 @@
       <c r="AE14" s="36"/>
       <c r="AG14" s="72"/>
     </row>
-    <row r="15" spans="1:35" s="37" customFormat="1" ht="17" customHeight="1">
-      <c r="A15" s="144"/>
+    <row r="15" spans="1:37" s="37" customFormat="1" ht="17" customHeight="1">
+      <c r="A15" s="145"/>
       <c r="B15" s="130" t="s">
         <v>391</v>
       </c>
@@ -10336,7 +10342,7 @@
       <c r="AE15" s="36"/>
       <c r="AG15" s="72"/>
     </row>
-    <row r="16" spans="1:35" s="37" customFormat="1">
+    <row r="16" spans="1:37" s="37" customFormat="1">
       <c r="A16" s="49"/>
       <c r="B16" s="130"/>
       <c r="C16" s="36"/>
@@ -10407,7 +10413,7 @@
       <c r="B18" s="136"/>
     </row>
     <row r="19" spans="1:33">
-      <c r="A19" s="145"/>
+      <c r="A19" s="143"/>
       <c r="B19" s="45"/>
       <c r="C19" s="29"/>
       <c r="D19" s="29"/>
@@ -10442,7 +10448,7 @@
       <c r="AG19" s="29"/>
     </row>
     <row r="20" spans="1:33">
-      <c r="A20" s="145"/>
+      <c r="A20" s="143"/>
       <c r="B20" s="46"/>
       <c r="C20" s="30"/>
       <c r="D20" s="30"/>
@@ -10477,7 +10483,7 @@
       <c r="AG20" s="30"/>
     </row>
     <row r="21" spans="1:33">
-      <c r="A21" s="145"/>
+      <c r="A21" s="143"/>
       <c r="B21" s="46"/>
       <c r="C21" s="30"/>
       <c r="D21" s="30"/>
@@ -10512,7 +10518,7 @@
       <c r="AG21" s="30"/>
     </row>
     <row r="22" spans="1:33">
-      <c r="A22" s="145"/>
+      <c r="A22" s="143"/>
       <c r="B22" s="45"/>
       <c r="C22" s="29"/>
       <c r="D22" s="29"/>
@@ -10547,7 +10553,7 @@
       <c r="AG22" s="29"/>
     </row>
     <row r="23" spans="1:33">
-      <c r="A23" s="145"/>
+      <c r="A23" s="143"/>
       <c r="B23" s="46"/>
       <c r="C23" s="30"/>
       <c r="D23" s="30"/>
@@ -10582,7 +10588,7 @@
       <c r="AG23" s="30"/>
     </row>
     <row r="24" spans="1:33">
-      <c r="A24" s="145"/>
+      <c r="A24" s="143"/>
       <c r="B24" s="46"/>
       <c r="C24" s="30"/>
       <c r="D24" s="30"/>
@@ -10617,7 +10623,7 @@
       <c r="AG24" s="30"/>
     </row>
     <row r="25" spans="1:33">
-      <c r="A25" s="145"/>
+      <c r="A25" s="143"/>
       <c r="B25" s="45"/>
       <c r="C25" s="29"/>
       <c r="D25" s="29"/>
@@ -10652,7 +10658,7 @@
       <c r="AG25" s="29"/>
     </row>
     <row r="26" spans="1:33">
-      <c r="A26" s="145"/>
+      <c r="A26" s="143"/>
       <c r="B26" s="46"/>
       <c r="C26" s="30"/>
       <c r="D26" s="30"/>
@@ -10687,7 +10693,7 @@
       <c r="AG26" s="30"/>
     </row>
     <row r="27" spans="1:33">
-      <c r="A27" s="145"/>
+      <c r="A27" s="143"/>
       <c r="B27" s="46"/>
       <c r="C27" s="30"/>
       <c r="D27" s="30"/>
@@ -10792,7 +10798,7 @@
       <c r="AG29" s="30"/>
     </row>
     <row r="30" spans="1:33">
-      <c r="A30" s="145"/>
+      <c r="A30" s="143"/>
       <c r="B30" s="45"/>
       <c r="C30" s="29"/>
       <c r="D30" s="29"/>
@@ -10827,7 +10833,7 @@
       <c r="AG30" s="29"/>
     </row>
     <row r="31" spans="1:33">
-      <c r="A31" s="145"/>
+      <c r="A31" s="143"/>
       <c r="B31" s="46"/>
       <c r="C31" s="30"/>
       <c r="D31" s="30"/>
@@ -10862,7 +10868,7 @@
       <c r="AG31" s="30"/>
     </row>
     <row r="32" spans="1:33">
-      <c r="A32" s="145"/>
+      <c r="A32" s="143"/>
       <c r="B32" s="46"/>
       <c r="C32" s="30"/>
       <c r="D32" s="30"/>
@@ -10897,7 +10903,7 @@
       <c r="AG32" s="30"/>
     </row>
     <row r="33" spans="1:33">
-      <c r="A33" s="145"/>
+      <c r="A33" s="143"/>
       <c r="B33" s="45"/>
       <c r="C33" s="29"/>
       <c r="D33" s="29"/>
@@ -10932,7 +10938,7 @@
       <c r="AG33" s="29"/>
     </row>
     <row r="34" spans="1:33">
-      <c r="A34" s="145"/>
+      <c r="A34" s="143"/>
       <c r="B34" s="46"/>
       <c r="C34" s="30"/>
       <c r="D34" s="30"/>
@@ -10967,7 +10973,7 @@
       <c r="AG34" s="30"/>
     </row>
     <row r="35" spans="1:33">
-      <c r="A35" s="145"/>
+      <c r="A35" s="143"/>
       <c r="B35" s="46"/>
       <c r="C35" s="30"/>
       <c r="D35" s="30"/>
@@ -11002,7 +11008,7 @@
       <c r="AG35" s="30"/>
     </row>
     <row r="36" spans="1:33">
-      <c r="A36" s="145"/>
+      <c r="A36" s="143"/>
       <c r="B36" s="45"/>
       <c r="C36" s="29"/>
       <c r="D36" s="29"/>
@@ -11037,7 +11043,7 @@
       <c r="AG36" s="29"/>
     </row>
     <row r="37" spans="1:33">
-      <c r="A37" s="145"/>
+      <c r="A37" s="143"/>
       <c r="B37" s="46"/>
       <c r="C37" s="30"/>
       <c r="D37" s="30"/>
@@ -11072,7 +11078,7 @@
       <c r="AG37" s="30"/>
     </row>
     <row r="38" spans="1:33">
-      <c r="A38" s="145"/>
+      <c r="A38" s="143"/>
       <c r="B38" s="46"/>
       <c r="C38" s="30"/>
       <c r="D38" s="30"/>
@@ -11212,7 +11218,7 @@
       <c r="AG41" s="30"/>
     </row>
     <row r="42" spans="1:33">
-      <c r="A42" s="145"/>
+      <c r="A42" s="143"/>
       <c r="B42" s="45"/>
       <c r="C42" s="29"/>
       <c r="D42" s="29"/>
@@ -11247,7 +11253,7 @@
       <c r="AG42" s="29"/>
     </row>
     <row r="43" spans="1:33">
-      <c r="A43" s="145"/>
+      <c r="A43" s="143"/>
       <c r="B43" s="46"/>
       <c r="C43" s="30"/>
       <c r="D43" s="30"/>
@@ -11282,7 +11288,7 @@
       <c r="AG43" s="30"/>
     </row>
     <row r="44" spans="1:33">
-      <c r="A44" s="145"/>
+      <c r="A44" s="143"/>
       <c r="B44" s="46"/>
       <c r="C44" s="30"/>
       <c r="D44" s="30"/>
@@ -11317,7 +11323,7 @@
       <c r="AG44" s="30"/>
     </row>
     <row r="45" spans="1:33">
-      <c r="A45" s="145"/>
+      <c r="A45" s="143"/>
       <c r="B45" s="45"/>
       <c r="C45" s="29"/>
       <c r="D45" s="29"/>
@@ -11352,7 +11358,7 @@
       <c r="AG45" s="29"/>
     </row>
     <row r="46" spans="1:33">
-      <c r="A46" s="145"/>
+      <c r="A46" s="143"/>
       <c r="B46" s="46"/>
       <c r="C46" s="30"/>
       <c r="D46" s="30"/>
@@ -11387,7 +11393,7 @@
       <c r="AG46" s="30"/>
     </row>
     <row r="47" spans="1:33">
-      <c r="A47" s="145"/>
+      <c r="A47" s="143"/>
       <c r="B47" s="46"/>
       <c r="C47" s="30"/>
       <c r="D47" s="30"/>
@@ -11422,7 +11428,7 @@
       <c r="AG47" s="30"/>
     </row>
     <row r="48" spans="1:33">
-      <c r="A48" s="145"/>
+      <c r="A48" s="143"/>
       <c r="B48" s="45"/>
       <c r="C48" s="29"/>
       <c r="D48" s="29"/>
@@ -11457,7 +11463,7 @@
       <c r="AG48" s="29"/>
     </row>
     <row r="49" spans="1:33">
-      <c r="A49" s="145"/>
+      <c r="A49" s="143"/>
       <c r="B49" s="46"/>
       <c r="C49" s="30"/>
       <c r="D49" s="30"/>
@@ -11492,7 +11498,7 @@
       <c r="AG49" s="30"/>
     </row>
     <row r="50" spans="1:33">
-      <c r="A50" s="145"/>
+      <c r="A50" s="143"/>
       <c r="B50" s="46"/>
       <c r="C50" s="30"/>
       <c r="D50" s="30"/>
@@ -11632,7 +11638,7 @@
       <c r="AG53" s="51"/>
     </row>
     <row r="54" spans="1:33">
-      <c r="A54" s="145"/>
+      <c r="A54" s="143"/>
       <c r="B54" s="45"/>
       <c r="C54" s="29"/>
       <c r="D54" s="29"/>
@@ -11667,7 +11673,7 @@
       <c r="AG54" s="29"/>
     </row>
     <row r="55" spans="1:33">
-      <c r="A55" s="145"/>
+      <c r="A55" s="143"/>
       <c r="B55" s="46"/>
       <c r="C55" s="30"/>
       <c r="D55" s="30"/>
@@ -11702,7 +11708,7 @@
       <c r="AG55" s="30"/>
     </row>
     <row r="56" spans="1:33">
-      <c r="A56" s="145"/>
+      <c r="A56" s="143"/>
       <c r="B56" s="46"/>
       <c r="C56" s="30"/>
       <c r="D56" s="30"/>
@@ -11772,7 +11778,7 @@
       <c r="AG57" s="30"/>
     </row>
     <row r="58" spans="1:33">
-      <c r="A58" s="145"/>
+      <c r="A58" s="143"/>
       <c r="B58" s="45"/>
       <c r="C58" s="29"/>
       <c r="D58" s="29"/>
@@ -11807,7 +11813,7 @@
       <c r="AG58" s="29"/>
     </row>
     <row r="59" spans="1:33">
-      <c r="A59" s="145"/>
+      <c r="A59" s="143"/>
       <c r="B59" s="46"/>
       <c r="C59" s="30"/>
       <c r="D59" s="30"/>
@@ -11842,7 +11848,7 @@
       <c r="AG59" s="30"/>
     </row>
     <row r="60" spans="1:33">
-      <c r="A60" s="145"/>
+      <c r="A60" s="143"/>
       <c r="B60" s="46"/>
       <c r="C60" s="30"/>
       <c r="D60" s="30"/>
@@ -11877,7 +11883,7 @@
       <c r="AG60" s="30"/>
     </row>
     <row r="61" spans="1:33">
-      <c r="A61" s="145"/>
+      <c r="A61" s="143"/>
       <c r="B61" s="45"/>
       <c r="C61" s="29"/>
       <c r="D61" s="29"/>
@@ -11912,7 +11918,7 @@
       <c r="AG61" s="29"/>
     </row>
     <row r="62" spans="1:33">
-      <c r="A62" s="145"/>
+      <c r="A62" s="143"/>
       <c r="B62" s="46"/>
       <c r="C62" s="30"/>
       <c r="D62" s="30"/>
@@ -11947,7 +11953,7 @@
       <c r="AG62" s="30"/>
     </row>
     <row r="63" spans="1:33">
-      <c r="A63" s="145"/>
+      <c r="A63" s="143"/>
       <c r="B63" s="46"/>
       <c r="C63" s="30"/>
       <c r="D63" s="30"/>
@@ -11982,7 +11988,7 @@
       <c r="AG63" s="30"/>
     </row>
     <row r="64" spans="1:33">
-      <c r="A64" s="145"/>
+      <c r="A64" s="143"/>
       <c r="B64" s="45"/>
       <c r="C64" s="29"/>
       <c r="D64" s="29"/>
@@ -12017,7 +12023,7 @@
       <c r="AG64" s="29"/>
     </row>
     <row r="65" spans="1:33">
-      <c r="A65" s="145"/>
+      <c r="A65" s="143"/>
       <c r="B65" s="46"/>
       <c r="C65" s="30"/>
       <c r="D65" s="30"/>
@@ -12052,7 +12058,7 @@
       <c r="AG65" s="30"/>
     </row>
     <row r="66" spans="1:33">
-      <c r="A66" s="145"/>
+      <c r="A66" s="143"/>
       <c r="B66" s="46"/>
       <c r="C66" s="30"/>
       <c r="D66" s="30"/>
@@ -12087,7 +12093,7 @@
       <c r="AG66" s="30"/>
     </row>
     <row r="67" spans="1:33">
-      <c r="A67" s="145"/>
+      <c r="A67" s="143"/>
       <c r="B67" s="45"/>
       <c r="C67" s="29"/>
       <c r="D67" s="29"/>
@@ -12122,7 +12128,7 @@
       <c r="AG67" s="29"/>
     </row>
     <row r="68" spans="1:33">
-      <c r="A68" s="145"/>
+      <c r="A68" s="143"/>
       <c r="B68" s="46"/>
       <c r="C68" s="30"/>
       <c r="D68" s="30"/>
@@ -12157,7 +12163,7 @@
       <c r="AG68" s="30"/>
     </row>
     <row r="69" spans="1:33">
-      <c r="A69" s="145"/>
+      <c r="A69" s="143"/>
       <c r="B69" s="46"/>
       <c r="C69" s="30"/>
       <c r="D69" s="30"/>
@@ -12192,7 +12198,7 @@
       <c r="AG69" s="30"/>
     </row>
     <row r="70" spans="1:33">
-      <c r="A70" s="145"/>
+      <c r="A70" s="143"/>
       <c r="B70" s="45"/>
       <c r="C70" s="29"/>
       <c r="D70" s="29"/>
@@ -12227,7 +12233,7 @@
       <c r="AG70" s="29"/>
     </row>
     <row r="71" spans="1:33">
-      <c r="A71" s="145"/>
+      <c r="A71" s="143"/>
       <c r="B71" s="46"/>
       <c r="C71" s="30"/>
       <c r="D71" s="30"/>
@@ -12262,7 +12268,7 @@
       <c r="AG71" s="30"/>
     </row>
     <row r="72" spans="1:33">
-      <c r="A72" s="145"/>
+      <c r="A72" s="143"/>
       <c r="B72" s="46"/>
       <c r="C72" s="30"/>
       <c r="D72" s="30"/>
@@ -12297,7 +12303,7 @@
       <c r="AG72" s="30"/>
     </row>
     <row r="73" spans="1:33">
-      <c r="A73" s="145"/>
+      <c r="A73" s="143"/>
       <c r="B73" s="45"/>
       <c r="C73" s="29"/>
       <c r="D73" s="29"/>
@@ -12332,7 +12338,7 @@
       <c r="AG73" s="29"/>
     </row>
     <row r="74" spans="1:33">
-      <c r="A74" s="145"/>
+      <c r="A74" s="143"/>
       <c r="B74" s="46"/>
       <c r="C74" s="30"/>
       <c r="D74" s="30"/>
@@ -12367,7 +12373,7 @@
       <c r="AG74" s="30"/>
     </row>
     <row r="75" spans="1:33">
-      <c r="A75" s="145"/>
+      <c r="A75" s="143"/>
       <c r="B75" s="46"/>
       <c r="C75" s="30"/>
       <c r="D75" s="30"/>
@@ -12545,51 +12551,51 @@
       <c r="A81" s="48"/>
     </row>
     <row r="82" spans="1:33">
-      <c r="A82" s="145"/>
+      <c r="A82" s="143"/>
       <c r="B82" s="45"/>
     </row>
     <row r="83" spans="1:33">
-      <c r="A83" s="145"/>
+      <c r="A83" s="143"/>
       <c r="B83" s="46"/>
     </row>
     <row r="84" spans="1:33">
-      <c r="A84" s="145"/>
+      <c r="A84" s="143"/>
       <c r="B84" s="46"/>
     </row>
     <row r="85" spans="1:33">
-      <c r="A85" s="145"/>
+      <c r="A85" s="143"/>
       <c r="B85" s="45"/>
     </row>
     <row r="86" spans="1:33">
-      <c r="A86" s="145"/>
+      <c r="A86" s="143"/>
       <c r="B86" s="46"/>
     </row>
     <row r="87" spans="1:33">
-      <c r="A87" s="145"/>
+      <c r="A87" s="143"/>
       <c r="B87" s="46"/>
     </row>
     <row r="88" spans="1:33">
-      <c r="A88" s="145"/>
+      <c r="A88" s="143"/>
       <c r="B88" s="45"/>
     </row>
     <row r="89" spans="1:33">
-      <c r="A89" s="145"/>
+      <c r="A89" s="143"/>
       <c r="B89" s="46"/>
     </row>
     <row r="90" spans="1:33">
-      <c r="A90" s="145"/>
+      <c r="A90" s="143"/>
       <c r="B90" s="46"/>
     </row>
     <row r="91" spans="1:33">
-      <c r="A91" s="145"/>
+      <c r="A91" s="143"/>
       <c r="B91" s="45"/>
     </row>
     <row r="92" spans="1:33">
-      <c r="A92" s="145"/>
+      <c r="A92" s="143"/>
       <c r="B92" s="46"/>
     </row>
     <row r="93" spans="1:33">
-      <c r="A93" s="145"/>
+      <c r="A93" s="143"/>
       <c r="B93" s="46"/>
     </row>
     <row r="94" spans="1:33">
@@ -12627,20 +12633,20 @@
       <c r="AG94" s="29"/>
     </row>
     <row r="96" spans="1:33">
-      <c r="A96" s="143"/>
+      <c r="A96" s="144"/>
       <c r="B96" s="45"/>
       <c r="C96" s="40"/>
       <c r="AA96" s="32"/>
       <c r="AC96" s="32"/>
     </row>
     <row r="97" spans="1:35">
-      <c r="A97" s="143"/>
+      <c r="A97" s="144"/>
       <c r="B97" s="46"/>
       <c r="C97" s="41"/>
       <c r="AC97" s="32"/>
     </row>
     <row r="98" spans="1:35">
-      <c r="A98" s="143"/>
+      <c r="A98" s="144"/>
       <c r="B98" s="46"/>
       <c r="C98" s="42"/>
       <c r="AA98" s="32"/>
@@ -12652,15 +12658,15 @@
       <c r="W99" s="139"/>
     </row>
     <row r="101" spans="1:35">
-      <c r="A101" s="144"/>
+      <c r="A101" s="145"/>
     </row>
     <row r="102" spans="1:35">
-      <c r="A102" s="144"/>
+      <c r="A102" s="145"/>
     </row>
     <row r="103" spans="1:35"/>
     <row r="104" spans="1:35"/>
     <row r="105" spans="1:35">
-      <c r="A105" s="143" t="s">
+      <c r="A105" s="144" t="s">
         <v>392</v>
       </c>
       <c r="B105" s="45" t="s">
@@ -12675,7 +12681,7 @@
       </c>
     </row>
     <row r="106" spans="1:35">
-      <c r="A106" s="143"/>
+      <c r="A106" s="144"/>
       <c r="B106" s="46" t="s">
         <v>22</v>
       </c>
@@ -12691,7 +12697,7 @@
       </c>
     </row>
     <row r="107" spans="1:35">
-      <c r="A107" s="143"/>
+      <c r="A107" s="144"/>
       <c r="B107" s="46" t="s">
         <v>23</v>
       </c>
@@ -12707,7 +12713,7 @@
       </c>
     </row>
     <row r="108" spans="1:35">
-      <c r="A108" s="143" t="s">
+      <c r="A108" s="144" t="s">
         <v>393</v>
       </c>
       <c r="B108" s="45" t="s">
@@ -12722,7 +12728,7 @@
       </c>
     </row>
     <row r="109" spans="1:35">
-      <c r="A109" s="143"/>
+      <c r="A109" s="144"/>
       <c r="B109" s="46" t="s">
         <v>22</v>
       </c>
@@ -12738,7 +12744,7 @@
       </c>
     </row>
     <row r="110" spans="1:35">
-      <c r="A110" s="143"/>
+      <c r="A110" s="144"/>
       <c r="B110" s="46" t="s">
         <v>23</v>
       </c>
@@ -12866,16 +12872,6 @@
     <row r="150" customFormat="1"/>
   </sheetData>
   <mergeCells count="26">
-    <mergeCell ref="A30:A32"/>
-    <mergeCell ref="A105:A107"/>
-    <mergeCell ref="A33:A35"/>
-    <mergeCell ref="A36:A38"/>
-    <mergeCell ref="A96:A98"/>
-    <mergeCell ref="A101:A102"/>
-    <mergeCell ref="A88:A90"/>
-    <mergeCell ref="A91:A93"/>
-    <mergeCell ref="A64:A66"/>
-    <mergeCell ref="A82:A84"/>
     <mergeCell ref="A108:A110"/>
     <mergeCell ref="A14:A15"/>
     <mergeCell ref="A85:A87"/>
@@ -12892,6 +12888,16 @@
     <mergeCell ref="A19:A21"/>
     <mergeCell ref="A22:A24"/>
     <mergeCell ref="A25:A27"/>
+    <mergeCell ref="A30:A32"/>
+    <mergeCell ref="A105:A107"/>
+    <mergeCell ref="A33:A35"/>
+    <mergeCell ref="A36:A38"/>
+    <mergeCell ref="A96:A98"/>
+    <mergeCell ref="A101:A102"/>
+    <mergeCell ref="A88:A90"/>
+    <mergeCell ref="A91:A93"/>
+    <mergeCell ref="A64:A66"/>
+    <mergeCell ref="A82:A84"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <legacyDrawing r:id="rId1"/>
@@ -13227,328 +13233,328 @@
       <c r="DF4" s="6"/>
     </row>
     <row r="5" spans="1:110" s="8" customFormat="1" ht="30" customHeight="1">
-      <c r="D5" s="146" t="s">
+      <c r="D5" s="155" t="s">
         <v>3</v>
       </c>
-      <c r="E5" s="147"/>
-      <c r="F5" s="147"/>
-      <c r="G5" s="147"/>
-      <c r="H5" s="147"/>
-      <c r="I5" s="147"/>
-      <c r="J5" s="147"/>
-      <c r="K5" s="147"/>
-      <c r="L5" s="147"/>
-      <c r="M5" s="147"/>
-      <c r="N5" s="147"/>
-      <c r="O5" s="147"/>
-      <c r="P5" s="147"/>
-      <c r="Q5" s="147"/>
-      <c r="R5" s="148"/>
-      <c r="S5" s="157" t="s">
+      <c r="E5" s="156"/>
+      <c r="F5" s="156"/>
+      <c r="G5" s="156"/>
+      <c r="H5" s="156"/>
+      <c r="I5" s="156"/>
+      <c r="J5" s="156"/>
+      <c r="K5" s="156"/>
+      <c r="L5" s="156"/>
+      <c r="M5" s="156"/>
+      <c r="N5" s="156"/>
+      <c r="O5" s="156"/>
+      <c r="P5" s="156"/>
+      <c r="Q5" s="156"/>
+      <c r="R5" s="157"/>
+      <c r="S5" s="159" t="s">
         <v>4</v>
       </c>
-      <c r="T5" s="158"/>
-      <c r="U5" s="158"/>
-      <c r="V5" s="158"/>
-      <c r="W5" s="158"/>
-      <c r="X5" s="158"/>
-      <c r="Y5" s="158"/>
-      <c r="Z5" s="158"/>
-      <c r="AA5" s="158"/>
-      <c r="AB5" s="158"/>
-      <c r="AC5" s="158"/>
-      <c r="AD5" s="158"/>
-      <c r="AE5" s="158"/>
-      <c r="AF5" s="158"/>
-      <c r="AG5" s="159"/>
-      <c r="AH5" s="146" t="s">
+      <c r="T5" s="160"/>
+      <c r="U5" s="160"/>
+      <c r="V5" s="160"/>
+      <c r="W5" s="160"/>
+      <c r="X5" s="160"/>
+      <c r="Y5" s="160"/>
+      <c r="Z5" s="160"/>
+      <c r="AA5" s="160"/>
+      <c r="AB5" s="160"/>
+      <c r="AC5" s="160"/>
+      <c r="AD5" s="160"/>
+      <c r="AE5" s="160"/>
+      <c r="AF5" s="160"/>
+      <c r="AG5" s="161"/>
+      <c r="AH5" s="155" t="s">
         <v>5</v>
       </c>
-      <c r="AI5" s="147"/>
-      <c r="AJ5" s="147"/>
-      <c r="AK5" s="147"/>
-      <c r="AL5" s="147"/>
-      <c r="AM5" s="147"/>
-      <c r="AN5" s="147"/>
-      <c r="AO5" s="147"/>
-      <c r="AP5" s="147"/>
-      <c r="AQ5" s="147"/>
-      <c r="AR5" s="147"/>
-      <c r="AS5" s="147"/>
-      <c r="AT5" s="147"/>
-      <c r="AU5" s="147"/>
-      <c r="AV5" s="148"/>
-      <c r="AW5" s="157" t="s">
+      <c r="AI5" s="156"/>
+      <c r="AJ5" s="156"/>
+      <c r="AK5" s="156"/>
+      <c r="AL5" s="156"/>
+      <c r="AM5" s="156"/>
+      <c r="AN5" s="156"/>
+      <c r="AO5" s="156"/>
+      <c r="AP5" s="156"/>
+      <c r="AQ5" s="156"/>
+      <c r="AR5" s="156"/>
+      <c r="AS5" s="156"/>
+      <c r="AT5" s="156"/>
+      <c r="AU5" s="156"/>
+      <c r="AV5" s="157"/>
+      <c r="AW5" s="159" t="s">
         <v>6</v>
       </c>
-      <c r="AX5" s="158"/>
-      <c r="AY5" s="158"/>
-      <c r="AZ5" s="158"/>
-      <c r="BA5" s="158"/>
-      <c r="BB5" s="158"/>
-      <c r="BC5" s="158"/>
-      <c r="BD5" s="158"/>
-      <c r="BE5" s="158"/>
-      <c r="BF5" s="158"/>
-      <c r="BG5" s="158"/>
-      <c r="BH5" s="158"/>
-      <c r="BI5" s="158"/>
-      <c r="BJ5" s="158"/>
-      <c r="BK5" s="159"/>
-      <c r="BL5" s="146" t="s">
+      <c r="AX5" s="160"/>
+      <c r="AY5" s="160"/>
+      <c r="AZ5" s="160"/>
+      <c r="BA5" s="160"/>
+      <c r="BB5" s="160"/>
+      <c r="BC5" s="160"/>
+      <c r="BD5" s="160"/>
+      <c r="BE5" s="160"/>
+      <c r="BF5" s="160"/>
+      <c r="BG5" s="160"/>
+      <c r="BH5" s="160"/>
+      <c r="BI5" s="160"/>
+      <c r="BJ5" s="160"/>
+      <c r="BK5" s="161"/>
+      <c r="BL5" s="155" t="s">
         <v>7</v>
       </c>
-      <c r="BM5" s="147"/>
-      <c r="BN5" s="147"/>
-      <c r="BO5" s="147"/>
-      <c r="BP5" s="147"/>
-      <c r="BQ5" s="147"/>
-      <c r="BR5" s="147"/>
-      <c r="BS5" s="147"/>
-      <c r="BT5" s="147"/>
-      <c r="BU5" s="147"/>
-      <c r="BV5" s="147"/>
-      <c r="BW5" s="147"/>
-      <c r="BX5" s="147"/>
-      <c r="BY5" s="147"/>
-      <c r="BZ5" s="148"/>
-      <c r="CA5" s="157" t="s">
+      <c r="BM5" s="156"/>
+      <c r="BN5" s="156"/>
+      <c r="BO5" s="156"/>
+      <c r="BP5" s="156"/>
+      <c r="BQ5" s="156"/>
+      <c r="BR5" s="156"/>
+      <c r="BS5" s="156"/>
+      <c r="BT5" s="156"/>
+      <c r="BU5" s="156"/>
+      <c r="BV5" s="156"/>
+      <c r="BW5" s="156"/>
+      <c r="BX5" s="156"/>
+      <c r="BY5" s="156"/>
+      <c r="BZ5" s="157"/>
+      <c r="CA5" s="159" t="s">
         <v>8</v>
       </c>
-      <c r="CB5" s="158"/>
-      <c r="CC5" s="158"/>
-      <c r="CD5" s="158"/>
-      <c r="CE5" s="159"/>
-      <c r="CF5" s="146" t="s">
+      <c r="CB5" s="160"/>
+      <c r="CC5" s="160"/>
+      <c r="CD5" s="160"/>
+      <c r="CE5" s="161"/>
+      <c r="CF5" s="155" t="s">
         <v>9</v>
       </c>
-      <c r="CG5" s="147"/>
-      <c r="CH5" s="147"/>
-      <c r="CI5" s="147"/>
-      <c r="CJ5" s="147"/>
-      <c r="CK5" s="147"/>
-      <c r="CL5" s="147"/>
-      <c r="CM5" s="147"/>
-      <c r="CN5" s="147"/>
-      <c r="CO5" s="147"/>
-      <c r="CP5" s="147"/>
-      <c r="CQ5" s="147"/>
-      <c r="CR5" s="147"/>
-      <c r="CS5" s="147"/>
-      <c r="CT5" s="148"/>
-      <c r="CU5" s="149" t="s">
+      <c r="CG5" s="156"/>
+      <c r="CH5" s="156"/>
+      <c r="CI5" s="156"/>
+      <c r="CJ5" s="156"/>
+      <c r="CK5" s="156"/>
+      <c r="CL5" s="156"/>
+      <c r="CM5" s="156"/>
+      <c r="CN5" s="156"/>
+      <c r="CO5" s="156"/>
+      <c r="CP5" s="156"/>
+      <c r="CQ5" s="156"/>
+      <c r="CR5" s="156"/>
+      <c r="CS5" s="156"/>
+      <c r="CT5" s="157"/>
+      <c r="CU5" s="146" t="s">
         <v>10</v>
       </c>
-      <c r="CV5" s="149"/>
-      <c r="CW5" s="149"/>
-      <c r="CX5" s="149"/>
-      <c r="CY5" s="149"/>
-      <c r="CZ5" s="150" t="s">
+      <c r="CV5" s="146"/>
+      <c r="CW5" s="146"/>
+      <c r="CX5" s="146"/>
+      <c r="CY5" s="146"/>
+      <c r="CZ5" s="158" t="s">
         <v>11</v>
       </c>
-      <c r="DA5" s="150"/>
-      <c r="DB5" s="150"/>
+      <c r="DA5" s="158"/>
+      <c r="DB5" s="158"/>
       <c r="DC5" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="DD5" s="150" t="s">
+      <c r="DD5" s="158" t="s">
         <v>13</v>
       </c>
-      <c r="DE5" s="150"/>
-      <c r="DF5" s="150"/>
+      <c r="DE5" s="158"/>
+      <c r="DF5" s="158"/>
     </row>
     <row r="6" spans="1:110" s="8" customFormat="1" ht="12.75" customHeight="1">
-      <c r="D6" s="151" t="s">
+      <c r="D6" s="147" t="s">
         <v>14</v>
       </c>
-      <c r="E6" s="152"/>
-      <c r="F6" s="153"/>
-      <c r="G6" s="151" t="s">
+      <c r="E6" s="148"/>
+      <c r="F6" s="149"/>
+      <c r="G6" s="147" t="s">
         <v>15</v>
       </c>
-      <c r="H6" s="152"/>
-      <c r="I6" s="153"/>
-      <c r="J6" s="151" t="s">
+      <c r="H6" s="148"/>
+      <c r="I6" s="149"/>
+      <c r="J6" s="147" t="s">
         <v>16</v>
       </c>
-      <c r="K6" s="152"/>
-      <c r="L6" s="153"/>
-      <c r="M6" s="151" t="s">
+      <c r="K6" s="148"/>
+      <c r="L6" s="149"/>
+      <c r="M6" s="147" t="s">
         <v>17</v>
       </c>
-      <c r="N6" s="152"/>
-      <c r="O6" s="153"/>
-      <c r="P6" s="151" t="s">
+      <c r="N6" s="148"/>
+      <c r="O6" s="149"/>
+      <c r="P6" s="147" t="s">
         <v>18</v>
       </c>
-      <c r="Q6" s="152"/>
-      <c r="R6" s="153"/>
-      <c r="S6" s="154" t="s">
+      <c r="Q6" s="148"/>
+      <c r="R6" s="149"/>
+      <c r="S6" s="152" t="s">
         <v>14</v>
       </c>
-      <c r="T6" s="155"/>
-      <c r="U6" s="156"/>
-      <c r="V6" s="154" t="s">
+      <c r="T6" s="153"/>
+      <c r="U6" s="154"/>
+      <c r="V6" s="152" t="s">
         <v>15</v>
       </c>
-      <c r="W6" s="155"/>
-      <c r="X6" s="156"/>
-      <c r="Y6" s="154" t="s">
+      <c r="W6" s="153"/>
+      <c r="X6" s="154"/>
+      <c r="Y6" s="152" t="s">
         <v>16</v>
       </c>
-      <c r="Z6" s="155"/>
-      <c r="AA6" s="156"/>
-      <c r="AB6" s="154" t="s">
+      <c r="Z6" s="153"/>
+      <c r="AA6" s="154"/>
+      <c r="AB6" s="152" t="s">
         <v>17</v>
       </c>
-      <c r="AC6" s="155"/>
-      <c r="AD6" s="156"/>
-      <c r="AE6" s="154" t="s">
+      <c r="AC6" s="153"/>
+      <c r="AD6" s="154"/>
+      <c r="AE6" s="152" t="s">
         <v>18</v>
       </c>
-      <c r="AF6" s="155"/>
-      <c r="AG6" s="156"/>
-      <c r="AH6" s="151" t="s">
+      <c r="AF6" s="153"/>
+      <c r="AG6" s="154"/>
+      <c r="AH6" s="147" t="s">
         <v>14</v>
       </c>
-      <c r="AI6" s="152"/>
-      <c r="AJ6" s="153"/>
-      <c r="AK6" s="151" t="s">
+      <c r="AI6" s="148"/>
+      <c r="AJ6" s="149"/>
+      <c r="AK6" s="147" t="s">
         <v>15</v>
       </c>
-      <c r="AL6" s="152"/>
-      <c r="AM6" s="153"/>
-      <c r="AN6" s="151" t="s">
+      <c r="AL6" s="148"/>
+      <c r="AM6" s="149"/>
+      <c r="AN6" s="147" t="s">
         <v>16</v>
       </c>
-      <c r="AO6" s="152"/>
-      <c r="AP6" s="153"/>
-      <c r="AQ6" s="151" t="s">
+      <c r="AO6" s="148"/>
+      <c r="AP6" s="149"/>
+      <c r="AQ6" s="147" t="s">
         <v>17</v>
       </c>
-      <c r="AR6" s="152"/>
-      <c r="AS6" s="153"/>
-      <c r="AT6" s="151" t="s">
+      <c r="AR6" s="148"/>
+      <c r="AS6" s="149"/>
+      <c r="AT6" s="147" t="s">
         <v>18</v>
       </c>
-      <c r="AU6" s="152"/>
-      <c r="AV6" s="153"/>
-      <c r="AW6" s="154" t="s">
+      <c r="AU6" s="148"/>
+      <c r="AV6" s="149"/>
+      <c r="AW6" s="152" t="s">
         <v>14</v>
       </c>
-      <c r="AX6" s="155"/>
-      <c r="AY6" s="156"/>
-      <c r="AZ6" s="154" t="s">
+      <c r="AX6" s="153"/>
+      <c r="AY6" s="154"/>
+      <c r="AZ6" s="152" t="s">
         <v>15</v>
       </c>
-      <c r="BA6" s="155"/>
-      <c r="BB6" s="156"/>
-      <c r="BC6" s="154" t="s">
+      <c r="BA6" s="153"/>
+      <c r="BB6" s="154"/>
+      <c r="BC6" s="152" t="s">
         <v>16</v>
       </c>
-      <c r="BD6" s="155"/>
-      <c r="BE6" s="156"/>
-      <c r="BF6" s="154" t="s">
+      <c r="BD6" s="153"/>
+      <c r="BE6" s="154"/>
+      <c r="BF6" s="152" t="s">
         <v>17</v>
       </c>
-      <c r="BG6" s="155"/>
-      <c r="BH6" s="156"/>
-      <c r="BI6" s="154" t="s">
+      <c r="BG6" s="153"/>
+      <c r="BH6" s="154"/>
+      <c r="BI6" s="152" t="s">
         <v>18</v>
       </c>
-      <c r="BJ6" s="155"/>
-      <c r="BK6" s="156"/>
-      <c r="BL6" s="151" t="s">
+      <c r="BJ6" s="153"/>
+      <c r="BK6" s="154"/>
+      <c r="BL6" s="147" t="s">
         <v>14</v>
       </c>
-      <c r="BM6" s="152"/>
-      <c r="BN6" s="153"/>
-      <c r="BO6" s="151" t="s">
+      <c r="BM6" s="148"/>
+      <c r="BN6" s="149"/>
+      <c r="BO6" s="147" t="s">
         <v>15</v>
       </c>
-      <c r="BP6" s="152"/>
-      <c r="BQ6" s="153"/>
-      <c r="BR6" s="151" t="s">
+      <c r="BP6" s="148"/>
+      <c r="BQ6" s="149"/>
+      <c r="BR6" s="147" t="s">
         <v>16</v>
       </c>
-      <c r="BS6" s="152"/>
-      <c r="BT6" s="153"/>
-      <c r="BU6" s="151" t="s">
+      <c r="BS6" s="148"/>
+      <c r="BT6" s="149"/>
+      <c r="BU6" s="147" t="s">
         <v>17</v>
       </c>
-      <c r="BV6" s="152"/>
-      <c r="BW6" s="153"/>
-      <c r="BX6" s="151" t="s">
+      <c r="BV6" s="148"/>
+      <c r="BW6" s="149"/>
+      <c r="BX6" s="147" t="s">
         <v>18</v>
       </c>
-      <c r="BY6" s="152"/>
-      <c r="BZ6" s="153"/>
-      <c r="CA6" s="160" t="s">
+      <c r="BY6" s="148"/>
+      <c r="BZ6" s="149"/>
+      <c r="CA6" s="150" t="s">
         <v>19</v>
       </c>
-      <c r="CB6" s="160" t="s">
+      <c r="CB6" s="150" t="s">
         <v>15</v>
       </c>
-      <c r="CC6" s="160" t="s">
+      <c r="CC6" s="150" t="s">
         <v>16</v>
       </c>
-      <c r="CD6" s="160" t="s">
+      <c r="CD6" s="150" t="s">
         <v>17</v>
       </c>
-      <c r="CE6" s="160" t="s">
+      <c r="CE6" s="150" t="s">
         <v>18</v>
       </c>
-      <c r="CF6" s="151" t="s">
+      <c r="CF6" s="147" t="s">
         <v>14</v>
       </c>
-      <c r="CG6" s="152"/>
-      <c r="CH6" s="153"/>
-      <c r="CI6" s="151" t="s">
+      <c r="CG6" s="148"/>
+      <c r="CH6" s="149"/>
+      <c r="CI6" s="147" t="s">
         <v>15</v>
       </c>
-      <c r="CJ6" s="152"/>
-      <c r="CK6" s="153"/>
-      <c r="CL6" s="151" t="s">
+      <c r="CJ6" s="148"/>
+      <c r="CK6" s="149"/>
+      <c r="CL6" s="147" t="s">
         <v>16</v>
       </c>
-      <c r="CM6" s="152"/>
-      <c r="CN6" s="153"/>
-      <c r="CO6" s="151" t="s">
+      <c r="CM6" s="148"/>
+      <c r="CN6" s="149"/>
+      <c r="CO6" s="147" t="s">
         <v>17</v>
       </c>
-      <c r="CP6" s="152"/>
-      <c r="CQ6" s="153"/>
-      <c r="CR6" s="151" t="s">
+      <c r="CP6" s="148"/>
+      <c r="CQ6" s="149"/>
+      <c r="CR6" s="147" t="s">
         <v>18</v>
       </c>
-      <c r="CS6" s="152"/>
-      <c r="CT6" s="153"/>
-      <c r="CU6" s="149" t="s">
+      <c r="CS6" s="148"/>
+      <c r="CT6" s="149"/>
+      <c r="CU6" s="146" t="s">
         <v>19</v>
       </c>
-      <c r="CV6" s="149" t="s">
+      <c r="CV6" s="146" t="s">
         <v>15</v>
       </c>
-      <c r="CW6" s="149" t="s">
+      <c r="CW6" s="146" t="s">
         <v>16</v>
       </c>
-      <c r="CX6" s="149" t="s">
+      <c r="CX6" s="146" t="s">
         <v>17</v>
       </c>
-      <c r="CY6" s="149" t="s">
+      <c r="CY6" s="146" t="s">
         <v>18</v>
       </c>
-      <c r="CZ6" s="150"/>
-      <c r="DA6" s="150"/>
-      <c r="DB6" s="150"/>
+      <c r="CZ6" s="158"/>
+      <c r="DA6" s="158"/>
+      <c r="DB6" s="158"/>
       <c r="DC6" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="DD6" s="150" t="s">
+      <c r="DD6" s="158" t="s">
         <v>20</v>
       </c>
-      <c r="DE6" s="150"/>
-      <c r="DF6" s="150"/>
+      <c r="DE6" s="158"/>
+      <c r="DF6" s="158"/>
     </row>
     <row r="7" spans="1:110" s="8" customFormat="1" ht="15">
       <c r="D7" s="11" t="s">
@@ -13776,15 +13782,15 @@
       <c r="BZ7" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="CA7" s="161"/>
-      <c r="CB7" s="161"/>
-      <c r="CC7" s="161" t="s">
+      <c r="CA7" s="151"/>
+      <c r="CB7" s="151"/>
+      <c r="CC7" s="151" t="s">
         <v>22</v>
       </c>
-      <c r="CD7" s="161" t="s">
+      <c r="CD7" s="151" t="s">
         <v>23</v>
       </c>
-      <c r="CE7" s="161" t="s">
+      <c r="CE7" s="151" t="s">
         <v>21</v>
       </c>
       <c r="CF7" s="11" t="s">
@@ -13832,15 +13838,15 @@
       <c r="CT7" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="CU7" s="149"/>
-      <c r="CV7" s="149"/>
-      <c r="CW7" s="149" t="s">
+      <c r="CU7" s="146"/>
+      <c r="CV7" s="146"/>
+      <c r="CW7" s="146" t="s">
         <v>22</v>
       </c>
-      <c r="CX7" s="149" t="s">
+      <c r="CX7" s="146" t="s">
         <v>23</v>
       </c>
-      <c r="CY7" s="149" t="s">
+      <c r="CY7" s="146" t="s">
         <v>21</v>
       </c>
       <c r="CZ7" s="17" t="s">
@@ -16599,40 +16605,6 @@
     </row>
   </sheetData>
   <mergeCells count="50">
-    <mergeCell ref="CV6:CV7"/>
-    <mergeCell ref="CW6:CW7"/>
-    <mergeCell ref="CX6:CX7"/>
-    <mergeCell ref="CY6:CY7"/>
-    <mergeCell ref="CF6:CH6"/>
-    <mergeCell ref="CI6:CK6"/>
-    <mergeCell ref="CL6:CN6"/>
-    <mergeCell ref="CO6:CQ6"/>
-    <mergeCell ref="CR6:CT6"/>
-    <mergeCell ref="CU6:CU7"/>
-    <mergeCell ref="CE6:CE7"/>
-    <mergeCell ref="BF6:BH6"/>
-    <mergeCell ref="BI6:BK6"/>
-    <mergeCell ref="BL6:BN6"/>
-    <mergeCell ref="BO6:BQ6"/>
-    <mergeCell ref="BR6:BT6"/>
-    <mergeCell ref="BU6:BW6"/>
-    <mergeCell ref="BX6:BZ6"/>
-    <mergeCell ref="CA6:CA7"/>
-    <mergeCell ref="CB6:CB7"/>
-    <mergeCell ref="CC6:CC7"/>
-    <mergeCell ref="CD6:CD7"/>
-    <mergeCell ref="BC6:BE6"/>
-    <mergeCell ref="V6:X6"/>
-    <mergeCell ref="Y6:AA6"/>
-    <mergeCell ref="AB6:AD6"/>
-    <mergeCell ref="AE6:AG6"/>
-    <mergeCell ref="AH6:AJ6"/>
-    <mergeCell ref="AK6:AM6"/>
-    <mergeCell ref="AN6:AP6"/>
-    <mergeCell ref="AQ6:AS6"/>
-    <mergeCell ref="AT6:AV6"/>
-    <mergeCell ref="AW6:AY6"/>
-    <mergeCell ref="AZ6:BB6"/>
     <mergeCell ref="CF5:CT5"/>
     <mergeCell ref="CU5:CY5"/>
     <mergeCell ref="CZ5:DB6"/>
@@ -16649,6 +16621,40 @@
     <mergeCell ref="AW5:BK5"/>
     <mergeCell ref="BL5:BZ5"/>
     <mergeCell ref="CA5:CE5"/>
+    <mergeCell ref="BC6:BE6"/>
+    <mergeCell ref="V6:X6"/>
+    <mergeCell ref="Y6:AA6"/>
+    <mergeCell ref="AB6:AD6"/>
+    <mergeCell ref="AE6:AG6"/>
+    <mergeCell ref="AH6:AJ6"/>
+    <mergeCell ref="AK6:AM6"/>
+    <mergeCell ref="AN6:AP6"/>
+    <mergeCell ref="AQ6:AS6"/>
+    <mergeCell ref="AT6:AV6"/>
+    <mergeCell ref="AW6:AY6"/>
+    <mergeCell ref="AZ6:BB6"/>
+    <mergeCell ref="CE6:CE7"/>
+    <mergeCell ref="BF6:BH6"/>
+    <mergeCell ref="BI6:BK6"/>
+    <mergeCell ref="BL6:BN6"/>
+    <mergeCell ref="BO6:BQ6"/>
+    <mergeCell ref="BR6:BT6"/>
+    <mergeCell ref="BU6:BW6"/>
+    <mergeCell ref="BX6:BZ6"/>
+    <mergeCell ref="CA6:CA7"/>
+    <mergeCell ref="CB6:CB7"/>
+    <mergeCell ref="CC6:CC7"/>
+    <mergeCell ref="CD6:CD7"/>
+    <mergeCell ref="CV6:CV7"/>
+    <mergeCell ref="CW6:CW7"/>
+    <mergeCell ref="CX6:CX7"/>
+    <mergeCell ref="CY6:CY7"/>
+    <mergeCell ref="CF6:CH6"/>
+    <mergeCell ref="CI6:CK6"/>
+    <mergeCell ref="CL6:CN6"/>
+    <mergeCell ref="CO6:CQ6"/>
+    <mergeCell ref="CR6:CT6"/>
+    <mergeCell ref="CU6:CU7"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -16963,8 +16969,8 @@
       </c>
     </row>
     <row r="4" spans="1:35">
-      <c r="A4" s="165"/>
-      <c r="B4" s="167"/>
+      <c r="A4" s="162"/>
+      <c r="B4" s="172"/>
       <c r="C4" s="40"/>
       <c r="D4" s="32"/>
       <c r="E4" s="32"/>
@@ -16999,8 +17005,8 @@
       <c r="AH4" s="32"/>
     </row>
     <row r="5" spans="1:35">
-      <c r="A5" s="176"/>
-      <c r="B5" s="162"/>
+      <c r="A5" s="163"/>
+      <c r="B5" s="166"/>
       <c r="C5" s="41"/>
       <c r="D5" s="30"/>
       <c r="E5" s="30"/>
@@ -17035,8 +17041,8 @@
       <c r="AH5" s="30"/>
     </row>
     <row r="6" spans="1:35">
-      <c r="A6" s="176"/>
-      <c r="B6" s="168"/>
+      <c r="A6" s="163"/>
+      <c r="B6" s="169"/>
       <c r="C6" s="42"/>
       <c r="D6" s="32"/>
       <c r="E6" s="32"/>
@@ -17071,8 +17077,8 @@
       <c r="AH6" s="30"/>
     </row>
     <row r="7" spans="1:35">
-      <c r="A7" s="176"/>
-      <c r="B7" s="167"/>
+      <c r="A7" s="163"/>
+      <c r="B7" s="172"/>
       <c r="C7" s="40"/>
       <c r="D7" s="30"/>
       <c r="E7" s="30"/>
@@ -17107,8 +17113,8 @@
       <c r="AH7" s="32"/>
     </row>
     <row r="8" spans="1:35">
-      <c r="A8" s="176"/>
-      <c r="B8" s="162"/>
+      <c r="A8" s="163"/>
+      <c r="B8" s="166"/>
       <c r="C8" s="41"/>
       <c r="D8" s="32"/>
       <c r="E8" s="32"/>
@@ -17143,8 +17149,8 @@
       <c r="AH8" s="30"/>
     </row>
     <row r="9" spans="1:35">
-      <c r="A9" s="176"/>
-      <c r="B9" s="168"/>
+      <c r="A9" s="163"/>
+      <c r="B9" s="169"/>
       <c r="C9" s="42"/>
       <c r="D9" s="30"/>
       <c r="E9" s="30"/>
@@ -17179,8 +17185,8 @@
       <c r="AH9" s="30"/>
     </row>
     <row r="10" spans="1:35">
-      <c r="A10" s="176"/>
-      <c r="B10" s="167"/>
+      <c r="A10" s="163"/>
+      <c r="B10" s="172"/>
       <c r="C10" s="40"/>
       <c r="D10" s="32"/>
       <c r="E10" s="32"/>
@@ -17215,8 +17221,8 @@
       <c r="AH10" s="32"/>
     </row>
     <row r="11" spans="1:35">
-      <c r="A11" s="176"/>
-      <c r="B11" s="162"/>
+      <c r="A11" s="163"/>
+      <c r="B11" s="166"/>
       <c r="C11" s="41"/>
       <c r="D11" s="30"/>
       <c r="E11" s="30"/>
@@ -17251,8 +17257,8 @@
       <c r="AH11" s="30"/>
     </row>
     <row r="12" spans="1:35">
-      <c r="A12" s="176"/>
-      <c r="B12" s="168"/>
+      <c r="A12" s="163"/>
+      <c r="B12" s="169"/>
       <c r="C12" s="42"/>
       <c r="D12" s="32"/>
       <c r="E12" s="32"/>
@@ -17287,8 +17293,8 @@
       <c r="AH12" s="30"/>
     </row>
     <row r="13" spans="1:35">
-      <c r="A13" s="176"/>
-      <c r="B13" s="167"/>
+      <c r="A13" s="163"/>
+      <c r="B13" s="172"/>
       <c r="C13" s="40"/>
       <c r="D13" s="30"/>
       <c r="E13" s="30"/>
@@ -17323,8 +17329,8 @@
       <c r="AH13" s="32"/>
     </row>
     <row r="14" spans="1:35">
-      <c r="A14" s="176"/>
-      <c r="B14" s="162"/>
+      <c r="A14" s="163"/>
+      <c r="B14" s="166"/>
       <c r="C14" s="41"/>
       <c r="D14" s="32"/>
       <c r="E14" s="32"/>
@@ -17359,8 +17365,8 @@
       <c r="AH14" s="30"/>
     </row>
     <row r="15" spans="1:35">
-      <c r="A15" s="176"/>
-      <c r="B15" s="168"/>
+      <c r="A15" s="163"/>
+      <c r="B15" s="169"/>
       <c r="C15" s="42"/>
       <c r="D15" s="30"/>
       <c r="E15" s="30"/>
@@ -17395,8 +17401,8 @@
       <c r="AH15" s="30"/>
     </row>
     <row r="16" spans="1:35">
-      <c r="A16" s="176"/>
-      <c r="B16" s="167"/>
+      <c r="A16" s="163"/>
+      <c r="B16" s="172"/>
       <c r="C16" s="40"/>
       <c r="D16" s="32"/>
       <c r="E16" s="32"/>
@@ -17431,8 +17437,8 @@
       <c r="AH16" s="32"/>
     </row>
     <row r="17" spans="1:34">
-      <c r="A17" s="176"/>
-      <c r="B17" s="162"/>
+      <c r="A17" s="163"/>
+      <c r="B17" s="166"/>
       <c r="C17" s="41"/>
       <c r="D17" s="30"/>
       <c r="E17" s="30"/>
@@ -17467,8 +17473,8 @@
       <c r="AH17" s="30"/>
     </row>
     <row r="18" spans="1:34">
-      <c r="A18" s="166"/>
-      <c r="B18" s="168"/>
+      <c r="A18" s="164"/>
+      <c r="B18" s="169"/>
       <c r="C18" s="42"/>
       <c r="D18" s="32"/>
       <c r="E18" s="32"/>
@@ -17503,8 +17509,8 @@
       <c r="AH18" s="30"/>
     </row>
     <row r="19" spans="1:34">
-      <c r="A19" s="163"/>
-      <c r="B19" s="162"/>
+      <c r="A19" s="165"/>
+      <c r="B19" s="166"/>
       <c r="C19" s="40"/>
       <c r="D19" s="32"/>
       <c r="E19" s="32"/>
@@ -17539,8 +17545,8 @@
       <c r="AH19" s="30"/>
     </row>
     <row r="20" spans="1:34">
-      <c r="A20" s="162"/>
-      <c r="B20" s="162"/>
+      <c r="A20" s="166"/>
+      <c r="B20" s="166"/>
       <c r="C20" s="41"/>
       <c r="D20" s="32"/>
       <c r="E20" s="32"/>
@@ -17575,8 +17581,8 @@
       <c r="AH20" s="30"/>
     </row>
     <row r="21" spans="1:34">
-      <c r="A21" s="164"/>
-      <c r="B21" s="162"/>
+      <c r="A21" s="167"/>
+      <c r="B21" s="166"/>
       <c r="C21" s="42"/>
       <c r="D21" s="32"/>
       <c r="E21" s="32"/>
@@ -17611,8 +17617,8 @@
       <c r="AH21" s="30"/>
     </row>
     <row r="22" spans="1:34">
-      <c r="A22" s="163"/>
-      <c r="B22" s="162"/>
+      <c r="A22" s="165"/>
+      <c r="B22" s="166"/>
       <c r="C22" s="40"/>
       <c r="D22" s="30"/>
       <c r="E22" s="30"/>
@@ -17647,8 +17653,8 @@
       <c r="AH22" s="32"/>
     </row>
     <row r="23" spans="1:34">
-      <c r="A23" s="162"/>
-      <c r="B23" s="162"/>
+      <c r="A23" s="166"/>
+      <c r="B23" s="166"/>
       <c r="C23" s="41"/>
       <c r="D23" s="32"/>
       <c r="E23" s="32"/>
@@ -17683,8 +17689,8 @@
       <c r="AH23" s="30"/>
     </row>
     <row r="24" spans="1:34">
-      <c r="A24" s="162"/>
-      <c r="B24" s="162"/>
+      <c r="A24" s="166"/>
+      <c r="B24" s="166"/>
       <c r="C24" s="42"/>
       <c r="D24" s="30"/>
       <c r="E24" s="30"/>
@@ -17719,8 +17725,8 @@
       <c r="AH24" s="30"/>
     </row>
     <row r="25" spans="1:34">
-      <c r="A25" s="162"/>
-      <c r="B25" s="162"/>
+      <c r="A25" s="166"/>
+      <c r="B25" s="166"/>
       <c r="C25" s="40"/>
       <c r="D25" s="32"/>
       <c r="E25" s="32"/>
@@ -17755,8 +17761,8 @@
       <c r="AH25" s="32"/>
     </row>
     <row r="26" spans="1:34">
-      <c r="A26" s="162"/>
-      <c r="B26" s="162"/>
+      <c r="A26" s="166"/>
+      <c r="B26" s="166"/>
       <c r="C26" s="41"/>
       <c r="D26" s="30"/>
       <c r="E26" s="30"/>
@@ -17791,8 +17797,8 @@
       <c r="AH26" s="30"/>
     </row>
     <row r="27" spans="1:34">
-      <c r="A27" s="162"/>
-      <c r="B27" s="162"/>
+      <c r="A27" s="166"/>
+      <c r="B27" s="166"/>
       <c r="C27" s="42"/>
       <c r="D27" s="32"/>
       <c r="E27" s="32"/>
@@ -17827,8 +17833,8 @@
       <c r="AH27" s="30"/>
     </row>
     <row r="28" spans="1:34">
-      <c r="A28" s="162"/>
-      <c r="B28" s="162"/>
+      <c r="A28" s="166"/>
+      <c r="B28" s="166"/>
       <c r="C28" s="40"/>
       <c r="D28" s="30"/>
       <c r="E28" s="30"/>
@@ -17863,8 +17869,8 @@
       <c r="AH28" s="32"/>
     </row>
     <row r="29" spans="1:34">
-      <c r="A29" s="162"/>
-      <c r="B29" s="162"/>
+      <c r="A29" s="166"/>
+      <c r="B29" s="166"/>
       <c r="C29" s="41"/>
       <c r="D29" s="32"/>
       <c r="E29" s="32"/>
@@ -17899,8 +17905,8 @@
       <c r="AH29" s="30"/>
     </row>
     <row r="30" spans="1:34">
-      <c r="A30" s="162"/>
-      <c r="B30" s="162"/>
+      <c r="A30" s="166"/>
+      <c r="B30" s="166"/>
       <c r="C30" s="42"/>
       <c r="D30" s="30"/>
       <c r="E30" s="30"/>
@@ -17935,8 +17941,8 @@
       <c r="AH30" s="30"/>
     </row>
     <row r="31" spans="1:34">
-      <c r="A31" s="162"/>
-      <c r="B31" s="162"/>
+      <c r="A31" s="166"/>
+      <c r="B31" s="166"/>
       <c r="C31" s="40"/>
       <c r="D31" s="32"/>
       <c r="E31" s="32"/>
@@ -17971,8 +17977,8 @@
       <c r="AH31" s="32"/>
     </row>
     <row r="32" spans="1:34">
-      <c r="A32" s="162"/>
-      <c r="B32" s="162"/>
+      <c r="A32" s="166"/>
+      <c r="B32" s="166"/>
       <c r="C32" s="41"/>
       <c r="D32" s="30"/>
       <c r="E32" s="30"/>
@@ -18007,8 +18013,8 @@
       <c r="AH32" s="30"/>
     </row>
     <row r="33" spans="1:34">
-      <c r="A33" s="162"/>
-      <c r="B33" s="162"/>
+      <c r="A33" s="166"/>
+      <c r="B33" s="166"/>
       <c r="C33" s="42"/>
       <c r="D33" s="32"/>
       <c r="E33" s="32"/>
@@ -18043,8 +18049,8 @@
       <c r="AH33" s="30"/>
     </row>
     <row r="34" spans="1:34">
-      <c r="A34" s="162"/>
-      <c r="B34" s="162"/>
+      <c r="A34" s="166"/>
+      <c r="B34" s="166"/>
       <c r="C34" s="40"/>
       <c r="D34" s="30"/>
       <c r="E34" s="30"/>
@@ -18079,8 +18085,8 @@
       <c r="AH34" s="32"/>
     </row>
     <row r="35" spans="1:34">
-      <c r="A35" s="162"/>
-      <c r="B35" s="162"/>
+      <c r="A35" s="166"/>
+      <c r="B35" s="166"/>
       <c r="C35" s="41"/>
       <c r="D35" s="32"/>
       <c r="E35" s="32"/>
@@ -18115,8 +18121,8 @@
       <c r="AH35" s="30"/>
     </row>
     <row r="36" spans="1:34">
-      <c r="A36" s="164"/>
-      <c r="B36" s="162"/>
+      <c r="A36" s="167"/>
+      <c r="B36" s="166"/>
       <c r="C36" s="42"/>
       <c r="D36" s="30"/>
       <c r="E36" s="30"/>
@@ -18151,8 +18157,8 @@
       <c r="AH36" s="30"/>
     </row>
     <row r="37" spans="1:34" ht="15.5" customHeight="1">
-      <c r="A37" s="163"/>
-      <c r="B37" s="162"/>
+      <c r="A37" s="165"/>
+      <c r="B37" s="166"/>
       <c r="C37" s="40"/>
       <c r="D37" s="32"/>
       <c r="E37" s="32"/>
@@ -18187,8 +18193,8 @@
       <c r="AH37" s="32"/>
     </row>
     <row r="38" spans="1:34">
-      <c r="A38" s="162"/>
-      <c r="B38" s="162"/>
+      <c r="A38" s="166"/>
+      <c r="B38" s="166"/>
       <c r="C38" s="41"/>
       <c r="D38" s="30"/>
       <c r="E38" s="30"/>
@@ -18223,8 +18229,8 @@
       <c r="AH38" s="30"/>
     </row>
     <row r="39" spans="1:34">
-      <c r="A39" s="162"/>
-      <c r="B39" s="162"/>
+      <c r="A39" s="166"/>
+      <c r="B39" s="166"/>
       <c r="C39" s="42"/>
       <c r="D39" s="32"/>
       <c r="E39" s="32"/>
@@ -18259,8 +18265,8 @@
       <c r="AH39" s="30"/>
     </row>
     <row r="40" spans="1:34">
-      <c r="A40" s="162"/>
-      <c r="B40" s="162"/>
+      <c r="A40" s="166"/>
+      <c r="B40" s="166"/>
       <c r="C40" s="40"/>
       <c r="D40" s="30"/>
       <c r="E40" s="30"/>
@@ -18295,8 +18301,8 @@
       <c r="AH40" s="32"/>
     </row>
     <row r="41" spans="1:34">
-      <c r="A41" s="162"/>
-      <c r="B41" s="162"/>
+      <c r="A41" s="166"/>
+      <c r="B41" s="166"/>
       <c r="C41" s="41"/>
       <c r="D41" s="32"/>
       <c r="E41" s="32"/>
@@ -18331,8 +18337,8 @@
       <c r="AH41" s="30"/>
     </row>
     <row r="42" spans="1:34">
-      <c r="A42" s="162"/>
-      <c r="B42" s="162"/>
+      <c r="A42" s="166"/>
+      <c r="B42" s="166"/>
       <c r="C42" s="42"/>
       <c r="D42" s="30"/>
       <c r="E42" s="30"/>
@@ -18367,8 +18373,8 @@
       <c r="AH42" s="30"/>
     </row>
     <row r="43" spans="1:34">
-      <c r="A43" s="162"/>
-      <c r="B43" s="162"/>
+      <c r="A43" s="166"/>
+      <c r="B43" s="166"/>
       <c r="C43" s="40"/>
       <c r="D43" s="32"/>
       <c r="E43" s="32"/>
@@ -18403,8 +18409,8 @@
       <c r="AH43" s="32"/>
     </row>
     <row r="44" spans="1:34">
-      <c r="A44" s="162"/>
-      <c r="B44" s="162"/>
+      <c r="A44" s="166"/>
+      <c r="B44" s="166"/>
       <c r="C44" s="41"/>
       <c r="D44" s="30"/>
       <c r="E44" s="30"/>
@@ -18439,8 +18445,8 @@
       <c r="AH44" s="30"/>
     </row>
     <row r="45" spans="1:34">
-      <c r="A45" s="162"/>
-      <c r="B45" s="162"/>
+      <c r="A45" s="166"/>
+      <c r="B45" s="166"/>
       <c r="C45" s="42"/>
       <c r="D45" s="32"/>
       <c r="E45" s="32"/>
@@ -18475,8 +18481,8 @@
       <c r="AH45" s="30"/>
     </row>
     <row r="46" spans="1:34">
-      <c r="A46" s="162"/>
-      <c r="B46" s="162"/>
+      <c r="A46" s="166"/>
+      <c r="B46" s="166"/>
       <c r="C46" s="40"/>
       <c r="D46" s="30"/>
       <c r="E46" s="30"/>
@@ -18511,8 +18517,8 @@
       <c r="AH46" s="32"/>
     </row>
     <row r="47" spans="1:34">
-      <c r="A47" s="162"/>
-      <c r="B47" s="162"/>
+      <c r="A47" s="166"/>
+      <c r="B47" s="166"/>
       <c r="C47" s="41"/>
       <c r="D47" s="32"/>
       <c r="E47" s="32"/>
@@ -18547,8 +18553,8 @@
       <c r="AH47" s="30"/>
     </row>
     <row r="48" spans="1:34">
-      <c r="A48" s="162"/>
-      <c r="B48" s="162"/>
+      <c r="A48" s="166"/>
+      <c r="B48" s="166"/>
       <c r="C48" s="42"/>
       <c r="D48" s="30"/>
       <c r="E48" s="30"/>
@@ -18583,8 +18589,8 @@
       <c r="AH48" s="30"/>
     </row>
     <row r="49" spans="1:34">
-      <c r="A49" s="162"/>
-      <c r="B49" s="162"/>
+      <c r="A49" s="166"/>
+      <c r="B49" s="166"/>
       <c r="C49" s="40"/>
       <c r="D49" s="32"/>
       <c r="E49" s="32"/>
@@ -18619,8 +18625,8 @@
       <c r="AH49" s="32"/>
     </row>
     <row r="50" spans="1:34">
-      <c r="A50" s="162"/>
-      <c r="B50" s="162"/>
+      <c r="A50" s="166"/>
+      <c r="B50" s="166"/>
       <c r="C50" s="41"/>
       <c r="D50" s="30"/>
       <c r="E50" s="30"/>
@@ -18655,8 +18661,8 @@
       <c r="AH50" s="30"/>
     </row>
     <row r="51" spans="1:34">
-      <c r="A51" s="164"/>
-      <c r="B51" s="162"/>
+      <c r="A51" s="167"/>
+      <c r="B51" s="166"/>
       <c r="C51" s="42"/>
       <c r="D51" s="32"/>
       <c r="E51" s="32"/>
@@ -18691,10 +18697,10 @@
       <c r="AH51" s="30"/>
     </row>
     <row r="52" spans="1:34" ht="15.5" customHeight="1">
-      <c r="A52" s="163" t="s">
+      <c r="A52" s="165" t="s">
         <v>6</v>
       </c>
-      <c r="B52" s="162" t="s">
+      <c r="B52" s="166" t="s">
         <v>14</v>
       </c>
       <c r="C52" s="40" t="s">
@@ -18785,8 +18791,8 @@
       </c>
     </row>
     <row r="53" spans="1:34">
-      <c r="A53" s="162"/>
-      <c r="B53" s="162"/>
+      <c r="A53" s="166"/>
+      <c r="B53" s="166"/>
       <c r="C53" s="41" t="s">
         <v>22</v>
       </c>
@@ -18875,8 +18881,8 @@
       </c>
     </row>
     <row r="54" spans="1:34">
-      <c r="A54" s="162"/>
-      <c r="B54" s="162"/>
+      <c r="A54" s="166"/>
+      <c r="B54" s="166"/>
       <c r="C54" s="42" t="s">
         <v>23</v>
       </c>
@@ -18965,8 +18971,8 @@
       </c>
     </row>
     <row r="55" spans="1:34">
-      <c r="A55" s="162"/>
-      <c r="B55" s="162" t="s">
+      <c r="A55" s="166"/>
+      <c r="B55" s="166" t="s">
         <v>15</v>
       </c>
       <c r="C55" s="40" t="s">
@@ -19057,8 +19063,8 @@
       </c>
     </row>
     <row r="56" spans="1:34">
-      <c r="A56" s="162"/>
-      <c r="B56" s="162"/>
+      <c r="A56" s="166"/>
+      <c r="B56" s="166"/>
       <c r="C56" s="41" t="s">
         <v>22</v>
       </c>
@@ -19147,8 +19153,8 @@
       </c>
     </row>
     <row r="57" spans="1:34">
-      <c r="A57" s="162"/>
-      <c r="B57" s="162"/>
+      <c r="A57" s="166"/>
+      <c r="B57" s="166"/>
       <c r="C57" s="42" t="s">
         <v>23</v>
       </c>
@@ -19236,8 +19242,8 @@
       </c>
     </row>
     <row r="58" spans="1:34">
-      <c r="A58" s="162"/>
-      <c r="B58" s="162" t="s">
+      <c r="A58" s="166"/>
+      <c r="B58" s="166" t="s">
         <v>16</v>
       </c>
       <c r="C58" s="40" t="s">
@@ -19328,8 +19334,8 @@
       </c>
     </row>
     <row r="59" spans="1:34">
-      <c r="A59" s="162"/>
-      <c r="B59" s="162"/>
+      <c r="A59" s="166"/>
+      <c r="B59" s="166"/>
       <c r="C59" s="41" t="s">
         <v>22</v>
       </c>
@@ -19418,8 +19424,8 @@
       </c>
     </row>
     <row r="60" spans="1:34">
-      <c r="A60" s="162"/>
-      <c r="B60" s="162"/>
+      <c r="A60" s="166"/>
+      <c r="B60" s="166"/>
       <c r="C60" s="42" t="s">
         <v>23</v>
       </c>
@@ -19508,8 +19514,8 @@
       </c>
     </row>
     <row r="61" spans="1:34">
-      <c r="A61" s="162"/>
-      <c r="B61" s="162" t="s">
+      <c r="A61" s="166"/>
+      <c r="B61" s="166" t="s">
         <v>17</v>
       </c>
       <c r="C61" s="40" t="s">
@@ -19600,8 +19606,8 @@
       </c>
     </row>
     <row r="62" spans="1:34">
-      <c r="A62" s="162"/>
-      <c r="B62" s="162"/>
+      <c r="A62" s="166"/>
+      <c r="B62" s="166"/>
       <c r="C62" s="41" t="s">
         <v>22</v>
       </c>
@@ -19690,8 +19696,8 @@
       </c>
     </row>
     <row r="63" spans="1:34">
-      <c r="A63" s="162"/>
-      <c r="B63" s="162"/>
+      <c r="A63" s="166"/>
+      <c r="B63" s="166"/>
       <c r="C63" s="42" t="s">
         <v>23</v>
       </c>
@@ -19780,8 +19786,8 @@
       </c>
     </row>
     <row r="64" spans="1:34">
-      <c r="A64" s="162"/>
-      <c r="B64" s="162" t="s">
+      <c r="A64" s="166"/>
+      <c r="B64" s="166" t="s">
         <v>18</v>
       </c>
       <c r="C64" s="40" t="s">
@@ -19872,8 +19878,8 @@
       </c>
     </row>
     <row r="65" spans="1:34">
-      <c r="A65" s="162"/>
-      <c r="B65" s="162"/>
+      <c r="A65" s="166"/>
+      <c r="B65" s="166"/>
       <c r="C65" s="41" t="s">
         <v>22</v>
       </c>
@@ -19962,8 +19968,8 @@
       </c>
     </row>
     <row r="66" spans="1:34">
-      <c r="A66" s="164"/>
-      <c r="B66" s="162"/>
+      <c r="A66" s="167"/>
+      <c r="B66" s="166"/>
       <c r="C66" s="42" t="s">
         <v>23</v>
       </c>
@@ -20052,8 +20058,8 @@
       </c>
     </row>
     <row r="67" spans="1:34" ht="15.5" customHeight="1">
-      <c r="A67" s="163"/>
-      <c r="B67" s="162"/>
+      <c r="A67" s="165"/>
+      <c r="B67" s="166"/>
       <c r="C67" s="40"/>
       <c r="D67" s="32"/>
       <c r="E67" s="32"/>
@@ -20088,8 +20094,8 @@
       <c r="AH67" s="32"/>
     </row>
     <row r="68" spans="1:34">
-      <c r="A68" s="162"/>
-      <c r="B68" s="162"/>
+      <c r="A68" s="166"/>
+      <c r="B68" s="166"/>
       <c r="C68" s="41"/>
       <c r="D68" s="30"/>
       <c r="E68" s="30"/>
@@ -20124,8 +20130,8 @@
       <c r="AH68" s="30"/>
     </row>
     <row r="69" spans="1:34">
-      <c r="A69" s="162"/>
-      <c r="B69" s="162"/>
+      <c r="A69" s="166"/>
+      <c r="B69" s="166"/>
       <c r="C69" s="42"/>
       <c r="D69" s="32"/>
       <c r="E69" s="32"/>
@@ -20160,8 +20166,8 @@
       <c r="AH69" s="30"/>
     </row>
     <row r="70" spans="1:34">
-      <c r="A70" s="162"/>
-      <c r="B70" s="162"/>
+      <c r="A70" s="166"/>
+      <c r="B70" s="166"/>
       <c r="C70" s="40"/>
       <c r="D70" s="30"/>
       <c r="E70" s="30"/>
@@ -20196,8 +20202,8 @@
       <c r="AH70" s="32"/>
     </row>
     <row r="71" spans="1:34">
-      <c r="A71" s="162"/>
-      <c r="B71" s="162"/>
+      <c r="A71" s="166"/>
+      <c r="B71" s="166"/>
       <c r="C71" s="41"/>
       <c r="D71" s="32"/>
       <c r="E71" s="32"/>
@@ -20232,8 +20238,8 @@
       <c r="AH71" s="30"/>
     </row>
     <row r="72" spans="1:34">
-      <c r="A72" s="162"/>
-      <c r="B72" s="162"/>
+      <c r="A72" s="166"/>
+      <c r="B72" s="166"/>
       <c r="C72" s="42"/>
       <c r="D72" s="30"/>
       <c r="E72" s="30"/>
@@ -20268,8 +20274,8 @@
       <c r="AH72" s="30"/>
     </row>
     <row r="73" spans="1:34">
-      <c r="A73" s="162"/>
-      <c r="B73" s="162"/>
+      <c r="A73" s="166"/>
+      <c r="B73" s="166"/>
       <c r="C73" s="40"/>
       <c r="D73" s="32"/>
       <c r="E73" s="32"/>
@@ -20304,8 +20310,8 @@
       <c r="AH73" s="32"/>
     </row>
     <row r="74" spans="1:34">
-      <c r="A74" s="162"/>
-      <c r="B74" s="162"/>
+      <c r="A74" s="166"/>
+      <c r="B74" s="166"/>
       <c r="C74" s="41"/>
       <c r="D74" s="30"/>
       <c r="E74" s="30"/>
@@ -20340,8 +20346,8 @@
       <c r="AH74" s="30"/>
     </row>
     <row r="75" spans="1:34">
-      <c r="A75" s="162"/>
-      <c r="B75" s="162"/>
+      <c r="A75" s="166"/>
+      <c r="B75" s="166"/>
       <c r="C75" s="42"/>
       <c r="D75" s="32"/>
       <c r="E75" s="32"/>
@@ -20376,8 +20382,8 @@
       <c r="AH75" s="30"/>
     </row>
     <row r="76" spans="1:34">
-      <c r="A76" s="162"/>
-      <c r="B76" s="162"/>
+      <c r="A76" s="166"/>
+      <c r="B76" s="166"/>
       <c r="C76" s="40"/>
       <c r="D76" s="30"/>
       <c r="E76" s="30"/>
@@ -20412,8 +20418,8 @@
       <c r="AH76" s="32"/>
     </row>
     <row r="77" spans="1:34">
-      <c r="A77" s="162"/>
-      <c r="B77" s="162"/>
+      <c r="A77" s="166"/>
+      <c r="B77" s="166"/>
       <c r="C77" s="41"/>
       <c r="D77" s="32"/>
       <c r="E77" s="32"/>
@@ -20448,8 +20454,8 @@
       <c r="AH77" s="30"/>
     </row>
     <row r="78" spans="1:34">
-      <c r="A78" s="162"/>
-      <c r="B78" s="162"/>
+      <c r="A78" s="166"/>
+      <c r="B78" s="166"/>
       <c r="C78" s="42"/>
       <c r="D78" s="30"/>
       <c r="E78" s="30"/>
@@ -20484,8 +20490,8 @@
       <c r="AH78" s="30"/>
     </row>
     <row r="79" spans="1:34">
-      <c r="A79" s="162"/>
-      <c r="B79" s="162"/>
+      <c r="A79" s="166"/>
+      <c r="B79" s="166"/>
       <c r="C79" s="40"/>
       <c r="D79" s="32"/>
       <c r="E79" s="32"/>
@@ -20520,8 +20526,8 @@
       <c r="AH79" s="32"/>
     </row>
     <row r="80" spans="1:34">
-      <c r="A80" s="162"/>
-      <c r="B80" s="162"/>
+      <c r="A80" s="166"/>
+      <c r="B80" s="166"/>
       <c r="C80" s="41"/>
       <c r="D80" s="30"/>
       <c r="E80" s="30"/>
@@ -20556,8 +20562,8 @@
       <c r="AH80" s="30"/>
     </row>
     <row r="81" spans="1:34">
-      <c r="A81" s="164"/>
-      <c r="B81" s="164"/>
+      <c r="A81" s="167"/>
+      <c r="B81" s="167"/>
       <c r="C81" s="42"/>
       <c r="D81" s="32"/>
       <c r="E81" s="32"/>
@@ -20592,9 +20598,9 @@
       <c r="AH81" s="30"/>
     </row>
     <row r="82" spans="1:34">
-      <c r="A82" s="170"/>
-      <c r="B82" s="165"/>
-      <c r="C82" s="166"/>
+      <c r="A82" s="168"/>
+      <c r="B82" s="162"/>
+      <c r="C82" s="164"/>
       <c r="D82" s="30"/>
       <c r="E82" s="30"/>
       <c r="F82" s="30"/>
@@ -20628,9 +20634,9 @@
       <c r="AH82" s="33"/>
     </row>
     <row r="83" spans="1:34">
-      <c r="A83" s="168"/>
-      <c r="B83" s="165"/>
-      <c r="C83" s="166"/>
+      <c r="A83" s="169"/>
+      <c r="B83" s="162"/>
+      <c r="C83" s="164"/>
       <c r="D83" s="32"/>
       <c r="E83" s="32"/>
       <c r="F83" s="32"/>
@@ -20664,9 +20670,9 @@
       <c r="AH83" s="33"/>
     </row>
     <row r="84" spans="1:34">
-      <c r="A84" s="168"/>
-      <c r="B84" s="165"/>
-      <c r="C84" s="166"/>
+      <c r="A84" s="169"/>
+      <c r="B84" s="162"/>
+      <c r="C84" s="164"/>
       <c r="D84" s="30"/>
       <c r="E84" s="30"/>
       <c r="F84" s="30"/>
@@ -20700,7 +20706,7 @@
       <c r="AH84" s="33"/>
     </row>
     <row r="85" spans="1:34">
-      <c r="A85" s="168"/>
+      <c r="A85" s="169"/>
       <c r="B85" s="96"/>
       <c r="C85" s="97"/>
       <c r="D85" s="32"/>
@@ -20736,7 +20742,7 @@
       <c r="AH85" s="33"/>
     </row>
     <row r="86" spans="1:34">
-      <c r="A86" s="172"/>
+      <c r="A86" s="170"/>
       <c r="B86" s="96"/>
       <c r="C86" s="97"/>
       <c r="D86" s="30"/>
@@ -20772,8 +20778,8 @@
       <c r="AH86" s="33"/>
     </row>
     <row r="87" spans="1:34">
-      <c r="A87" s="163"/>
-      <c r="B87" s="162"/>
+      <c r="A87" s="165"/>
+      <c r="B87" s="166"/>
       <c r="C87" s="40"/>
       <c r="D87" s="32"/>
       <c r="E87" s="32"/>
@@ -20808,8 +20814,8 @@
       <c r="AH87" s="33"/>
     </row>
     <row r="88" spans="1:34">
-      <c r="A88" s="162"/>
-      <c r="B88" s="162"/>
+      <c r="A88" s="166"/>
+      <c r="B88" s="166"/>
       <c r="C88" s="41"/>
       <c r="D88" s="30"/>
       <c r="E88" s="30"/>
@@ -20844,8 +20850,8 @@
       <c r="AH88" s="34"/>
     </row>
     <row r="89" spans="1:34">
-      <c r="A89" s="162"/>
-      <c r="B89" s="162"/>
+      <c r="A89" s="166"/>
+      <c r="B89" s="166"/>
       <c r="C89" s="42"/>
       <c r="D89" s="32"/>
       <c r="E89" s="32"/>
@@ -20880,8 +20886,8 @@
       <c r="AH89" s="34"/>
     </row>
     <row r="90" spans="1:34">
-      <c r="A90" s="162"/>
-      <c r="B90" s="162"/>
+      <c r="A90" s="166"/>
+      <c r="B90" s="166"/>
       <c r="C90" s="40"/>
       <c r="D90" s="30"/>
       <c r="E90" s="30"/>
@@ -20916,8 +20922,8 @@
       <c r="AH90" s="33"/>
     </row>
     <row r="91" spans="1:34">
-      <c r="A91" s="162"/>
-      <c r="B91" s="162"/>
+      <c r="A91" s="166"/>
+      <c r="B91" s="166"/>
       <c r="C91" s="41"/>
       <c r="D91" s="32"/>
       <c r="E91" s="32"/>
@@ -20952,8 +20958,8 @@
       <c r="AH91" s="34"/>
     </row>
     <row r="92" spans="1:34">
-      <c r="A92" s="162"/>
-      <c r="B92" s="162"/>
+      <c r="A92" s="166"/>
+      <c r="B92" s="166"/>
       <c r="C92" s="42"/>
       <c r="D92" s="30"/>
       <c r="E92" s="30"/>
@@ -20988,8 +20994,8 @@
       <c r="AH92" s="34"/>
     </row>
     <row r="93" spans="1:34">
-      <c r="A93" s="162"/>
-      <c r="B93" s="162"/>
+      <c r="A93" s="166"/>
+      <c r="B93" s="166"/>
       <c r="C93" s="40"/>
       <c r="D93" s="32"/>
       <c r="E93" s="32"/>
@@ -21024,8 +21030,8 @@
       <c r="AH93" s="33"/>
     </row>
     <row r="94" spans="1:34">
-      <c r="A94" s="162"/>
-      <c r="B94" s="162"/>
+      <c r="A94" s="166"/>
+      <c r="B94" s="166"/>
       <c r="C94" s="41"/>
       <c r="D94" s="30"/>
       <c r="E94" s="30"/>
@@ -21060,8 +21066,8 @@
       <c r="AH94" s="34"/>
     </row>
     <row r="95" spans="1:34">
-      <c r="A95" s="162"/>
-      <c r="B95" s="162"/>
+      <c r="A95" s="166"/>
+      <c r="B95" s="166"/>
       <c r="C95" s="42"/>
       <c r="D95" s="32"/>
       <c r="E95" s="32"/>
@@ -21096,8 +21102,8 @@
       <c r="AH95" s="34"/>
     </row>
     <row r="96" spans="1:34">
-      <c r="A96" s="162"/>
-      <c r="B96" s="162"/>
+      <c r="A96" s="166"/>
+      <c r="B96" s="166"/>
       <c r="C96" s="40"/>
       <c r="D96" s="30"/>
       <c r="E96" s="30"/>
@@ -21132,8 +21138,8 @@
       <c r="AH96" s="33"/>
     </row>
     <row r="97" spans="1:34">
-      <c r="A97" s="162"/>
-      <c r="B97" s="162"/>
+      <c r="A97" s="166"/>
+      <c r="B97" s="166"/>
       <c r="C97" s="41"/>
       <c r="D97" s="32"/>
       <c r="E97" s="32"/>
@@ -21168,8 +21174,8 @@
       <c r="AH97" s="34"/>
     </row>
     <row r="98" spans="1:34">
-      <c r="A98" s="162"/>
-      <c r="B98" s="162"/>
+      <c r="A98" s="166"/>
+      <c r="B98" s="166"/>
       <c r="C98" s="42"/>
       <c r="D98" s="30"/>
       <c r="E98" s="30"/>
@@ -21204,8 +21210,8 @@
       <c r="AH98" s="34"/>
     </row>
     <row r="99" spans="1:34">
-      <c r="A99" s="162"/>
-      <c r="B99" s="162"/>
+      <c r="A99" s="166"/>
+      <c r="B99" s="166"/>
       <c r="C99" s="40"/>
       <c r="D99" s="32"/>
       <c r="E99" s="32"/>
@@ -21240,8 +21246,8 @@
       <c r="AH99" s="33"/>
     </row>
     <row r="100" spans="1:34">
-      <c r="A100" s="162"/>
-      <c r="B100" s="162"/>
+      <c r="A100" s="166"/>
+      <c r="B100" s="166"/>
       <c r="C100" s="41"/>
       <c r="D100" s="30"/>
       <c r="E100" s="30"/>
@@ -21276,8 +21282,8 @@
       <c r="AH100" s="34"/>
     </row>
     <row r="101" spans="1:34">
-      <c r="A101" s="164"/>
-      <c r="B101" s="164"/>
+      <c r="A101" s="167"/>
+      <c r="B101" s="167"/>
       <c r="C101" s="42"/>
       <c r="D101" s="32"/>
       <c r="E101" s="32"/>
@@ -21312,9 +21318,9 @@
       <c r="AH101" s="34"/>
     </row>
     <row r="102" spans="1:34">
-      <c r="A102" s="173"/>
-      <c r="B102" s="165"/>
-      <c r="C102" s="166"/>
+      <c r="A102" s="174"/>
+      <c r="B102" s="162"/>
+      <c r="C102" s="164"/>
       <c r="D102" s="30"/>
       <c r="E102" s="30"/>
       <c r="F102" s="30"/>
@@ -21348,9 +21354,9 @@
       <c r="AH102" s="33"/>
     </row>
     <row r="103" spans="1:34">
-      <c r="A103" s="174"/>
-      <c r="B103" s="165"/>
-      <c r="C103" s="166"/>
+      <c r="A103" s="175"/>
+      <c r="B103" s="162"/>
+      <c r="C103" s="164"/>
       <c r="D103" s="32"/>
       <c r="E103" s="32"/>
       <c r="F103" s="32"/>
@@ -21384,9 +21390,9 @@
       <c r="AH103" s="33"/>
     </row>
     <row r="104" spans="1:34">
-      <c r="A104" s="174"/>
-      <c r="B104" s="165"/>
-      <c r="C104" s="166"/>
+      <c r="A104" s="175"/>
+      <c r="B104" s="162"/>
+      <c r="C104" s="164"/>
       <c r="D104" s="30"/>
       <c r="E104" s="30"/>
       <c r="F104" s="30"/>
@@ -21420,9 +21426,9 @@
       <c r="AH104" s="33"/>
     </row>
     <row r="105" spans="1:34">
-      <c r="A105" s="174"/>
-      <c r="B105" s="165"/>
-      <c r="C105" s="166"/>
+      <c r="A105" s="175"/>
+      <c r="B105" s="162"/>
+      <c r="C105" s="164"/>
       <c r="D105" s="32"/>
       <c r="E105" s="32"/>
       <c r="F105" s="32"/>
@@ -21456,9 +21462,9 @@
       <c r="AH105" s="33"/>
     </row>
     <row r="106" spans="1:34">
-      <c r="A106" s="175"/>
-      <c r="B106" s="165"/>
-      <c r="C106" s="166"/>
+      <c r="A106" s="176"/>
+      <c r="B106" s="162"/>
+      <c r="C106" s="164"/>
       <c r="D106" s="30"/>
       <c r="E106" s="30"/>
       <c r="F106" s="30"/>
@@ -21492,8 +21498,8 @@
       <c r="AH106" s="33"/>
     </row>
     <row r="107" spans="1:34" ht="15.5" customHeight="1">
-      <c r="A107" s="169"/>
-      <c r="B107" s="170"/>
+      <c r="A107" s="171"/>
+      <c r="B107" s="168"/>
       <c r="C107" s="43"/>
       <c r="D107" s="32"/>
       <c r="E107" s="32"/>
@@ -21528,8 +21534,8 @@
       <c r="AH107" s="32"/>
     </row>
     <row r="108" spans="1:34">
-      <c r="A108" s="167"/>
-      <c r="B108" s="168"/>
+      <c r="A108" s="172"/>
+      <c r="B108" s="169"/>
       <c r="C108" s="44"/>
       <c r="D108" s="30"/>
       <c r="E108" s="30"/>
@@ -21564,8 +21570,8 @@
       <c r="AH108" s="30"/>
     </row>
     <row r="109" spans="1:34">
-      <c r="A109" s="171"/>
-      <c r="B109" s="172"/>
+      <c r="A109" s="173"/>
+      <c r="B109" s="170"/>
       <c r="C109" s="44"/>
       <c r="D109" s="32"/>
       <c r="E109" s="32"/>
@@ -21636,8 +21642,8 @@
       <c r="AH110" s="129"/>
     </row>
     <row r="111" spans="1:34" ht="15.5" customHeight="1">
-      <c r="A111" s="169"/>
-      <c r="B111" s="170"/>
+      <c r="A111" s="171"/>
+      <c r="B111" s="168"/>
       <c r="C111" s="43"/>
       <c r="D111" s="32"/>
       <c r="E111" s="32"/>
@@ -21672,8 +21678,8 @@
       <c r="AH111" s="32"/>
     </row>
     <row r="112" spans="1:34">
-      <c r="A112" s="167"/>
-      <c r="B112" s="168"/>
+      <c r="A112" s="172"/>
+      <c r="B112" s="169"/>
       <c r="C112" s="44"/>
       <c r="D112" s="30"/>
       <c r="E112" s="30"/>
@@ -21708,8 +21714,8 @@
       <c r="AH112" s="30"/>
     </row>
     <row r="113" spans="1:34">
-      <c r="A113" s="167"/>
-      <c r="B113" s="168"/>
+      <c r="A113" s="172"/>
+      <c r="B113" s="169"/>
       <c r="C113" s="44"/>
       <c r="D113" s="32"/>
       <c r="E113" s="32"/>
@@ -21753,7 +21759,7 @@
       <c r="AE115" s="33"/>
     </row>
     <row r="117" spans="1:34" ht="27.5" customHeight="1">
-      <c r="A117" s="143"/>
+      <c r="A117" s="144"/>
       <c r="B117" s="137"/>
       <c r="Z117" s="131"/>
       <c r="AA117" s="131"/>
@@ -21761,7 +21767,7 @@
       <c r="AC117" s="131"/>
     </row>
     <row r="118" spans="1:34">
-      <c r="A118" s="143"/>
+      <c r="A118" s="144"/>
       <c r="B118" s="137"/>
       <c r="Z118" s="131"/>
       <c r="AA118" s="131"/>
@@ -21769,7 +21775,7 @@
       <c r="AC118" s="131"/>
     </row>
     <row r="119" spans="1:34">
-      <c r="A119" s="143"/>
+      <c r="A119" s="144"/>
       <c r="B119" s="137"/>
       <c r="Z119" s="131"/>
       <c r="AA119" s="131"/>
@@ -21777,7 +21783,7 @@
       <c r="AC119" s="131"/>
     </row>
     <row r="120" spans="1:34">
-      <c r="A120" s="143"/>
+      <c r="A120" s="144"/>
       <c r="B120" s="137"/>
       <c r="Z120" s="131"/>
       <c r="AA120" s="131"/>
@@ -21785,7 +21791,7 @@
       <c r="AC120" s="131"/>
     </row>
     <row r="121" spans="1:34">
-      <c r="A121" s="143"/>
+      <c r="A121" s="144"/>
       <c r="B121" s="137"/>
       <c r="Z121" s="131"/>
       <c r="AA121" s="131"/>
@@ -21793,7 +21799,7 @@
       <c r="AC121" s="131"/>
     </row>
     <row r="122" spans="1:34">
-      <c r="A122" s="143"/>
+      <c r="A122" s="144"/>
       <c r="B122" s="137"/>
       <c r="Z122" s="131"/>
       <c r="AA122" s="131"/>
@@ -21801,7 +21807,7 @@
       <c r="AC122" s="131"/>
     </row>
     <row r="123" spans="1:34">
-      <c r="A123" s="143"/>
+      <c r="A123" s="144"/>
       <c r="B123" s="137"/>
       <c r="Z123" s="131"/>
       <c r="AA123" s="131"/>
@@ -21809,7 +21815,7 @@
       <c r="AC123" s="131"/>
     </row>
     <row r="124" spans="1:34">
-      <c r="A124" s="143"/>
+      <c r="A124" s="144"/>
       <c r="B124" s="137"/>
       <c r="Z124" s="131"/>
       <c r="AA124" s="131"/>
@@ -21817,7 +21823,7 @@
       <c r="AC124" s="131"/>
     </row>
     <row r="125" spans="1:34">
-      <c r="A125" s="143"/>
+      <c r="A125" s="144"/>
       <c r="B125" s="137"/>
       <c r="Z125" s="131"/>
       <c r="AA125" s="131"/>
@@ -21825,20 +21831,20 @@
       <c r="AC125" s="131"/>
     </row>
     <row r="126" spans="1:34">
-      <c r="A126" s="143"/>
+      <c r="A126" s="144"/>
       <c r="B126" s="137"/>
       <c r="C126" s="43"/>
     </row>
     <row r="127" spans="1:34">
-      <c r="A127" s="143"/>
+      <c r="A127" s="144"/>
       <c r="C127" s="44"/>
     </row>
     <row r="128" spans="1:34">
-      <c r="A128" s="143"/>
+      <c r="A128" s="144"/>
       <c r="C128" s="44"/>
     </row>
     <row r="129" spans="1:35">
-      <c r="A129" s="143" t="s">
+      <c r="A129" s="144" t="s">
         <v>394</v>
       </c>
       <c r="B129" s="137" t="s">
@@ -21852,19 +21858,19 @@
       </c>
     </row>
     <row r="130" spans="1:35">
-      <c r="A130" s="143"/>
+      <c r="A130" s="144"/>
       <c r="C130" s="44" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="131" spans="1:35">
-      <c r="A131" s="143"/>
+      <c r="A131" s="144"/>
       <c r="C131" s="44" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="132" spans="1:35">
-      <c r="A132" s="143" t="s">
+      <c r="A132" s="144" t="s">
         <v>396</v>
       </c>
       <c r="B132" s="137" t="s">
@@ -21880,7 +21886,7 @@
       <c r="AI132" s="32"/>
     </row>
     <row r="133" spans="1:35">
-      <c r="A133" s="143"/>
+      <c r="A133" s="144"/>
       <c r="C133" s="44" t="s">
         <v>22</v>
       </c>
@@ -21890,7 +21896,7 @@
       </c>
     </row>
     <row r="134" spans="1:35">
-      <c r="A134" s="143"/>
+      <c r="A134" s="144"/>
       <c r="C134" s="44" t="s">
         <v>23</v>
       </c>
@@ -21900,7 +21906,7 @@
       </c>
     </row>
     <row r="135" spans="1:35">
-      <c r="A135" s="143" t="s">
+      <c r="A135" s="144" t="s">
         <v>398</v>
       </c>
       <c r="B135" s="137" t="s">
@@ -21915,7 +21921,7 @@
       </c>
     </row>
     <row r="136" spans="1:35">
-      <c r="A136" s="143"/>
+      <c r="A136" s="144"/>
       <c r="C136" s="44" t="s">
         <v>22</v>
       </c>
@@ -21925,7 +21931,7 @@
       </c>
     </row>
     <row r="137" spans="1:35">
-      <c r="A137" s="143"/>
+      <c r="A137" s="144"/>
       <c r="C137" s="44" t="s">
         <v>23</v>
       </c>
@@ -21936,47 +21942,6 @@
     </row>
   </sheetData>
   <mergeCells count="57">
-    <mergeCell ref="A135:A137"/>
-    <mergeCell ref="A132:A134"/>
-    <mergeCell ref="A117:A119"/>
-    <mergeCell ref="A120:A122"/>
-    <mergeCell ref="A123:A125"/>
-    <mergeCell ref="A129:A131"/>
-    <mergeCell ref="A126:A128"/>
-    <mergeCell ref="A4:A18"/>
-    <mergeCell ref="A22:A36"/>
-    <mergeCell ref="A37:A51"/>
-    <mergeCell ref="A52:A66"/>
-    <mergeCell ref="A82:A86"/>
-    <mergeCell ref="A87:A101"/>
-    <mergeCell ref="A107:B109"/>
-    <mergeCell ref="A111:B113"/>
-    <mergeCell ref="A102:A106"/>
-    <mergeCell ref="B102:C102"/>
-    <mergeCell ref="B103:C103"/>
-    <mergeCell ref="B104:C104"/>
-    <mergeCell ref="B105:C105"/>
-    <mergeCell ref="B106:C106"/>
-    <mergeCell ref="B96:B98"/>
-    <mergeCell ref="B99:B101"/>
-    <mergeCell ref="B4:B6"/>
-    <mergeCell ref="B7:B9"/>
-    <mergeCell ref="B10:B12"/>
-    <mergeCell ref="B13:B15"/>
-    <mergeCell ref="B16:B18"/>
-    <mergeCell ref="B22:B24"/>
-    <mergeCell ref="B25:B27"/>
-    <mergeCell ref="B28:B30"/>
-    <mergeCell ref="B31:B33"/>
-    <mergeCell ref="B34:B36"/>
-    <mergeCell ref="B58:B60"/>
-    <mergeCell ref="B61:B63"/>
-    <mergeCell ref="B64:B66"/>
-    <mergeCell ref="B37:B39"/>
-    <mergeCell ref="B40:B42"/>
-    <mergeCell ref="B43:B45"/>
-    <mergeCell ref="B46:B48"/>
-    <mergeCell ref="B49:B51"/>
     <mergeCell ref="B19:B21"/>
     <mergeCell ref="A19:A21"/>
     <mergeCell ref="B87:B89"/>
@@ -21993,6 +21958,47 @@
     <mergeCell ref="B79:B81"/>
     <mergeCell ref="B52:B54"/>
     <mergeCell ref="B55:B57"/>
+    <mergeCell ref="B58:B60"/>
+    <mergeCell ref="B61:B63"/>
+    <mergeCell ref="B64:B66"/>
+    <mergeCell ref="B37:B39"/>
+    <mergeCell ref="B40:B42"/>
+    <mergeCell ref="B43:B45"/>
+    <mergeCell ref="B46:B48"/>
+    <mergeCell ref="B49:B51"/>
+    <mergeCell ref="B22:B24"/>
+    <mergeCell ref="B25:B27"/>
+    <mergeCell ref="B28:B30"/>
+    <mergeCell ref="B31:B33"/>
+    <mergeCell ref="B34:B36"/>
+    <mergeCell ref="B4:B6"/>
+    <mergeCell ref="B7:B9"/>
+    <mergeCell ref="B10:B12"/>
+    <mergeCell ref="B13:B15"/>
+    <mergeCell ref="B16:B18"/>
+    <mergeCell ref="A87:A101"/>
+    <mergeCell ref="A107:B109"/>
+    <mergeCell ref="A111:B113"/>
+    <mergeCell ref="A102:A106"/>
+    <mergeCell ref="B102:C102"/>
+    <mergeCell ref="B103:C103"/>
+    <mergeCell ref="B104:C104"/>
+    <mergeCell ref="B105:C105"/>
+    <mergeCell ref="B106:C106"/>
+    <mergeCell ref="B96:B98"/>
+    <mergeCell ref="B99:B101"/>
+    <mergeCell ref="A4:A18"/>
+    <mergeCell ref="A22:A36"/>
+    <mergeCell ref="A37:A51"/>
+    <mergeCell ref="A52:A66"/>
+    <mergeCell ref="A82:A86"/>
+    <mergeCell ref="A135:A137"/>
+    <mergeCell ref="A132:A134"/>
+    <mergeCell ref="A117:A119"/>
+    <mergeCell ref="A120:A122"/>
+    <mergeCell ref="A123:A125"/>
+    <mergeCell ref="A129:A131"/>
+    <mergeCell ref="A126:A128"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -22362,7 +22368,7 @@
       <c r="AH4" s="28"/>
     </row>
     <row r="5" spans="1:36">
-      <c r="A5" s="145"/>
+      <c r="A5" s="143"/>
       <c r="B5" s="53"/>
       <c r="C5" s="45"/>
       <c r="D5" s="29"/>
@@ -22398,7 +22404,7 @@
       <c r="AH5" s="29"/>
     </row>
     <row r="6" spans="1:36">
-      <c r="A6" s="145"/>
+      <c r="A6" s="143"/>
       <c r="B6" s="53"/>
       <c r="C6" s="46"/>
       <c r="D6" s="30"/>
@@ -22434,7 +22440,7 @@
       <c r="AH6" s="30"/>
     </row>
     <row r="7" spans="1:36">
-      <c r="A7" s="145"/>
+      <c r="A7" s="143"/>
       <c r="B7" s="53"/>
       <c r="C7" s="46"/>
       <c r="D7" s="30"/>
@@ -22470,8 +22476,8 @@
       <c r="AH7" s="30"/>
     </row>
     <row r="8" spans="1:36">
-      <c r="A8" s="145"/>
-      <c r="B8" s="167"/>
+      <c r="A8" s="143"/>
+      <c r="B8" s="172"/>
       <c r="C8" s="40"/>
       <c r="D8" s="32"/>
       <c r="E8" s="32"/>
@@ -22506,8 +22512,8 @@
       <c r="AH8" s="32"/>
     </row>
     <row r="9" spans="1:36">
-      <c r="A9" s="145"/>
-      <c r="B9" s="162"/>
+      <c r="A9" s="143"/>
+      <c r="B9" s="166"/>
       <c r="C9" s="41"/>
       <c r="D9" s="30"/>
       <c r="E9" s="30"/>
@@ -22542,8 +22548,8 @@
       <c r="AH9" s="30"/>
     </row>
     <row r="10" spans="1:36">
-      <c r="A10" s="145"/>
-      <c r="B10" s="168"/>
+      <c r="A10" s="143"/>
+      <c r="B10" s="169"/>
       <c r="C10" s="42"/>
       <c r="D10" s="32"/>
       <c r="E10" s="32"/>
@@ -22578,8 +22584,8 @@
       <c r="AH10" s="30"/>
     </row>
     <row r="11" spans="1:36">
-      <c r="A11" s="145"/>
-      <c r="B11" s="167"/>
+      <c r="A11" s="143"/>
+      <c r="B11" s="172"/>
       <c r="C11" s="40"/>
       <c r="D11" s="30"/>
       <c r="E11" s="30"/>
@@ -22614,8 +22620,8 @@
       <c r="AH11" s="32"/>
     </row>
     <row r="12" spans="1:36">
-      <c r="A12" s="145"/>
-      <c r="B12" s="162"/>
+      <c r="A12" s="143"/>
+      <c r="B12" s="166"/>
       <c r="C12" s="41"/>
       <c r="D12" s="32"/>
       <c r="E12" s="32"/>
@@ -22650,8 +22656,8 @@
       <c r="AH12" s="30"/>
     </row>
     <row r="13" spans="1:36">
-      <c r="A13" s="145"/>
-      <c r="B13" s="168"/>
+      <c r="A13" s="143"/>
+      <c r="B13" s="169"/>
       <c r="C13" s="42"/>
       <c r="D13" s="30"/>
       <c r="E13" s="30"/>
@@ -22686,7 +22692,7 @@
       <c r="AH13" s="30"/>
     </row>
     <row r="14" spans="1:36">
-      <c r="A14" s="145"/>
+      <c r="A14" s="143"/>
       <c r="B14" s="177"/>
       <c r="C14" s="40"/>
       <c r="D14" s="32"/>
@@ -22722,7 +22728,7 @@
       <c r="AH14" s="32"/>
     </row>
     <row r="15" spans="1:36">
-      <c r="A15" s="145"/>
+      <c r="A15" s="143"/>
       <c r="B15" s="178"/>
       <c r="C15" s="41"/>
       <c r="D15" s="30"/>
@@ -22758,7 +22764,7 @@
       <c r="AH15" s="30"/>
     </row>
     <row r="16" spans="1:36">
-      <c r="A16" s="145"/>
+      <c r="A16" s="143"/>
       <c r="B16" s="179"/>
       <c r="C16" s="42"/>
       <c r="D16" s="32"/>
@@ -22794,56 +22800,56 @@
       <c r="AH16" s="30"/>
     </row>
     <row r="17" spans="1:31">
-      <c r="A17" s="145"/>
-      <c r="B17" s="167"/>
+      <c r="A17" s="143"/>
+      <c r="B17" s="172"/>
       <c r="C17" s="40"/>
       <c r="AB17" s="32"/>
       <c r="AE17" s="32"/>
     </row>
     <row r="18" spans="1:31">
-      <c r="A18" s="145"/>
-      <c r="B18" s="162"/>
+      <c r="A18" s="143"/>
+      <c r="B18" s="166"/>
       <c r="C18" s="41"/>
       <c r="AB18" s="32"/>
       <c r="AE18" s="32"/>
     </row>
     <row r="19" spans="1:31">
-      <c r="A19" s="145"/>
-      <c r="B19" s="168"/>
+      <c r="A19" s="143"/>
+      <c r="B19" s="169"/>
       <c r="C19" s="42"/>
       <c r="AB19" s="32"/>
       <c r="AE19" s="32"/>
     </row>
     <row r="20" spans="1:31">
-      <c r="A20" s="145"/>
-      <c r="B20" s="167"/>
+      <c r="A20" s="143"/>
+      <c r="B20" s="172"/>
       <c r="C20" s="40"/>
       <c r="AB20" s="32"/>
       <c r="AE20" s="32"/>
     </row>
     <row r="21" spans="1:31">
-      <c r="A21" s="145"/>
-      <c r="B21" s="162"/>
+      <c r="A21" s="143"/>
+      <c r="B21" s="166"/>
       <c r="C21" s="41"/>
       <c r="AB21" s="32"/>
       <c r="AE21" s="32"/>
     </row>
     <row r="22" spans="1:31">
-      <c r="A22" s="145"/>
-      <c r="B22" s="168"/>
+      <c r="A22" s="143"/>
+      <c r="B22" s="169"/>
       <c r="C22" s="42"/>
       <c r="AB22" s="32"/>
       <c r="AE22" s="32"/>
     </row>
     <row r="23" spans="1:31">
-      <c r="A23" s="145"/>
+      <c r="A23" s="143"/>
       <c r="B23" s="177"/>
       <c r="C23" s="41"/>
       <c r="AB23" s="32"/>
       <c r="AE23" s="32"/>
     </row>
     <row r="24" spans="1:31">
-      <c r="A24" s="145"/>
+      <c r="A24" s="143"/>
       <c r="B24" s="178"/>
       <c r="C24" s="41"/>
       <c r="X24" s="32"/>
@@ -22851,7 +22857,7 @@
       <c r="AE24" s="32"/>
     </row>
     <row r="25" spans="1:31">
-      <c r="A25" s="145"/>
+      <c r="A25" s="143"/>
       <c r="B25" s="179"/>
       <c r="C25" s="41"/>
       <c r="X25" s="32"/>
@@ -22859,92 +22865,92 @@
       <c r="AE25" s="32"/>
     </row>
     <row r="26" spans="1:31">
-      <c r="A26" s="145"/>
-      <c r="B26" s="167"/>
+      <c r="A26" s="143"/>
+      <c r="B26" s="172"/>
       <c r="C26" s="40"/>
       <c r="X26" s="32"/>
       <c r="AB26" s="32"/>
       <c r="AE26" s="32"/>
     </row>
     <row r="27" spans="1:31">
-      <c r="A27" s="145"/>
-      <c r="B27" s="162"/>
+      <c r="A27" s="143"/>
+      <c r="B27" s="166"/>
       <c r="C27" s="41"/>
       <c r="X27" s="32"/>
       <c r="AB27" s="54"/>
       <c r="AE27" s="32"/>
     </row>
     <row r="28" spans="1:31">
-      <c r="A28" s="145"/>
-      <c r="B28" s="168"/>
+      <c r="A28" s="143"/>
+      <c r="B28" s="169"/>
       <c r="C28" s="42"/>
       <c r="X28" s="32"/>
       <c r="AE28" s="32"/>
     </row>
     <row r="29" spans="1:31">
-      <c r="A29" s="145"/>
-      <c r="B29" s="167"/>
+      <c r="A29" s="143"/>
+      <c r="B29" s="172"/>
       <c r="C29" s="40"/>
       <c r="X29" s="32"/>
       <c r="AE29" s="32"/>
     </row>
     <row r="30" spans="1:31">
-      <c r="A30" s="145"/>
-      <c r="B30" s="162"/>
+      <c r="A30" s="143"/>
+      <c r="B30" s="166"/>
       <c r="C30" s="41"/>
       <c r="X30" s="32"/>
       <c r="AE30" s="32"/>
     </row>
     <row r="31" spans="1:31">
-      <c r="A31" s="145"/>
-      <c r="B31" s="168"/>
+      <c r="A31" s="143"/>
+      <c r="B31" s="169"/>
       <c r="C31" s="42"/>
       <c r="X31" s="32"/>
       <c r="AE31" s="32"/>
     </row>
     <row r="32" spans="1:31">
-      <c r="A32" s="145"/>
-      <c r="B32" s="167"/>
+      <c r="A32" s="143"/>
+      <c r="B32" s="172"/>
       <c r="C32" s="40"/>
       <c r="X32" s="32"/>
       <c r="AE32" s="32"/>
     </row>
     <row r="33" spans="1:36">
-      <c r="A33" s="145"/>
-      <c r="B33" s="162"/>
+      <c r="A33" s="143"/>
+      <c r="B33" s="166"/>
       <c r="C33" s="41"/>
       <c r="X33" s="32"/>
       <c r="AE33" s="32"/>
     </row>
     <row r="34" spans="1:36">
-      <c r="A34" s="145"/>
-      <c r="B34" s="168"/>
+      <c r="A34" s="143"/>
+      <c r="B34" s="169"/>
       <c r="C34" s="42"/>
       <c r="X34" s="32"/>
       <c r="AE34" s="32"/>
     </row>
     <row r="35" spans="1:36">
-      <c r="A35" s="162"/>
+      <c r="A35" s="166"/>
       <c r="B35" s="177"/>
       <c r="C35" s="40"/>
       <c r="X35" s="32"/>
       <c r="AE35" s="32"/>
     </row>
     <row r="36" spans="1:36">
-      <c r="A36" s="162"/>
+      <c r="A36" s="166"/>
       <c r="B36" s="178"/>
       <c r="C36" s="41"/>
       <c r="X36" s="32"/>
       <c r="AE36" s="32"/>
     </row>
     <row r="37" spans="1:36">
-      <c r="A37" s="162"/>
+      <c r="A37" s="166"/>
       <c r="B37" s="179"/>
       <c r="C37" s="42"/>
       <c r="AE37" s="32"/>
     </row>
     <row r="38" spans="1:36">
-      <c r="A38" s="162" t="s">
+      <c r="A38" s="166" t="s">
         <v>390</v>
       </c>
       <c r="B38" s="177" t="s">
@@ -22958,7 +22964,7 @@
       </c>
     </row>
     <row r="39" spans="1:36">
-      <c r="A39" s="162"/>
+      <c r="A39" s="166"/>
       <c r="B39" s="178"/>
       <c r="C39" s="41" t="s">
         <v>22</v>
@@ -22968,7 +22974,7 @@
       </c>
     </row>
     <row r="40" spans="1:36">
-      <c r="A40" s="162"/>
+      <c r="A40" s="166"/>
       <c r="B40" s="179"/>
       <c r="C40" s="42" t="s">
         <v>23</v>
@@ -22978,7 +22984,7 @@
       </c>
     </row>
     <row r="41" spans="1:36">
-      <c r="A41" s="162" t="s">
+      <c r="A41" s="166" t="s">
         <v>395</v>
       </c>
       <c r="B41" s="177" t="s">
@@ -23004,7 +23010,7 @@
       </c>
     </row>
     <row r="42" spans="1:36">
-      <c r="A42" s="162"/>
+      <c r="A42" s="166"/>
       <c r="B42" s="178"/>
       <c r="C42" s="41" t="s">
         <v>22</v>
@@ -23023,7 +23029,7 @@
       </c>
     </row>
     <row r="43" spans="1:36">
-      <c r="A43" s="162"/>
+      <c r="A43" s="166"/>
       <c r="B43" s="179"/>
       <c r="C43" s="42" t="s">
         <v>23</v>
@@ -23042,7 +23048,7 @@
       </c>
     </row>
     <row r="44" spans="1:36">
-      <c r="A44" s="162" t="s">
+      <c r="A44" s="166" t="s">
         <v>400</v>
       </c>
       <c r="B44" s="177" t="s">
@@ -23065,7 +23071,7 @@
       </c>
     </row>
     <row r="45" spans="1:36">
-      <c r="A45" s="162"/>
+      <c r="A45" s="166"/>
       <c r="B45" s="178"/>
       <c r="C45" s="41" t="s">
         <v>22</v>
@@ -23081,7 +23087,7 @@
       </c>
     </row>
     <row r="46" spans="1:36">
-      <c r="A46" s="162"/>
+      <c r="A46" s="166"/>
       <c r="B46" s="179"/>
       <c r="C46" s="42" t="s">
         <v>23</v>
@@ -23097,7 +23103,7 @@
       </c>
     </row>
     <row r="47" spans="1:36" ht="30">
-      <c r="A47" s="168" t="s">
+      <c r="A47" s="169" t="s">
         <v>382</v>
       </c>
       <c r="B47" s="135" t="s">
@@ -23112,7 +23118,7 @@
       <c r="AE47" s="32"/>
     </row>
     <row r="48" spans="1:36" ht="30">
-      <c r="A48" s="168"/>
+      <c r="A48" s="169"/>
       <c r="B48" s="135" t="s">
         <v>102</v>
       </c>
@@ -23129,11 +23135,14 @@
     </row>
   </sheetData>
   <mergeCells count="22">
-    <mergeCell ref="A5:A7"/>
-    <mergeCell ref="B8:B10"/>
-    <mergeCell ref="B11:B13"/>
-    <mergeCell ref="B14:B16"/>
-    <mergeCell ref="A8:A16"/>
+    <mergeCell ref="B41:B43"/>
+    <mergeCell ref="A38:A40"/>
+    <mergeCell ref="A41:A43"/>
+    <mergeCell ref="A47:A48"/>
+    <mergeCell ref="B35:B37"/>
+    <mergeCell ref="A35:A37"/>
+    <mergeCell ref="A44:A46"/>
+    <mergeCell ref="B44:B46"/>
     <mergeCell ref="B23:B25"/>
     <mergeCell ref="B38:B40"/>
     <mergeCell ref="B29:B31"/>
@@ -23143,14 +23152,11 @@
     <mergeCell ref="B17:B19"/>
     <mergeCell ref="B20:B22"/>
     <mergeCell ref="B26:B28"/>
-    <mergeCell ref="B41:B43"/>
-    <mergeCell ref="A38:A40"/>
-    <mergeCell ref="A41:A43"/>
-    <mergeCell ref="A47:A48"/>
-    <mergeCell ref="B35:B37"/>
-    <mergeCell ref="A35:A37"/>
-    <mergeCell ref="A44:A46"/>
-    <mergeCell ref="B44:B46"/>
+    <mergeCell ref="A5:A7"/>
+    <mergeCell ref="B8:B10"/>
+    <mergeCell ref="B11:B13"/>
+    <mergeCell ref="B14:B16"/>
+    <mergeCell ref="A8:A16"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -24205,15 +24211,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8">
-      <c r="A1" s="206" t="s">
+      <c r="A1" s="191" t="s">
         <v>233</v>
       </c>
       <c r="B1" s="73"/>
-      <c r="C1" s="206" t="s">
+      <c r="C1" s="191" t="s">
         <v>235</v>
       </c>
       <c r="D1" s="73"/>
-      <c r="E1" s="206" t="s">
+      <c r="E1" s="191" t="s">
         <v>237</v>
       </c>
       <c r="F1" s="73"/>
@@ -24223,15 +24229,15 @@
       <c r="H1" s="73"/>
     </row>
     <row r="2" spans="1:8" ht="27" thickBot="1">
-      <c r="A2" s="207"/>
+      <c r="A2" s="192"/>
       <c r="B2" s="74" t="s">
         <v>234</v>
       </c>
-      <c r="C2" s="207"/>
+      <c r="C2" s="192"/>
       <c r="D2" s="74" t="s">
         <v>236</v>
       </c>
-      <c r="E2" s="207"/>
+      <c r="E2" s="192"/>
       <c r="F2" s="74" t="s">
         <v>238</v>
       </c>
@@ -24260,7 +24266,7 @@
       <c r="C4" s="79"/>
       <c r="D4" s="79"/>
       <c r="E4" s="79"/>
-      <c r="F4" s="196" t="s">
+      <c r="F4" s="189" t="s">
         <v>244</v>
       </c>
       <c r="G4" s="79"/>
@@ -24282,7 +24288,7 @@
       <c r="E5" s="80">
         <v>0</v>
       </c>
-      <c r="F5" s="198"/>
+      <c r="F5" s="190"/>
       <c r="G5" s="80" t="s">
         <v>245</v>
       </c>
@@ -24296,7 +24302,7 @@
       <c r="C6" s="79"/>
       <c r="D6" s="79"/>
       <c r="E6" s="79"/>
-      <c r="F6" s="196" t="s">
+      <c r="F6" s="189" t="s">
         <v>244</v>
       </c>
       <c r="G6" s="79"/>
@@ -24318,7 +24324,7 @@
       <c r="E7" s="80">
         <v>0</v>
       </c>
-      <c r="F7" s="198"/>
+      <c r="F7" s="190"/>
       <c r="G7" s="80" t="s">
         <v>245</v>
       </c>
@@ -24332,7 +24338,7 @@
       <c r="C8" s="79"/>
       <c r="D8" s="79"/>
       <c r="E8" s="79"/>
-      <c r="F8" s="196" t="s">
+      <c r="F8" s="189" t="s">
         <v>244</v>
       </c>
       <c r="G8" s="79"/>
@@ -24354,7 +24360,7 @@
       <c r="E9" s="80">
         <v>0</v>
       </c>
-      <c r="F9" s="198"/>
+      <c r="F9" s="190"/>
       <c r="G9" s="80" t="s">
         <v>245</v>
       </c>
@@ -24364,28 +24370,28 @@
     </row>
     <row r="10" spans="1:8" ht="24" customHeight="1" thickBot="1">
       <c r="A10" s="76"/>
-      <c r="B10" s="199" t="s">
+      <c r="B10" s="193" t="s">
         <v>249</v>
       </c>
-      <c r="C10" s="200"/>
-      <c r="D10" s="200"/>
-      <c r="E10" s="200"/>
-      <c r="F10" s="200"/>
-      <c r="G10" s="200"/>
-      <c r="H10" s="201"/>
+      <c r="C10" s="194"/>
+      <c r="D10" s="194"/>
+      <c r="E10" s="194"/>
+      <c r="F10" s="194"/>
+      <c r="G10" s="194"/>
+      <c r="H10" s="195"/>
     </row>
     <row r="11" spans="1:8">
       <c r="A11" s="82"/>
-      <c r="B11" s="196" t="s">
+      <c r="B11" s="189" t="s">
         <v>250</v>
       </c>
-      <c r="C11" s="196" t="s">
+      <c r="C11" s="189" t="s">
         <v>251</v>
       </c>
-      <c r="D11" s="196" t="s">
+      <c r="D11" s="189" t="s">
         <v>252</v>
       </c>
-      <c r="E11" s="196" t="s">
+      <c r="E11" s="189" t="s">
         <v>253</v>
       </c>
       <c r="F11" s="83"/>
@@ -24396,10 +24402,10 @@
       <c r="A12" s="78">
         <v>1</v>
       </c>
-      <c r="B12" s="198"/>
-      <c r="C12" s="198"/>
-      <c r="D12" s="198"/>
-      <c r="E12" s="198"/>
+      <c r="B12" s="190"/>
+      <c r="C12" s="190"/>
+      <c r="D12" s="190"/>
+      <c r="E12" s="190"/>
       <c r="F12" s="80" t="s">
         <v>254</v>
       </c>
@@ -24412,7 +24418,7 @@
     </row>
     <row r="13" spans="1:8">
       <c r="A13" s="82"/>
-      <c r="B13" s="196" t="s">
+      <c r="B13" s="189" t="s">
         <v>257</v>
       </c>
       <c r="C13" s="81" t="s">
@@ -24432,7 +24438,7 @@
       <c r="A14" s="84">
         <v>2</v>
       </c>
-      <c r="B14" s="197"/>
+      <c r="B14" s="196"/>
       <c r="C14" s="81" t="s">
         <v>259</v>
       </c>
@@ -24454,7 +24460,7 @@
     </row>
     <row r="15" spans="1:8" ht="17" thickBot="1">
       <c r="A15" s="85"/>
-      <c r="B15" s="198"/>
+      <c r="B15" s="190"/>
       <c r="C15" s="86"/>
       <c r="D15" s="80" t="s">
         <v>262</v>
@@ -24468,25 +24474,25 @@
     </row>
     <row r="16" spans="1:8" s="37" customFormat="1">
       <c r="A16" s="102"/>
-      <c r="B16" s="189" t="s">
+      <c r="B16" s="197" t="s">
         <v>265</v>
       </c>
-      <c r="C16" s="204">
+      <c r="C16" s="199">
         <v>0.5</v>
       </c>
-      <c r="D16" s="204">
+      <c r="D16" s="199">
         <v>0.7</v>
       </c>
-      <c r="E16" s="204">
+      <c r="E16" s="199">
         <v>0.9</v>
       </c>
-      <c r="F16" s="189" t="s">
+      <c r="F16" s="197" t="s">
         <v>254</v>
       </c>
-      <c r="G16" s="189" t="s">
+      <c r="G16" s="197" t="s">
         <v>266</v>
       </c>
-      <c r="H16" s="189" t="s">
+      <c r="H16" s="197" t="s">
         <v>256</v>
       </c>
     </row>
@@ -24494,35 +24500,35 @@
       <c r="A17" s="99">
         <v>3</v>
       </c>
-      <c r="B17" s="190"/>
-      <c r="C17" s="205"/>
-      <c r="D17" s="205"/>
-      <c r="E17" s="205"/>
-      <c r="F17" s="190"/>
-      <c r="G17" s="190"/>
-      <c r="H17" s="190"/>
+      <c r="B17" s="198"/>
+      <c r="C17" s="200"/>
+      <c r="D17" s="200"/>
+      <c r="E17" s="200"/>
+      <c r="F17" s="198"/>
+      <c r="G17" s="198"/>
+      <c r="H17" s="198"/>
     </row>
     <row r="18" spans="1:8">
       <c r="A18" s="82"/>
-      <c r="B18" s="196" t="s">
+      <c r="B18" s="189" t="s">
         <v>267</v>
       </c>
-      <c r="C18" s="196" t="s">
+      <c r="C18" s="189" t="s">
         <v>268</v>
       </c>
-      <c r="D18" s="196" t="s">
+      <c r="D18" s="189" t="s">
         <v>245</v>
       </c>
-      <c r="E18" s="196" t="s">
+      <c r="E18" s="189" t="s">
         <v>245</v>
       </c>
-      <c r="F18" s="196" t="s">
+      <c r="F18" s="189" t="s">
         <v>269</v>
       </c>
-      <c r="G18" s="196" t="s">
+      <c r="G18" s="189" t="s">
         <v>255</v>
       </c>
-      <c r="H18" s="196" t="s">
+      <c r="H18" s="189" t="s">
         <v>270</v>
       </c>
     </row>
@@ -24530,13 +24536,13 @@
       <c r="A19" s="78">
         <v>4</v>
       </c>
-      <c r="B19" s="198"/>
-      <c r="C19" s="198"/>
-      <c r="D19" s="198"/>
-      <c r="E19" s="198"/>
-      <c r="F19" s="198"/>
-      <c r="G19" s="198"/>
-      <c r="H19" s="198"/>
+      <c r="B19" s="190"/>
+      <c r="C19" s="190"/>
+      <c r="D19" s="190"/>
+      <c r="E19" s="190"/>
+      <c r="F19" s="190"/>
+      <c r="G19" s="190"/>
+      <c r="H19" s="190"/>
     </row>
     <row r="20" spans="1:8" ht="27" thickBot="1">
       <c r="A20" s="78">
@@ -24592,25 +24598,25 @@
     </row>
     <row r="22" spans="1:8" ht="17" thickBot="1">
       <c r="A22" s="88"/>
-      <c r="B22" s="199" t="s">
+      <c r="B22" s="193" t="s">
         <v>276</v>
       </c>
-      <c r="C22" s="200"/>
-      <c r="D22" s="200"/>
-      <c r="E22" s="200"/>
-      <c r="F22" s="200"/>
-      <c r="G22" s="200"/>
-      <c r="H22" s="201"/>
+      <c r="C22" s="194"/>
+      <c r="D22" s="194"/>
+      <c r="E22" s="194"/>
+      <c r="F22" s="194"/>
+      <c r="G22" s="194"/>
+      <c r="H22" s="195"/>
     </row>
     <row r="23" spans="1:8">
       <c r="A23" s="89"/>
-      <c r="B23" s="196" t="s">
+      <c r="B23" s="189" t="s">
         <v>277</v>
       </c>
       <c r="C23" s="79"/>
       <c r="D23" s="90"/>
       <c r="E23" s="79"/>
-      <c r="F23" s="196" t="s">
+      <c r="F23" s="189" t="s">
         <v>281</v>
       </c>
       <c r="G23" s="90"/>
@@ -24620,7 +24626,7 @@
       <c r="A24" s="78">
         <v>1</v>
       </c>
-      <c r="B24" s="198"/>
+      <c r="B24" s="190"/>
       <c r="C24" s="80" t="s">
         <v>278</v>
       </c>
@@ -24630,7 +24636,7 @@
       <c r="E24" s="80" t="s">
         <v>280</v>
       </c>
-      <c r="F24" s="198"/>
+      <c r="F24" s="190"/>
       <c r="G24" s="80" t="s">
         <v>282</v>
       </c>
@@ -24640,25 +24646,25 @@
     </row>
     <row r="25" spans="1:8" s="37" customFormat="1">
       <c r="A25" s="98"/>
-      <c r="B25" s="189" t="s">
+      <c r="B25" s="197" t="s">
         <v>284</v>
       </c>
-      <c r="C25" s="202">
+      <c r="C25" s="201">
         <v>2765</v>
       </c>
-      <c r="D25" s="189" t="s">
+      <c r="D25" s="197" t="s">
         <v>285</v>
       </c>
-      <c r="E25" s="189" t="s">
+      <c r="E25" s="197" t="s">
         <v>46</v>
       </c>
-      <c r="F25" s="189" t="s">
+      <c r="F25" s="197" t="s">
         <v>286</v>
       </c>
-      <c r="G25" s="189" t="s">
+      <c r="G25" s="197" t="s">
         <v>272</v>
       </c>
-      <c r="H25" s="189" t="s">
+      <c r="H25" s="197" t="s">
         <v>287</v>
       </c>
     </row>
@@ -24666,23 +24672,23 @@
       <c r="A26" s="99">
         <v>2</v>
       </c>
-      <c r="B26" s="190"/>
-      <c r="C26" s="203"/>
-      <c r="D26" s="190"/>
-      <c r="E26" s="190"/>
-      <c r="F26" s="190"/>
-      <c r="G26" s="190"/>
-      <c r="H26" s="190"/>
+      <c r="B26" s="198"/>
+      <c r="C26" s="202"/>
+      <c r="D26" s="198"/>
+      <c r="E26" s="198"/>
+      <c r="F26" s="198"/>
+      <c r="G26" s="198"/>
+      <c r="H26" s="198"/>
     </row>
     <row r="27" spans="1:8">
       <c r="A27" s="82"/>
-      <c r="B27" s="196" t="s">
+      <c r="B27" s="189" t="s">
         <v>288</v>
       </c>
       <c r="C27" s="79"/>
       <c r="D27" s="79"/>
       <c r="E27" s="79"/>
-      <c r="F27" s="196" t="s">
+      <c r="F27" s="189" t="s">
         <v>289</v>
       </c>
       <c r="G27" s="79"/>
@@ -24692,7 +24698,7 @@
       <c r="A28" s="78">
         <v>3</v>
       </c>
-      <c r="B28" s="198"/>
+      <c r="B28" s="190"/>
       <c r="C28" s="91">
         <v>3.5999999999999997E-2</v>
       </c>
@@ -24702,7 +24708,7 @@
       <c r="E28" s="92">
         <v>0.95</v>
       </c>
-      <c r="F28" s="198"/>
+      <c r="F28" s="190"/>
       <c r="G28" s="80" t="s">
         <v>272</v>
       </c>
@@ -24712,13 +24718,13 @@
     </row>
     <row r="29" spans="1:8">
       <c r="A29" s="77"/>
-      <c r="B29" s="196" t="s">
+      <c r="B29" s="189" t="s">
         <v>290</v>
       </c>
       <c r="C29" s="79"/>
       <c r="D29" s="79"/>
       <c r="E29" s="79"/>
-      <c r="F29" s="196" t="s">
+      <c r="F29" s="189" t="s">
         <v>289</v>
       </c>
       <c r="G29" s="79"/>
@@ -24728,7 +24734,7 @@
       <c r="A30" s="78">
         <v>4</v>
       </c>
-      <c r="B30" s="198"/>
+      <c r="B30" s="190"/>
       <c r="C30" s="92">
         <v>0.79</v>
       </c>
@@ -24738,7 +24744,7 @@
       <c r="E30" s="92">
         <v>0.95</v>
       </c>
-      <c r="F30" s="198"/>
+      <c r="F30" s="190"/>
       <c r="G30" s="80" t="s">
         <v>272</v>
       </c>
@@ -24812,7 +24818,7 @@
     </row>
     <row r="34" spans="1:8" s="37" customFormat="1">
       <c r="A34" s="98"/>
-      <c r="B34" s="189" t="s">
+      <c r="B34" s="197" t="s">
         <v>300</v>
       </c>
       <c r="C34" s="100" t="s">
@@ -24824,13 +24830,13 @@
       <c r="E34" s="100" t="s">
         <v>301</v>
       </c>
-      <c r="F34" s="189" t="s">
+      <c r="F34" s="197" t="s">
         <v>303</v>
       </c>
-      <c r="G34" s="189" t="s">
+      <c r="G34" s="197" t="s">
         <v>304</v>
       </c>
-      <c r="H34" s="189" t="s">
+      <c r="H34" s="197" t="s">
         <v>305</v>
       </c>
     </row>
@@ -24838,7 +24844,7 @@
       <c r="A35" s="99">
         <v>7</v>
       </c>
-      <c r="B35" s="190"/>
+      <c r="B35" s="198"/>
       <c r="C35" s="101" t="s">
         <v>302</v>
       </c>
@@ -24848,13 +24854,13 @@
       <c r="E35" s="101" t="s">
         <v>302</v>
       </c>
-      <c r="F35" s="190"/>
-      <c r="G35" s="190"/>
-      <c r="H35" s="190"/>
+      <c r="F35" s="198"/>
+      <c r="G35" s="198"/>
+      <c r="H35" s="198"/>
     </row>
     <row r="36" spans="1:8" s="37" customFormat="1">
       <c r="A36" s="98"/>
-      <c r="B36" s="189" t="s">
+      <c r="B36" s="197" t="s">
         <v>306</v>
       </c>
       <c r="C36" s="100" t="s">
@@ -24868,7 +24874,7 @@
       </c>
       <c r="F36" s="103"/>
       <c r="G36" s="103"/>
-      <c r="H36" s="189" t="s">
+      <c r="H36" s="197" t="s">
         <v>305</v>
       </c>
     </row>
@@ -24876,7 +24882,7 @@
       <c r="A37" s="99">
         <v>8</v>
       </c>
-      <c r="B37" s="190"/>
+      <c r="B37" s="198"/>
       <c r="C37" s="101" t="s">
         <v>308</v>
       </c>
@@ -24892,11 +24898,11 @@
       <c r="G37" s="101" t="s">
         <v>304</v>
       </c>
-      <c r="H37" s="190"/>
+      <c r="H37" s="198"/>
     </row>
     <row r="38" spans="1:8" s="37" customFormat="1">
       <c r="A38" s="102"/>
-      <c r="B38" s="191" t="s">
+      <c r="B38" s="205" t="s">
         <v>313</v>
       </c>
       <c r="C38" s="100" t="s">
@@ -24916,7 +24922,7 @@
       <c r="A39" s="104">
         <v>9</v>
       </c>
-      <c r="B39" s="192"/>
+      <c r="B39" s="206"/>
       <c r="C39" s="100" t="s">
         <v>315</v>
       </c>
@@ -24938,7 +24944,7 @@
     </row>
     <row r="40" spans="1:8" s="37" customFormat="1" ht="17" thickBot="1">
       <c r="A40" s="105"/>
-      <c r="B40" s="193"/>
+      <c r="B40" s="207"/>
       <c r="C40" s="101" t="s">
         <v>316</v>
       </c>
@@ -24953,10 +24959,10 @@
       <c r="H40" s="106"/>
     </row>
     <row r="41" spans="1:8">
-      <c r="A41" s="194">
+      <c r="A41" s="203">
         <v>10</v>
       </c>
-      <c r="B41" s="196" t="s">
+      <c r="B41" s="189" t="s">
         <v>321</v>
       </c>
       <c r="C41" s="81" t="s">
@@ -24968,19 +24974,19 @@
       <c r="E41" s="81" t="s">
         <v>326</v>
       </c>
-      <c r="F41" s="196" t="s">
+      <c r="F41" s="189" t="s">
         <v>303</v>
       </c>
-      <c r="G41" s="196" t="s">
+      <c r="G41" s="189" t="s">
         <v>304</v>
       </c>
-      <c r="H41" s="196" t="s">
+      <c r="H41" s="189" t="s">
         <v>305</v>
       </c>
     </row>
     <row r="42" spans="1:8" ht="26">
-      <c r="A42" s="195"/>
-      <c r="B42" s="197"/>
+      <c r="A42" s="204"/>
+      <c r="B42" s="196"/>
       <c r="C42" s="81" t="s">
         <v>323</v>
       </c>
@@ -24990,9 +24996,9 @@
       <c r="E42" s="81" t="s">
         <v>327</v>
       </c>
-      <c r="F42" s="197"/>
-      <c r="G42" s="197"/>
-      <c r="H42" s="197"/>
+      <c r="F42" s="196"/>
+      <c r="G42" s="196"/>
+      <c r="H42" s="196"/>
     </row>
     <row r="43" spans="1:8">
       <c r="A43" s="107">
@@ -25554,22 +25560,32 @@
     </row>
   </sheetData>
   <mergeCells count="52">
-    <mergeCell ref="F6:F7"/>
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="C1:C2"/>
-    <mergeCell ref="E1:E2"/>
-    <mergeCell ref="F4:F5"/>
-    <mergeCell ref="F8:F9"/>
-    <mergeCell ref="B10:H10"/>
-    <mergeCell ref="B11:B12"/>
-    <mergeCell ref="C11:C12"/>
-    <mergeCell ref="D11:D12"/>
-    <mergeCell ref="E11:E12"/>
-    <mergeCell ref="B13:B15"/>
-    <mergeCell ref="B16:B17"/>
-    <mergeCell ref="C16:C17"/>
-    <mergeCell ref="D16:D17"/>
-    <mergeCell ref="E16:E17"/>
+    <mergeCell ref="G34:G35"/>
+    <mergeCell ref="H34:H35"/>
+    <mergeCell ref="B36:B37"/>
+    <mergeCell ref="H36:H37"/>
+    <mergeCell ref="B38:B40"/>
+    <mergeCell ref="A41:A42"/>
+    <mergeCell ref="B41:B42"/>
+    <mergeCell ref="F41:F42"/>
+    <mergeCell ref="G41:G42"/>
+    <mergeCell ref="H41:H42"/>
+    <mergeCell ref="B27:B28"/>
+    <mergeCell ref="F27:F28"/>
+    <mergeCell ref="B29:B30"/>
+    <mergeCell ref="F29:F30"/>
+    <mergeCell ref="B34:B35"/>
+    <mergeCell ref="F34:F35"/>
+    <mergeCell ref="B22:H22"/>
+    <mergeCell ref="B23:B24"/>
+    <mergeCell ref="F23:F24"/>
+    <mergeCell ref="B25:B26"/>
+    <mergeCell ref="C25:C26"/>
+    <mergeCell ref="D25:D26"/>
+    <mergeCell ref="E25:E26"/>
+    <mergeCell ref="F25:F26"/>
+    <mergeCell ref="G25:G26"/>
+    <mergeCell ref="H25:H26"/>
     <mergeCell ref="G16:G17"/>
     <mergeCell ref="H16:H17"/>
     <mergeCell ref="B18:B19"/>
@@ -25580,32 +25596,22 @@
     <mergeCell ref="G18:G19"/>
     <mergeCell ref="H18:H19"/>
     <mergeCell ref="F16:F17"/>
-    <mergeCell ref="B22:H22"/>
-    <mergeCell ref="B23:B24"/>
-    <mergeCell ref="F23:F24"/>
-    <mergeCell ref="B25:B26"/>
-    <mergeCell ref="C25:C26"/>
-    <mergeCell ref="D25:D26"/>
-    <mergeCell ref="E25:E26"/>
-    <mergeCell ref="F25:F26"/>
-    <mergeCell ref="G25:G26"/>
-    <mergeCell ref="H25:H26"/>
-    <mergeCell ref="B27:B28"/>
-    <mergeCell ref="F27:F28"/>
-    <mergeCell ref="B29:B30"/>
-    <mergeCell ref="F29:F30"/>
-    <mergeCell ref="B34:B35"/>
-    <mergeCell ref="F34:F35"/>
-    <mergeCell ref="A41:A42"/>
-    <mergeCell ref="B41:B42"/>
-    <mergeCell ref="F41:F42"/>
-    <mergeCell ref="G41:G42"/>
-    <mergeCell ref="H41:H42"/>
-    <mergeCell ref="G34:G35"/>
-    <mergeCell ref="H34:H35"/>
-    <mergeCell ref="B36:B37"/>
-    <mergeCell ref="H36:H37"/>
-    <mergeCell ref="B38:B40"/>
+    <mergeCell ref="B13:B15"/>
+    <mergeCell ref="B16:B17"/>
+    <mergeCell ref="C16:C17"/>
+    <mergeCell ref="D16:D17"/>
+    <mergeCell ref="E16:E17"/>
+    <mergeCell ref="F8:F9"/>
+    <mergeCell ref="B10:H10"/>
+    <mergeCell ref="B11:B12"/>
+    <mergeCell ref="C11:C12"/>
+    <mergeCell ref="D11:D12"/>
+    <mergeCell ref="E11:E12"/>
+    <mergeCell ref="F6:F7"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="C1:C2"/>
+    <mergeCell ref="E1:E2"/>
+    <mergeCell ref="F4:F5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -25623,6 +25629,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="9ef0ecd9-0ead-4309-8654-c6fc6a0aeea6">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="68eaa246-66f5-4d4b-bc2d-4cd6ec79d795" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100714250AEEB2AC4409DE69A29E07D1293" ma:contentTypeVersion="12" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="2c479027f39f79bf5fe77e0c13ff8fe0">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="9ef0ecd9-0ead-4309-8654-c6fc6a0aeea6" xmlns:ns3="68eaa246-66f5-4d4b-bc2d-4cd6ec79d795" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0ac27669cc00f86f1897f89f498d9d9b" ns2:_="" ns3:_="">
     <xsd:import namespace="9ef0ecd9-0ead-4309-8654-c6fc6a0aeea6"/>
@@ -25825,27 +25851,32 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{317F62B1-8FBE-489E-AF5B-00C050AC7470}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="9ef0ecd9-0ead-4309-8654-c6fc6a0aeea6"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="68eaa246-66f5-4d4b-bc2d-4cd6ec79d795"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="9ef0ecd9-0ead-4309-8654-c6fc6a0aeea6">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="68eaa246-66f5-4d4b-bc2d-4cd6ec79d795" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{83D1394D-06CD-4C52-A98B-8D3C2B511CE9}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CA56E987-09E7-4B23-987F-390DA95286EF}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -25862,29 +25893,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{83D1394D-06CD-4C52-A98B-8D3C2B511CE9}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{317F62B1-8FBE-489E-AF5B-00C050AC7470}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="68eaa246-66f5-4d4b-bc2d-4cd6ec79d795"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="9ef0ecd9-0ead-4309-8654-c6fc6a0aeea6"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Adding the CrI of data used for DR recalibration
- Data used for DR recalibration were in the graphs with their uncertainty around the points
</commit_message>
<xml_diff>
--- a/data/All_clinics_data.xlsx
+++ b/data/All_clinics_data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10713"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10817"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://unsw-my.sharepoint.com/personal/z5288872_ad_unsw_edu_au/Documents/Modelling HIV [Quang]/PNG-Transmission-Model/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1706" documentId="13_ncr:1_{B01AED12-C7E5-C04A-9CE5-A2F269A7A508}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{632C31A9-A870-CA40-92BB-35D4F8CAFFCB}"/>
+  <xr:revisionPtr revIDLastSave="1711" documentId="13_ncr:1_{B01AED12-C7E5-C04A-9CE5-A2F269A7A508}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EA2D54C7-ACB6-5444-8458-37788F16ED54}"/>
   <bookViews>
-    <workbookView xWindow="-32400" yWindow="500" windowWidth="30220" windowHeight="21100" activeTab="1" xr2:uid="{2E625105-1FFC-624E-9A6F-F385E9B192AB}"/>
+    <workbookView xWindow="-35520" yWindow="500" windowWidth="30220" windowHeight="21100" activeTab="4" xr2:uid="{2E625105-1FFC-624E-9A6F-F385E9B192AB}"/>
   </bookViews>
   <sheets>
     <sheet name="(Hidden) Estimates" sheetId="2" state="hidden" r:id="rId1"/>
@@ -566,6 +566,19 @@
     <author>tc={63BCE664-920C-4105-A504-661B565134AC}</author>
     <author>tc={FF276D0F-D862-4FF6-89AB-F438D91D0B8D}</author>
     <author>tc={AC12B5DC-EFA5-4F50-997B-C5B23BA197C9}</author>
+    <author>tc={4DC48738-F485-DB4B-B83C-EF5CDCA1CFE5}</author>
+    <author>tc={4495969F-67C0-5A43-B6C4-B096D7617834}</author>
+    <author>tc={B7DB655E-57BA-F84D-9095-BFA40D56F2DA}</author>
+    <author>tc={82A9A190-579D-7647-AE62-F0EF2EE0EAC8}</author>
+    <author>tc={842B4E81-A8C2-9141-A850-E27C575B1BDD}</author>
+    <author>tc={5C3CD516-F572-9F4D-9D3A-33C1A4EF1D63}</author>
+    <author>tc={D1E6B6E1-8390-9542-A5BE-C3D691472392}</author>
+    <author>tc={483DF72C-630B-224A-8C91-F3449694FB33}</author>
+    <author>tc={DF9D3516-F1FB-A44D-972A-A9696A2C4491}</author>
+    <author>tc={DC0C8AD1-6E1A-714E-841E-44C7FE3CBE3C}</author>
+    <author>tc={8CFF051A-8773-B542-9A29-B56DA0003DFE}</author>
+    <author>tc={9AA9C820-4780-E14A-929A-A4E5139059E3}</author>
+    <author>tc={76C901CC-D9D7-EF45-9A0D-94106F74102F}</author>
   </authors>
   <commentList>
     <comment ref="AB1" authorId="0" shapeId="0" xr:uid="{D6060EDE-255E-4CEA-93CC-9BC87BD3A694}">
@@ -888,6 +901,120 @@
 </t>
       </text>
     </comment>
+    <comment ref="X49" authorId="37" shapeId="0" xr:uid="{4DC48738-F485-DB4B-B83C-EF5CDCA1CFE5}">
+      <text>
+        <t xml:space="preserve">[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Gare, J., Ryan, C. E., David, M., Timbi, D., Kaima, P., Kombati, Z., . . . Hearps, A. C. (2014). Presence of HIV drug resistance in antiretroviral therapy-naive and -experienced patients from Papua New Guinea. Journal of Antimicrobial Chemotherapy, 69(8), 2183-2186. doi:10.1093/jac/dku089
+</t>
+      </text>
+    </comment>
+    <comment ref="AA49" authorId="38" shapeId="0" xr:uid="{4495969F-67C0-5A43-B6C4-B096D7617834}">
+      <text>
+        <t xml:space="preserve">[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Lavu, E., Kave, E., Mosoro, E., Markby, J., Aleksic, E., Gare, J., . . . Jordan, M. R. (2017). High levels of transmitted HIV drug resistance in a study in Papua New Guinea. PLoS ONE, 12(2). doi:10.1371/journal.pone.0170265
+</t>
+      </text>
+    </comment>
+    <comment ref="AB49" authorId="39" shapeId="0" xr:uid="{B7DB655E-57BA-F84D-9095-BFA40D56F2DA}">
+      <text>
+        <t xml:space="preserve">[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Lavu, E., Kave, E., Mosoro, E., Markby, J., Aleksic, E., Gare, J., . . . Jordan, M. R. (2017). High levels of transmitted HIV drug resistance in a study in Papua New Guinea. PLoS ONE, 12(2). doi:10.1371/journal.pone.0170265
+</t>
+      </text>
+    </comment>
+    <comment ref="AE49" authorId="40" shapeId="0" xr:uid="{82A9A190-579D-7647-AE62-F0EF2EE0EAC8}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Gare, J., et al. (2022). "High prevalence of pre-treatment HIV drug resistance in Papua New Guinea: findings from the first nationally representative pre-treatment HIV drug resistance study." BMC Infect Dis 22(1): 266.</t>
+      </text>
+    </comment>
+    <comment ref="AJ49" authorId="41" shapeId="0" xr:uid="{842B4E81-A8C2-9141-A850-E27C575B1BDD}">
+      <text>
+        <t xml:space="preserve">[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Gillian Scott- emails communication June 14th 
+</t>
+      </text>
+    </comment>
+    <comment ref="AA50" authorId="42" shapeId="0" xr:uid="{5C3CD516-F572-9F4D-9D3A-33C1A4EF1D63}">
+      <text>
+        <t xml:space="preserve">[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Lavu, E., Kave, E., Mosoro, E., Markby, J., Aleksic, E., Gare, J., . . . Jordan, M. R. (2017). High levels of transmitted HIV drug resistance in a study in Papua New Guinea. PLoS ONE, 12(2). doi:10.1371/journal.pone.0170265
+</t>
+      </text>
+    </comment>
+    <comment ref="AB50" authorId="43" shapeId="0" xr:uid="{D1E6B6E1-8390-9542-A5BE-C3D691472392}">
+      <text>
+        <t xml:space="preserve">[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Lavu, E., Kave, E., Mosoro, E., Markby, J., Aleksic, E., Gare, J., . . . Jordan, M. R. (2017). High levels of transmitted HIV drug resistance in a study in Papua New Guinea. PLoS ONE, 12(2). doi:10.1371/journal.pone.0170265
+</t>
+      </text>
+    </comment>
+    <comment ref="AE50" authorId="44" shapeId="0" xr:uid="{483DF72C-630B-224A-8C91-F3449694FB33}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Gare, J., et al. (2022). "High prevalence of pre-treatment HIV drug resistance in Papua New Guinea: findings from the first nationally representative pre-treatment HIV drug resistance study." BMC Infect Dis 22(1): 266.</t>
+      </text>
+    </comment>
+    <comment ref="AJ50" authorId="45" shapeId="0" xr:uid="{DF9D3516-F1FB-A44D-972A-A9696A2C4491}">
+      <text>
+        <t xml:space="preserve">[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Gillian Scott- emails communication June 14th 
+</t>
+      </text>
+    </comment>
+    <comment ref="AA51" authorId="46" shapeId="0" xr:uid="{DC0C8AD1-6E1A-714E-841E-44C7FE3CBE3C}">
+      <text>
+        <t xml:space="preserve">[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Lavu, E., Kave, E., Mosoro, E., Markby, J., Aleksic, E., Gare, J., . . . Jordan, M. R. (2017). High levels of transmitted HIV drug resistance in a study in Papua New Guinea. PLoS ONE, 12(2). doi:10.1371/journal.pone.0170265
+</t>
+      </text>
+    </comment>
+    <comment ref="AB51" authorId="47" shapeId="0" xr:uid="{8CFF051A-8773-B542-9A29-B56DA0003DFE}">
+      <text>
+        <t xml:space="preserve">[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Lavu, E., Kave, E., Mosoro, E., Markby, J., Aleksic, E., Gare, J., . . . Jordan, M. R. (2017). High levels of transmitted HIV drug resistance in a study in Papua New Guinea. PLoS ONE, 12(2). doi:10.1371/journal.pone.0170265
+</t>
+      </text>
+    </comment>
+    <comment ref="AE51" authorId="48" shapeId="0" xr:uid="{9AA9C820-4780-E14A-929A-A4E5139059E3}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Gare, J., et al. (2022). "High prevalence of pre-treatment HIV drug resistance in Papua New Guinea: findings from the first nationally representative pre-treatment HIV drug resistance study." BMC Infect Dis 22(1): 266.</t>
+      </text>
+    </comment>
+    <comment ref="AJ51" authorId="49" shapeId="0" xr:uid="{76C901CC-D9D7-EF45-9A0D-94106F74102F}">
+      <text>
+        <t xml:space="preserve">[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Gillian Scott- emails communication June 14th 
+</t>
+      </text>
+    </comment>
   </commentList>
 </comments>
 </file>
@@ -911,7 +1038,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2812" uniqueCount="427">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2817" uniqueCount="428">
   <si>
     <t>HIV estimates with uncertainty bounds</t>
   </si>
@@ -2211,6 +2338,9 @@
   <si>
     <t>9.03 [7.41 - 11.19]</t>
   </si>
+  <si>
+    <t xml:space="preserve">Overall prevalence of PDR amongst those who are ART naïve (%) -depraciated </t>
+  </si>
 </sst>
 </file>
 
@@ -2219,7 +2349,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="28">
+  <fonts count="29">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -2405,6 +2535,12 @@
       <color theme="1"/>
       <name val="Times New Roman"/>
       <family val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="13">
@@ -3353,17 +3489,14 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
@@ -3371,7 +3504,22 @@
     <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="2" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="2" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="49" fontId="5" fillId="3" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="2" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="5" fillId="2" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -3383,12 +3531,6 @@
     <xf numFmtId="49" fontId="5" fillId="2" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="5" fillId="3" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="3" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="49" fontId="5" fillId="3" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
@@ -3396,18 +3538,6 @@
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="5" fillId="3" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="2" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="2" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="2" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="5" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -3419,40 +3549,43 @@
     <xf numFmtId="49" fontId="5" fillId="3" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="5" fillId="3" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="5" fillId="3" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="37" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="10" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="5" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="37" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="10" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="39" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="5" fillId="0" borderId="38" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="5" fillId="0" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="39" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="5" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -3462,6 +3595,9 @@
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="5" fillId="0" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="5" fillId="0" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -3500,16 +3636,34 @@
     <xf numFmtId="0" fontId="12" fillId="5" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="25" fillId="4" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="4" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="4" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="4" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="4" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="9" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="9" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="25" fillId="9" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="9" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="25" fillId="9" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="7" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="7" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="25" fillId="9" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="8" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -3521,13 +3675,10 @@
     <xf numFmtId="0" fontId="22" fillId="8" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="9" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="25" fillId="4" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="4" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="4" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="25" fillId="4" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="9" fontId="25" fillId="4" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -3536,26 +3687,11 @@
     <xf numFmtId="9" fontId="25" fillId="4" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="25" fillId="4" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="7" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="25" fillId="4" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="7" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="9" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="9" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="4" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="4" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="4" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -4310,6 +4446,55 @@
     <text xml:space="preserve">Gillian Scott- emails communication June 14th 
 </text>
   </threadedComment>
+  <threadedComment ref="X49" dT="2023-05-16T04:57:30.14" personId="{ADA2A9C4-E859-804B-89A0-69D598442343}" id="{4DC48738-F485-DB4B-B83C-EF5CDCA1CFE5}">
+    <text xml:space="preserve">Gare, J., Ryan, C. E., David, M., Timbi, D., Kaima, P., Kombati, Z., . . . Hearps, A. C. (2014). Presence of HIV drug resistance in antiretroviral therapy-naive and -experienced patients from Papua New Guinea. Journal of Antimicrobial Chemotherapy, 69(8), 2183-2186. doi:10.1093/jac/dku089
+</text>
+  </threadedComment>
+  <threadedComment ref="AA49" dT="2023-05-16T04:54:40.02" personId="{ADA2A9C4-E859-804B-89A0-69D598442343}" id="{4495969F-67C0-5A43-B6C4-B096D7617834}">
+    <text xml:space="preserve">Lavu, E., Kave, E., Mosoro, E., Markby, J., Aleksic, E., Gare, J., . . . Jordan, M. R. (2017). High levels of transmitted HIV drug resistance in a study in Papua New Guinea. PLoS ONE, 12(2). doi:10.1371/journal.pone.0170265
+</text>
+  </threadedComment>
+  <threadedComment ref="AB49" dT="2023-05-16T04:55:31.18" personId="{ADA2A9C4-E859-804B-89A0-69D598442343}" id="{B7DB655E-57BA-F84D-9095-BFA40D56F2DA}">
+    <text xml:space="preserve">Lavu, E., Kave, E., Mosoro, E., Markby, J., Aleksic, E., Gare, J., . . . Jordan, M. R. (2017). High levels of transmitted HIV drug resistance in a study in Papua New Guinea. PLoS ONE, 12(2). doi:10.1371/journal.pone.0170265
+</text>
+  </threadedComment>
+  <threadedComment ref="AE49" dT="2022-04-20T07:44:41.89" personId="{F7AE736D-4AAE-4F5E-8C98-4CA249D52645}" id="{82A9A190-579D-7647-AE62-F0EF2EE0EAC8}">
+    <text>Gare, J., et al. (2022). "High prevalence of pre-treatment HIV drug resistance in Papua New Guinea: findings from the first nationally representative pre-treatment HIV drug resistance study." BMC Infect Dis 22(1): 266.</text>
+  </threadedComment>
+  <threadedComment ref="AJ49" dT="2023-06-15T01:18:51.22" personId="{ADA2A9C4-E859-804B-89A0-69D598442343}" id="{842B4E81-A8C2-9141-A850-E27C575B1BDD}">
+    <text xml:space="preserve">Gillian Scott- emails communication June 14th 
+</text>
+  </threadedComment>
+  <threadedComment ref="AA50" dT="2023-05-16T04:54:49.66" personId="{ADA2A9C4-E859-804B-89A0-69D598442343}" id="{5C3CD516-F572-9F4D-9D3A-33C1A4EF1D63}">
+    <text xml:space="preserve">Lavu, E., Kave, E., Mosoro, E., Markby, J., Aleksic, E., Gare, J., . . . Jordan, M. R. (2017). High levels of transmitted HIV drug resistance in a study in Papua New Guinea. PLoS ONE, 12(2). doi:10.1371/journal.pone.0170265
+</text>
+  </threadedComment>
+  <threadedComment ref="AB50" dT="2023-05-16T04:55:36.01" personId="{ADA2A9C4-E859-804B-89A0-69D598442343}" id="{D1E6B6E1-8390-9542-A5BE-C3D691472392}">
+    <text xml:space="preserve">Lavu, E., Kave, E., Mosoro, E., Markby, J., Aleksic, E., Gare, J., . . . Jordan, M. R. (2017). High levels of transmitted HIV drug resistance in a study in Papua New Guinea. PLoS ONE, 12(2). doi:10.1371/journal.pone.0170265
+</text>
+  </threadedComment>
+  <threadedComment ref="AE50" dT="2022-04-20T07:44:45.62" personId="{F7AE736D-4AAE-4F5E-8C98-4CA249D52645}" id="{483DF72C-630B-224A-8C91-F3449694FB33}">
+    <text>Gare, J., et al. (2022). "High prevalence of pre-treatment HIV drug resistance in Papua New Guinea: findings from the first nationally representative pre-treatment HIV drug resistance study." BMC Infect Dis 22(1): 266.</text>
+  </threadedComment>
+  <threadedComment ref="AJ50" dT="2023-06-15T01:19:36.91" personId="{ADA2A9C4-E859-804B-89A0-69D598442343}" id="{DF9D3516-F1FB-A44D-972A-A9696A2C4491}">
+    <text xml:space="preserve">Gillian Scott- emails communication June 14th 
+</text>
+  </threadedComment>
+  <threadedComment ref="AA51" dT="2023-05-16T04:55:25.71" personId="{ADA2A9C4-E859-804B-89A0-69D598442343}" id="{DC0C8AD1-6E1A-714E-841E-44C7FE3CBE3C}">
+    <text xml:space="preserve">Lavu, E., Kave, E., Mosoro, E., Markby, J., Aleksic, E., Gare, J., . . . Jordan, M. R. (2017). High levels of transmitted HIV drug resistance in a study in Papua New Guinea. PLoS ONE, 12(2). doi:10.1371/journal.pone.0170265
+</text>
+  </threadedComment>
+  <threadedComment ref="AB51" dT="2023-05-16T04:55:42.12" personId="{ADA2A9C4-E859-804B-89A0-69D598442343}" id="{8CFF051A-8773-B542-9A29-B56DA0003DFE}">
+    <text xml:space="preserve">Lavu, E., Kave, E., Mosoro, E., Markby, J., Aleksic, E., Gare, J., . . . Jordan, M. R. (2017). High levels of transmitted HIV drug resistance in a study in Papua New Guinea. PLoS ONE, 12(2). doi:10.1371/journal.pone.0170265
+</text>
+  </threadedComment>
+  <threadedComment ref="AE51" dT="2022-04-20T07:44:48.76" personId="{F7AE736D-4AAE-4F5E-8C98-4CA249D52645}" id="{9AA9C820-4780-E14A-929A-A4E5139059E3}">
+    <text>Gare, J., et al. (2022). "High prevalence of pre-treatment HIV drug resistance in Papua New Guinea: findings from the first nationally representative pre-treatment HIV drug resistance study." BMC Infect Dis 22(1): 266.</text>
+  </threadedComment>
+  <threadedComment ref="AJ51" dT="2023-06-15T01:19:41.15" personId="{ADA2A9C4-E859-804B-89A0-69D598442343}" id="{76C901CC-D9D7-EF45-9A0D-94106F74102F}">
+    <text xml:space="preserve">Gillian Scott- emails communication June 14th 
+</text>
+  </threadedComment>
 </ThreadedComments>
 </file>
 
@@ -4467,86 +4652,86 @@
       <c r="AY4" s="23"/>
     </row>
     <row r="5" spans="1:54" s="7" customFormat="1" ht="39.5" customHeight="1">
-      <c r="D5" s="141" t="s">
+      <c r="D5" s="140" t="s">
         <v>27</v>
       </c>
-      <c r="E5" s="141"/>
-      <c r="F5" s="141"/>
-      <c r="G5" s="140" t="s">
+      <c r="E5" s="140"/>
+      <c r="F5" s="140"/>
+      <c r="G5" s="141" t="s">
         <v>28</v>
       </c>
-      <c r="H5" s="140"/>
-      <c r="I5" s="140"/>
-      <c r="J5" s="141" t="s">
+      <c r="H5" s="141"/>
+      <c r="I5" s="141"/>
+      <c r="J5" s="140" t="s">
         <v>29</v>
       </c>
-      <c r="K5" s="141"/>
-      <c r="L5" s="141"/>
-      <c r="M5" s="140" t="s">
+      <c r="K5" s="140"/>
+      <c r="L5" s="140"/>
+      <c r="M5" s="141" t="s">
         <v>30</v>
       </c>
-      <c r="N5" s="140"/>
-      <c r="O5" s="140"/>
-      <c r="P5" s="141" t="s">
+      <c r="N5" s="141"/>
+      <c r="O5" s="141"/>
+      <c r="P5" s="140" t="s">
         <v>31</v>
       </c>
-      <c r="Q5" s="141"/>
-      <c r="R5" s="141"/>
-      <c r="S5" s="140" t="s">
+      <c r="Q5" s="140"/>
+      <c r="R5" s="140"/>
+      <c r="S5" s="141" t="s">
         <v>32</v>
       </c>
-      <c r="T5" s="140"/>
-      <c r="U5" s="140"/>
-      <c r="V5" s="141" t="s">
+      <c r="T5" s="141"/>
+      <c r="U5" s="141"/>
+      <c r="V5" s="140" t="s">
         <v>33</v>
       </c>
-      <c r="W5" s="141"/>
-      <c r="X5" s="141"/>
-      <c r="Y5" s="140" t="s">
+      <c r="W5" s="140"/>
+      <c r="X5" s="140"/>
+      <c r="Y5" s="141" t="s">
         <v>34</v>
       </c>
-      <c r="Z5" s="140"/>
-      <c r="AA5" s="140"/>
-      <c r="AB5" s="141" t="s">
+      <c r="Z5" s="141"/>
+      <c r="AA5" s="141"/>
+      <c r="AB5" s="140" t="s">
         <v>35</v>
       </c>
-      <c r="AC5" s="141"/>
-      <c r="AD5" s="141"/>
-      <c r="AE5" s="140" t="s">
+      <c r="AC5" s="140"/>
+      <c r="AD5" s="140"/>
+      <c r="AE5" s="141" t="s">
         <v>36</v>
       </c>
-      <c r="AF5" s="140"/>
-      <c r="AG5" s="140"/>
-      <c r="AH5" s="141" t="s">
+      <c r="AF5" s="141"/>
+      <c r="AG5" s="141"/>
+      <c r="AH5" s="140" t="s">
         <v>37</v>
       </c>
-      <c r="AI5" s="141"/>
-      <c r="AJ5" s="141"/>
-      <c r="AK5" s="140" t="s">
+      <c r="AI5" s="140"/>
+      <c r="AJ5" s="140"/>
+      <c r="AK5" s="141" t="s">
         <v>38</v>
       </c>
-      <c r="AL5" s="140"/>
-      <c r="AM5" s="140"/>
-      <c r="AN5" s="141" t="s">
+      <c r="AL5" s="141"/>
+      <c r="AM5" s="141"/>
+      <c r="AN5" s="140" t="s">
         <v>11</v>
       </c>
-      <c r="AO5" s="141"/>
-      <c r="AP5" s="141"/>
-      <c r="AQ5" s="140" t="s">
+      <c r="AO5" s="140"/>
+      <c r="AP5" s="140"/>
+      <c r="AQ5" s="141" t="s">
         <v>39</v>
       </c>
-      <c r="AR5" s="140"/>
-      <c r="AS5" s="140"/>
-      <c r="AT5" s="141" t="s">
+      <c r="AR5" s="141"/>
+      <c r="AS5" s="141"/>
+      <c r="AT5" s="140" t="s">
         <v>40</v>
       </c>
-      <c r="AU5" s="141"/>
-      <c r="AV5" s="141"/>
-      <c r="AW5" s="140" t="s">
+      <c r="AU5" s="140"/>
+      <c r="AV5" s="140"/>
+      <c r="AW5" s="141" t="s">
         <v>41</v>
       </c>
-      <c r="AX5" s="140"/>
-      <c r="AY5" s="140"/>
+      <c r="AX5" s="141"/>
+      <c r="AY5" s="141"/>
       <c r="AZ5" s="142" t="s">
         <v>99</v>
       </c>
@@ -9515,11 +9700,6 @@
     </row>
   </sheetData>
   <mergeCells count="17">
-    <mergeCell ref="D5:F5"/>
-    <mergeCell ref="G5:I5"/>
-    <mergeCell ref="J5:L5"/>
-    <mergeCell ref="M5:O5"/>
-    <mergeCell ref="P5:R5"/>
     <mergeCell ref="AE5:AG5"/>
     <mergeCell ref="AH5:AJ5"/>
     <mergeCell ref="AK5:AM5"/>
@@ -9532,6 +9712,11 @@
     <mergeCell ref="V5:X5"/>
     <mergeCell ref="Y5:AA5"/>
     <mergeCell ref="AB5:AD5"/>
+    <mergeCell ref="D5:F5"/>
+    <mergeCell ref="G5:I5"/>
+    <mergeCell ref="J5:L5"/>
+    <mergeCell ref="M5:O5"/>
+    <mergeCell ref="P5:R5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -10263,7 +10448,7 @@
       <c r="AG13" s="29"/>
     </row>
     <row r="14" spans="1:37" s="37" customFormat="1" ht="17" customHeight="1">
-      <c r="A14" s="145" t="s">
+      <c r="A14" s="144" t="s">
         <v>376</v>
       </c>
       <c r="B14" s="130" t="s">
@@ -10304,7 +10489,7 @@
       <c r="AG14" s="72"/>
     </row>
     <row r="15" spans="1:37" s="37" customFormat="1" ht="17" customHeight="1">
-      <c r="A15" s="145"/>
+      <c r="A15" s="144"/>
       <c r="B15" s="130" t="s">
         <v>391</v>
       </c>
@@ -10413,7 +10598,7 @@
       <c r="B18" s="136"/>
     </row>
     <row r="19" spans="1:33">
-      <c r="A19" s="143"/>
+      <c r="A19" s="145"/>
       <c r="B19" s="45"/>
       <c r="C19" s="29"/>
       <c r="D19" s="29"/>
@@ -10448,7 +10633,7 @@
       <c r="AG19" s="29"/>
     </row>
     <row r="20" spans="1:33">
-      <c r="A20" s="143"/>
+      <c r="A20" s="145"/>
       <c r="B20" s="46"/>
       <c r="C20" s="30"/>
       <c r="D20" s="30"/>
@@ -10483,7 +10668,7 @@
       <c r="AG20" s="30"/>
     </row>
     <row r="21" spans="1:33">
-      <c r="A21" s="143"/>
+      <c r="A21" s="145"/>
       <c r="B21" s="46"/>
       <c r="C21" s="30"/>
       <c r="D21" s="30"/>
@@ -10518,7 +10703,7 @@
       <c r="AG21" s="30"/>
     </row>
     <row r="22" spans="1:33">
-      <c r="A22" s="143"/>
+      <c r="A22" s="145"/>
       <c r="B22" s="45"/>
       <c r="C22" s="29"/>
       <c r="D22" s="29"/>
@@ -10553,7 +10738,7 @@
       <c r="AG22" s="29"/>
     </row>
     <row r="23" spans="1:33">
-      <c r="A23" s="143"/>
+      <c r="A23" s="145"/>
       <c r="B23" s="46"/>
       <c r="C23" s="30"/>
       <c r="D23" s="30"/>
@@ -10588,7 +10773,7 @@
       <c r="AG23" s="30"/>
     </row>
     <row r="24" spans="1:33">
-      <c r="A24" s="143"/>
+      <c r="A24" s="145"/>
       <c r="B24" s="46"/>
       <c r="C24" s="30"/>
       <c r="D24" s="30"/>
@@ -10623,7 +10808,7 @@
       <c r="AG24" s="30"/>
     </row>
     <row r="25" spans="1:33">
-      <c r="A25" s="143"/>
+      <c r="A25" s="145"/>
       <c r="B25" s="45"/>
       <c r="C25" s="29"/>
       <c r="D25" s="29"/>
@@ -10658,7 +10843,7 @@
       <c r="AG25" s="29"/>
     </row>
     <row r="26" spans="1:33">
-      <c r="A26" s="143"/>
+      <c r="A26" s="145"/>
       <c r="B26" s="46"/>
       <c r="C26" s="30"/>
       <c r="D26" s="30"/>
@@ -10693,7 +10878,7 @@
       <c r="AG26" s="30"/>
     </row>
     <row r="27" spans="1:33">
-      <c r="A27" s="143"/>
+      <c r="A27" s="145"/>
       <c r="B27" s="46"/>
       <c r="C27" s="30"/>
       <c r="D27" s="30"/>
@@ -10798,7 +10983,7 @@
       <c r="AG29" s="30"/>
     </row>
     <row r="30" spans="1:33">
-      <c r="A30" s="143"/>
+      <c r="A30" s="145"/>
       <c r="B30" s="45"/>
       <c r="C30" s="29"/>
       <c r="D30" s="29"/>
@@ -10833,7 +11018,7 @@
       <c r="AG30" s="29"/>
     </row>
     <row r="31" spans="1:33">
-      <c r="A31" s="143"/>
+      <c r="A31" s="145"/>
       <c r="B31" s="46"/>
       <c r="C31" s="30"/>
       <c r="D31" s="30"/>
@@ -10868,7 +11053,7 @@
       <c r="AG31" s="30"/>
     </row>
     <row r="32" spans="1:33">
-      <c r="A32" s="143"/>
+      <c r="A32" s="145"/>
       <c r="B32" s="46"/>
       <c r="C32" s="30"/>
       <c r="D32" s="30"/>
@@ -10903,7 +11088,7 @@
       <c r="AG32" s="30"/>
     </row>
     <row r="33" spans="1:33">
-      <c r="A33" s="143"/>
+      <c r="A33" s="145"/>
       <c r="B33" s="45"/>
       <c r="C33" s="29"/>
       <c r="D33" s="29"/>
@@ -10938,7 +11123,7 @@
       <c r="AG33" s="29"/>
     </row>
     <row r="34" spans="1:33">
-      <c r="A34" s="143"/>
+      <c r="A34" s="145"/>
       <c r="B34" s="46"/>
       <c r="C34" s="30"/>
       <c r="D34" s="30"/>
@@ -10973,7 +11158,7 @@
       <c r="AG34" s="30"/>
     </row>
     <row r="35" spans="1:33">
-      <c r="A35" s="143"/>
+      <c r="A35" s="145"/>
       <c r="B35" s="46"/>
       <c r="C35" s="30"/>
       <c r="D35" s="30"/>
@@ -11008,7 +11193,7 @@
       <c r="AG35" s="30"/>
     </row>
     <row r="36" spans="1:33">
-      <c r="A36" s="143"/>
+      <c r="A36" s="145"/>
       <c r="B36" s="45"/>
       <c r="C36" s="29"/>
       <c r="D36" s="29"/>
@@ -11043,7 +11228,7 @@
       <c r="AG36" s="29"/>
     </row>
     <row r="37" spans="1:33">
-      <c r="A37" s="143"/>
+      <c r="A37" s="145"/>
       <c r="B37" s="46"/>
       <c r="C37" s="30"/>
       <c r="D37" s="30"/>
@@ -11078,7 +11263,7 @@
       <c r="AG37" s="30"/>
     </row>
     <row r="38" spans="1:33">
-      <c r="A38" s="143"/>
+      <c r="A38" s="145"/>
       <c r="B38" s="46"/>
       <c r="C38" s="30"/>
       <c r="D38" s="30"/>
@@ -11218,7 +11403,7 @@
       <c r="AG41" s="30"/>
     </row>
     <row r="42" spans="1:33">
-      <c r="A42" s="143"/>
+      <c r="A42" s="145"/>
       <c r="B42" s="45"/>
       <c r="C42" s="29"/>
       <c r="D42" s="29"/>
@@ -11253,7 +11438,7 @@
       <c r="AG42" s="29"/>
     </row>
     <row r="43" spans="1:33">
-      <c r="A43" s="143"/>
+      <c r="A43" s="145"/>
       <c r="B43" s="46"/>
       <c r="C43" s="30"/>
       <c r="D43" s="30"/>
@@ -11288,7 +11473,7 @@
       <c r="AG43" s="30"/>
     </row>
     <row r="44" spans="1:33">
-      <c r="A44" s="143"/>
+      <c r="A44" s="145"/>
       <c r="B44" s="46"/>
       <c r="C44" s="30"/>
       <c r="D44" s="30"/>
@@ -11323,7 +11508,7 @@
       <c r="AG44" s="30"/>
     </row>
     <row r="45" spans="1:33">
-      <c r="A45" s="143"/>
+      <c r="A45" s="145"/>
       <c r="B45" s="45"/>
       <c r="C45" s="29"/>
       <c r="D45" s="29"/>
@@ -11358,7 +11543,7 @@
       <c r="AG45" s="29"/>
     </row>
     <row r="46" spans="1:33">
-      <c r="A46" s="143"/>
+      <c r="A46" s="145"/>
       <c r="B46" s="46"/>
       <c r="C46" s="30"/>
       <c r="D46" s="30"/>
@@ -11393,7 +11578,7 @@
       <c r="AG46" s="30"/>
     </row>
     <row r="47" spans="1:33">
-      <c r="A47" s="143"/>
+      <c r="A47" s="145"/>
       <c r="B47" s="46"/>
       <c r="C47" s="30"/>
       <c r="D47" s="30"/>
@@ -11428,7 +11613,7 @@
       <c r="AG47" s="30"/>
     </row>
     <row r="48" spans="1:33">
-      <c r="A48" s="143"/>
+      <c r="A48" s="145"/>
       <c r="B48" s="45"/>
       <c r="C48" s="29"/>
       <c r="D48" s="29"/>
@@ -11463,7 +11648,7 @@
       <c r="AG48" s="29"/>
     </row>
     <row r="49" spans="1:33">
-      <c r="A49" s="143"/>
+      <c r="A49" s="145"/>
       <c r="B49" s="46"/>
       <c r="C49" s="30"/>
       <c r="D49" s="30"/>
@@ -11498,7 +11683,7 @@
       <c r="AG49" s="30"/>
     </row>
     <row r="50" spans="1:33">
-      <c r="A50" s="143"/>
+      <c r="A50" s="145"/>
       <c r="B50" s="46"/>
       <c r="C50" s="30"/>
       <c r="D50" s="30"/>
@@ -11638,7 +11823,7 @@
       <c r="AG53" s="51"/>
     </row>
     <row r="54" spans="1:33">
-      <c r="A54" s="143"/>
+      <c r="A54" s="145"/>
       <c r="B54" s="45"/>
       <c r="C54" s="29"/>
       <c r="D54" s="29"/>
@@ -11673,7 +11858,7 @@
       <c r="AG54" s="29"/>
     </row>
     <row r="55" spans="1:33">
-      <c r="A55" s="143"/>
+      <c r="A55" s="145"/>
       <c r="B55" s="46"/>
       <c r="C55" s="30"/>
       <c r="D55" s="30"/>
@@ -11708,7 +11893,7 @@
       <c r="AG55" s="30"/>
     </row>
     <row r="56" spans="1:33">
-      <c r="A56" s="143"/>
+      <c r="A56" s="145"/>
       <c r="B56" s="46"/>
       <c r="C56" s="30"/>
       <c r="D56" s="30"/>
@@ -11778,7 +11963,7 @@
       <c r="AG57" s="30"/>
     </row>
     <row r="58" spans="1:33">
-      <c r="A58" s="143"/>
+      <c r="A58" s="145"/>
       <c r="B58" s="45"/>
       <c r="C58" s="29"/>
       <c r="D58" s="29"/>
@@ -11813,7 +11998,7 @@
       <c r="AG58" s="29"/>
     </row>
     <row r="59" spans="1:33">
-      <c r="A59" s="143"/>
+      <c r="A59" s="145"/>
       <c r="B59" s="46"/>
       <c r="C59" s="30"/>
       <c r="D59" s="30"/>
@@ -11848,7 +12033,7 @@
       <c r="AG59" s="30"/>
     </row>
     <row r="60" spans="1:33">
-      <c r="A60" s="143"/>
+      <c r="A60" s="145"/>
       <c r="B60" s="46"/>
       <c r="C60" s="30"/>
       <c r="D60" s="30"/>
@@ -11883,7 +12068,7 @@
       <c r="AG60" s="30"/>
     </row>
     <row r="61" spans="1:33">
-      <c r="A61" s="143"/>
+      <c r="A61" s="145"/>
       <c r="B61" s="45"/>
       <c r="C61" s="29"/>
       <c r="D61" s="29"/>
@@ -11918,7 +12103,7 @@
       <c r="AG61" s="29"/>
     </row>
     <row r="62" spans="1:33">
-      <c r="A62" s="143"/>
+      <c r="A62" s="145"/>
       <c r="B62" s="46"/>
       <c r="C62" s="30"/>
       <c r="D62" s="30"/>
@@ -11953,7 +12138,7 @@
       <c r="AG62" s="30"/>
     </row>
     <row r="63" spans="1:33">
-      <c r="A63" s="143"/>
+      <c r="A63" s="145"/>
       <c r="B63" s="46"/>
       <c r="C63" s="30"/>
       <c r="D63" s="30"/>
@@ -11988,7 +12173,7 @@
       <c r="AG63" s="30"/>
     </row>
     <row r="64" spans="1:33">
-      <c r="A64" s="143"/>
+      <c r="A64" s="145"/>
       <c r="B64" s="45"/>
       <c r="C64" s="29"/>
       <c r="D64" s="29"/>
@@ -12023,7 +12208,7 @@
       <c r="AG64" s="29"/>
     </row>
     <row r="65" spans="1:33">
-      <c r="A65" s="143"/>
+      <c r="A65" s="145"/>
       <c r="B65" s="46"/>
       <c r="C65" s="30"/>
       <c r="D65" s="30"/>
@@ -12058,7 +12243,7 @@
       <c r="AG65" s="30"/>
     </row>
     <row r="66" spans="1:33">
-      <c r="A66" s="143"/>
+      <c r="A66" s="145"/>
       <c r="B66" s="46"/>
       <c r="C66" s="30"/>
       <c r="D66" s="30"/>
@@ -12093,7 +12278,7 @@
       <c r="AG66" s="30"/>
     </row>
     <row r="67" spans="1:33">
-      <c r="A67" s="143"/>
+      <c r="A67" s="145"/>
       <c r="B67" s="45"/>
       <c r="C67" s="29"/>
       <c r="D67" s="29"/>
@@ -12128,7 +12313,7 @@
       <c r="AG67" s="29"/>
     </row>
     <row r="68" spans="1:33">
-      <c r="A68" s="143"/>
+      <c r="A68" s="145"/>
       <c r="B68" s="46"/>
       <c r="C68" s="30"/>
       <c r="D68" s="30"/>
@@ -12163,7 +12348,7 @@
       <c r="AG68" s="30"/>
     </row>
     <row r="69" spans="1:33">
-      <c r="A69" s="143"/>
+      <c r="A69" s="145"/>
       <c r="B69" s="46"/>
       <c r="C69" s="30"/>
       <c r="D69" s="30"/>
@@ -12198,7 +12383,7 @@
       <c r="AG69" s="30"/>
     </row>
     <row r="70" spans="1:33">
-      <c r="A70" s="143"/>
+      <c r="A70" s="145"/>
       <c r="B70" s="45"/>
       <c r="C70" s="29"/>
       <c r="D70" s="29"/>
@@ -12233,7 +12418,7 @@
       <c r="AG70" s="29"/>
     </row>
     <row r="71" spans="1:33">
-      <c r="A71" s="143"/>
+      <c r="A71" s="145"/>
       <c r="B71" s="46"/>
       <c r="C71" s="30"/>
       <c r="D71" s="30"/>
@@ -12268,7 +12453,7 @@
       <c r="AG71" s="30"/>
     </row>
     <row r="72" spans="1:33">
-      <c r="A72" s="143"/>
+      <c r="A72" s="145"/>
       <c r="B72" s="46"/>
       <c r="C72" s="30"/>
       <c r="D72" s="30"/>
@@ -12303,7 +12488,7 @@
       <c r="AG72" s="30"/>
     </row>
     <row r="73" spans="1:33">
-      <c r="A73" s="143"/>
+      <c r="A73" s="145"/>
       <c r="B73" s="45"/>
       <c r="C73" s="29"/>
       <c r="D73" s="29"/>
@@ -12338,7 +12523,7 @@
       <c r="AG73" s="29"/>
     </row>
     <row r="74" spans="1:33">
-      <c r="A74" s="143"/>
+      <c r="A74" s="145"/>
       <c r="B74" s="46"/>
       <c r="C74" s="30"/>
       <c r="D74" s="30"/>
@@ -12373,7 +12558,7 @@
       <c r="AG74" s="30"/>
     </row>
     <row r="75" spans="1:33">
-      <c r="A75" s="143"/>
+      <c r="A75" s="145"/>
       <c r="B75" s="46"/>
       <c r="C75" s="30"/>
       <c r="D75" s="30"/>
@@ -12551,51 +12736,51 @@
       <c r="A81" s="48"/>
     </row>
     <row r="82" spans="1:33">
-      <c r="A82" s="143"/>
+      <c r="A82" s="145"/>
       <c r="B82" s="45"/>
     </row>
     <row r="83" spans="1:33">
-      <c r="A83" s="143"/>
+      <c r="A83" s="145"/>
       <c r="B83" s="46"/>
     </row>
     <row r="84" spans="1:33">
-      <c r="A84" s="143"/>
+      <c r="A84" s="145"/>
       <c r="B84" s="46"/>
     </row>
     <row r="85" spans="1:33">
-      <c r="A85" s="143"/>
+      <c r="A85" s="145"/>
       <c r="B85" s="45"/>
     </row>
     <row r="86" spans="1:33">
-      <c r="A86" s="143"/>
+      <c r="A86" s="145"/>
       <c r="B86" s="46"/>
     </row>
     <row r="87" spans="1:33">
-      <c r="A87" s="143"/>
+      <c r="A87" s="145"/>
       <c r="B87" s="46"/>
     </row>
     <row r="88" spans="1:33">
-      <c r="A88" s="143"/>
+      <c r="A88" s="145"/>
       <c r="B88" s="45"/>
     </row>
     <row r="89" spans="1:33">
-      <c r="A89" s="143"/>
+      <c r="A89" s="145"/>
       <c r="B89" s="46"/>
     </row>
     <row r="90" spans="1:33">
-      <c r="A90" s="143"/>
+      <c r="A90" s="145"/>
       <c r="B90" s="46"/>
     </row>
     <row r="91" spans="1:33">
-      <c r="A91" s="143"/>
+      <c r="A91" s="145"/>
       <c r="B91" s="45"/>
     </row>
     <row r="92" spans="1:33">
-      <c r="A92" s="143"/>
+      <c r="A92" s="145"/>
       <c r="B92" s="46"/>
     </row>
     <row r="93" spans="1:33">
-      <c r="A93" s="143"/>
+      <c r="A93" s="145"/>
       <c r="B93" s="46"/>
     </row>
     <row r="94" spans="1:33">
@@ -12633,20 +12818,20 @@
       <c r="AG94" s="29"/>
     </row>
     <row r="96" spans="1:33">
-      <c r="A96" s="144"/>
+      <c r="A96" s="143"/>
       <c r="B96" s="45"/>
       <c r="C96" s="40"/>
       <c r="AA96" s="32"/>
       <c r="AC96" s="32"/>
     </row>
     <row r="97" spans="1:35">
-      <c r="A97" s="144"/>
+      <c r="A97" s="143"/>
       <c r="B97" s="46"/>
       <c r="C97" s="41"/>
       <c r="AC97" s="32"/>
     </row>
     <row r="98" spans="1:35">
-      <c r="A98" s="144"/>
+      <c r="A98" s="143"/>
       <c r="B98" s="46"/>
       <c r="C98" s="42"/>
       <c r="AA98" s="32"/>
@@ -12658,15 +12843,15 @@
       <c r="W99" s="139"/>
     </row>
     <row r="101" spans="1:35">
-      <c r="A101" s="145"/>
+      <c r="A101" s="144"/>
     </row>
     <row r="102" spans="1:35">
-      <c r="A102" s="145"/>
+      <c r="A102" s="144"/>
     </row>
     <row r="103" spans="1:35"/>
     <row r="104" spans="1:35"/>
     <row r="105" spans="1:35">
-      <c r="A105" s="144" t="s">
+      <c r="A105" s="143" t="s">
         <v>392</v>
       </c>
       <c r="B105" s="45" t="s">
@@ -12681,7 +12866,7 @@
       </c>
     </row>
     <row r="106" spans="1:35">
-      <c r="A106" s="144"/>
+      <c r="A106" s="143"/>
       <c r="B106" s="46" t="s">
         <v>22</v>
       </c>
@@ -12697,7 +12882,7 @@
       </c>
     </row>
     <row r="107" spans="1:35">
-      <c r="A107" s="144"/>
+      <c r="A107" s="143"/>
       <c r="B107" s="46" t="s">
         <v>23</v>
       </c>
@@ -12713,7 +12898,7 @@
       </c>
     </row>
     <row r="108" spans="1:35">
-      <c r="A108" s="144" t="s">
+      <c r="A108" s="143" t="s">
         <v>393</v>
       </c>
       <c r="B108" s="45" t="s">
@@ -12728,7 +12913,7 @@
       </c>
     </row>
     <row r="109" spans="1:35">
-      <c r="A109" s="144"/>
+      <c r="A109" s="143"/>
       <c r="B109" s="46" t="s">
         <v>22</v>
       </c>
@@ -12744,7 +12929,7 @@
       </c>
     </row>
     <row r="110" spans="1:35">
-      <c r="A110" s="144"/>
+      <c r="A110" s="143"/>
       <c r="B110" s="46" t="s">
         <v>23</v>
       </c>
@@ -12872,6 +13057,16 @@
     <row r="150" customFormat="1"/>
   </sheetData>
   <mergeCells count="26">
+    <mergeCell ref="A30:A32"/>
+    <mergeCell ref="A105:A107"/>
+    <mergeCell ref="A33:A35"/>
+    <mergeCell ref="A36:A38"/>
+    <mergeCell ref="A96:A98"/>
+    <mergeCell ref="A101:A102"/>
+    <mergeCell ref="A88:A90"/>
+    <mergeCell ref="A91:A93"/>
+    <mergeCell ref="A64:A66"/>
+    <mergeCell ref="A82:A84"/>
     <mergeCell ref="A108:A110"/>
     <mergeCell ref="A14:A15"/>
     <mergeCell ref="A85:A87"/>
@@ -12888,16 +13083,6 @@
     <mergeCell ref="A19:A21"/>
     <mergeCell ref="A22:A24"/>
     <mergeCell ref="A25:A27"/>
-    <mergeCell ref="A30:A32"/>
-    <mergeCell ref="A105:A107"/>
-    <mergeCell ref="A33:A35"/>
-    <mergeCell ref="A36:A38"/>
-    <mergeCell ref="A96:A98"/>
-    <mergeCell ref="A101:A102"/>
-    <mergeCell ref="A88:A90"/>
-    <mergeCell ref="A91:A93"/>
-    <mergeCell ref="A64:A66"/>
-    <mergeCell ref="A82:A84"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <legacyDrawing r:id="rId1"/>
@@ -13233,328 +13418,328 @@
       <c r="DF4" s="6"/>
     </row>
     <row r="5" spans="1:110" s="8" customFormat="1" ht="30" customHeight="1">
-      <c r="D5" s="155" t="s">
+      <c r="D5" s="146" t="s">
         <v>3</v>
       </c>
-      <c r="E5" s="156"/>
-      <c r="F5" s="156"/>
-      <c r="G5" s="156"/>
-      <c r="H5" s="156"/>
-      <c r="I5" s="156"/>
-      <c r="J5" s="156"/>
-      <c r="K5" s="156"/>
-      <c r="L5" s="156"/>
-      <c r="M5" s="156"/>
-      <c r="N5" s="156"/>
-      <c r="O5" s="156"/>
-      <c r="P5" s="156"/>
-      <c r="Q5" s="156"/>
-      <c r="R5" s="157"/>
-      <c r="S5" s="159" t="s">
+      <c r="E5" s="147"/>
+      <c r="F5" s="147"/>
+      <c r="G5" s="147"/>
+      <c r="H5" s="147"/>
+      <c r="I5" s="147"/>
+      <c r="J5" s="147"/>
+      <c r="K5" s="147"/>
+      <c r="L5" s="147"/>
+      <c r="M5" s="147"/>
+      <c r="N5" s="147"/>
+      <c r="O5" s="147"/>
+      <c r="P5" s="147"/>
+      <c r="Q5" s="147"/>
+      <c r="R5" s="148"/>
+      <c r="S5" s="157" t="s">
         <v>4</v>
       </c>
-      <c r="T5" s="160"/>
-      <c r="U5" s="160"/>
-      <c r="V5" s="160"/>
-      <c r="W5" s="160"/>
-      <c r="X5" s="160"/>
-      <c r="Y5" s="160"/>
-      <c r="Z5" s="160"/>
-      <c r="AA5" s="160"/>
-      <c r="AB5" s="160"/>
-      <c r="AC5" s="160"/>
-      <c r="AD5" s="160"/>
-      <c r="AE5" s="160"/>
-      <c r="AF5" s="160"/>
-      <c r="AG5" s="161"/>
-      <c r="AH5" s="155" t="s">
+      <c r="T5" s="158"/>
+      <c r="U5" s="158"/>
+      <c r="V5" s="158"/>
+      <c r="W5" s="158"/>
+      <c r="X5" s="158"/>
+      <c r="Y5" s="158"/>
+      <c r="Z5" s="158"/>
+      <c r="AA5" s="158"/>
+      <c r="AB5" s="158"/>
+      <c r="AC5" s="158"/>
+      <c r="AD5" s="158"/>
+      <c r="AE5" s="158"/>
+      <c r="AF5" s="158"/>
+      <c r="AG5" s="159"/>
+      <c r="AH5" s="146" t="s">
         <v>5</v>
       </c>
-      <c r="AI5" s="156"/>
-      <c r="AJ5" s="156"/>
-      <c r="AK5" s="156"/>
-      <c r="AL5" s="156"/>
-      <c r="AM5" s="156"/>
-      <c r="AN5" s="156"/>
-      <c r="AO5" s="156"/>
-      <c r="AP5" s="156"/>
-      <c r="AQ5" s="156"/>
-      <c r="AR5" s="156"/>
-      <c r="AS5" s="156"/>
-      <c r="AT5" s="156"/>
-      <c r="AU5" s="156"/>
-      <c r="AV5" s="157"/>
-      <c r="AW5" s="159" t="s">
+      <c r="AI5" s="147"/>
+      <c r="AJ5" s="147"/>
+      <c r="AK5" s="147"/>
+      <c r="AL5" s="147"/>
+      <c r="AM5" s="147"/>
+      <c r="AN5" s="147"/>
+      <c r="AO5" s="147"/>
+      <c r="AP5" s="147"/>
+      <c r="AQ5" s="147"/>
+      <c r="AR5" s="147"/>
+      <c r="AS5" s="147"/>
+      <c r="AT5" s="147"/>
+      <c r="AU5" s="147"/>
+      <c r="AV5" s="148"/>
+      <c r="AW5" s="157" t="s">
         <v>6</v>
       </c>
-      <c r="AX5" s="160"/>
-      <c r="AY5" s="160"/>
-      <c r="AZ5" s="160"/>
-      <c r="BA5" s="160"/>
-      <c r="BB5" s="160"/>
-      <c r="BC5" s="160"/>
-      <c r="BD5" s="160"/>
-      <c r="BE5" s="160"/>
-      <c r="BF5" s="160"/>
-      <c r="BG5" s="160"/>
-      <c r="BH5" s="160"/>
-      <c r="BI5" s="160"/>
-      <c r="BJ5" s="160"/>
-      <c r="BK5" s="161"/>
-      <c r="BL5" s="155" t="s">
+      <c r="AX5" s="158"/>
+      <c r="AY5" s="158"/>
+      <c r="AZ5" s="158"/>
+      <c r="BA5" s="158"/>
+      <c r="BB5" s="158"/>
+      <c r="BC5" s="158"/>
+      <c r="BD5" s="158"/>
+      <c r="BE5" s="158"/>
+      <c r="BF5" s="158"/>
+      <c r="BG5" s="158"/>
+      <c r="BH5" s="158"/>
+      <c r="BI5" s="158"/>
+      <c r="BJ5" s="158"/>
+      <c r="BK5" s="159"/>
+      <c r="BL5" s="146" t="s">
         <v>7</v>
       </c>
-      <c r="BM5" s="156"/>
-      <c r="BN5" s="156"/>
-      <c r="BO5" s="156"/>
-      <c r="BP5" s="156"/>
-      <c r="BQ5" s="156"/>
-      <c r="BR5" s="156"/>
-      <c r="BS5" s="156"/>
-      <c r="BT5" s="156"/>
-      <c r="BU5" s="156"/>
-      <c r="BV5" s="156"/>
-      <c r="BW5" s="156"/>
-      <c r="BX5" s="156"/>
-      <c r="BY5" s="156"/>
-      <c r="BZ5" s="157"/>
-      <c r="CA5" s="159" t="s">
+      <c r="BM5" s="147"/>
+      <c r="BN5" s="147"/>
+      <c r="BO5" s="147"/>
+      <c r="BP5" s="147"/>
+      <c r="BQ5" s="147"/>
+      <c r="BR5" s="147"/>
+      <c r="BS5" s="147"/>
+      <c r="BT5" s="147"/>
+      <c r="BU5" s="147"/>
+      <c r="BV5" s="147"/>
+      <c r="BW5" s="147"/>
+      <c r="BX5" s="147"/>
+      <c r="BY5" s="147"/>
+      <c r="BZ5" s="148"/>
+      <c r="CA5" s="157" t="s">
         <v>8</v>
       </c>
-      <c r="CB5" s="160"/>
-      <c r="CC5" s="160"/>
-      <c r="CD5" s="160"/>
-      <c r="CE5" s="161"/>
-      <c r="CF5" s="155" t="s">
+      <c r="CB5" s="158"/>
+      <c r="CC5" s="158"/>
+      <c r="CD5" s="158"/>
+      <c r="CE5" s="159"/>
+      <c r="CF5" s="146" t="s">
         <v>9</v>
       </c>
-      <c r="CG5" s="156"/>
-      <c r="CH5" s="156"/>
-      <c r="CI5" s="156"/>
-      <c r="CJ5" s="156"/>
-      <c r="CK5" s="156"/>
-      <c r="CL5" s="156"/>
-      <c r="CM5" s="156"/>
-      <c r="CN5" s="156"/>
-      <c r="CO5" s="156"/>
-      <c r="CP5" s="156"/>
-      <c r="CQ5" s="156"/>
-      <c r="CR5" s="156"/>
-      <c r="CS5" s="156"/>
-      <c r="CT5" s="157"/>
-      <c r="CU5" s="146" t="s">
+      <c r="CG5" s="147"/>
+      <c r="CH5" s="147"/>
+      <c r="CI5" s="147"/>
+      <c r="CJ5" s="147"/>
+      <c r="CK5" s="147"/>
+      <c r="CL5" s="147"/>
+      <c r="CM5" s="147"/>
+      <c r="CN5" s="147"/>
+      <c r="CO5" s="147"/>
+      <c r="CP5" s="147"/>
+      <c r="CQ5" s="147"/>
+      <c r="CR5" s="147"/>
+      <c r="CS5" s="147"/>
+      <c r="CT5" s="148"/>
+      <c r="CU5" s="149" t="s">
         <v>10</v>
       </c>
-      <c r="CV5" s="146"/>
-      <c r="CW5" s="146"/>
-      <c r="CX5" s="146"/>
-      <c r="CY5" s="146"/>
-      <c r="CZ5" s="158" t="s">
+      <c r="CV5" s="149"/>
+      <c r="CW5" s="149"/>
+      <c r="CX5" s="149"/>
+      <c r="CY5" s="149"/>
+      <c r="CZ5" s="150" t="s">
         <v>11</v>
       </c>
-      <c r="DA5" s="158"/>
-      <c r="DB5" s="158"/>
+      <c r="DA5" s="150"/>
+      <c r="DB5" s="150"/>
       <c r="DC5" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="DD5" s="158" t="s">
+      <c r="DD5" s="150" t="s">
         <v>13</v>
       </c>
-      <c r="DE5" s="158"/>
-      <c r="DF5" s="158"/>
+      <c r="DE5" s="150"/>
+      <c r="DF5" s="150"/>
     </row>
     <row r="6" spans="1:110" s="8" customFormat="1" ht="12.75" customHeight="1">
-      <c r="D6" s="147" t="s">
+      <c r="D6" s="151" t="s">
         <v>14</v>
       </c>
-      <c r="E6" s="148"/>
-      <c r="F6" s="149"/>
-      <c r="G6" s="147" t="s">
+      <c r="E6" s="152"/>
+      <c r="F6" s="153"/>
+      <c r="G6" s="151" t="s">
         <v>15</v>
       </c>
-      <c r="H6" s="148"/>
-      <c r="I6" s="149"/>
-      <c r="J6" s="147" t="s">
+      <c r="H6" s="152"/>
+      <c r="I6" s="153"/>
+      <c r="J6" s="151" t="s">
         <v>16</v>
       </c>
-      <c r="K6" s="148"/>
-      <c r="L6" s="149"/>
-      <c r="M6" s="147" t="s">
+      <c r="K6" s="152"/>
+      <c r="L6" s="153"/>
+      <c r="M6" s="151" t="s">
         <v>17</v>
       </c>
-      <c r="N6" s="148"/>
-      <c r="O6" s="149"/>
-      <c r="P6" s="147" t="s">
+      <c r="N6" s="152"/>
+      <c r="O6" s="153"/>
+      <c r="P6" s="151" t="s">
         <v>18</v>
       </c>
-      <c r="Q6" s="148"/>
-      <c r="R6" s="149"/>
-      <c r="S6" s="152" t="s">
+      <c r="Q6" s="152"/>
+      <c r="R6" s="153"/>
+      <c r="S6" s="154" t="s">
         <v>14</v>
       </c>
-      <c r="T6" s="153"/>
-      <c r="U6" s="154"/>
-      <c r="V6" s="152" t="s">
+      <c r="T6" s="155"/>
+      <c r="U6" s="156"/>
+      <c r="V6" s="154" t="s">
         <v>15</v>
       </c>
-      <c r="W6" s="153"/>
-      <c r="X6" s="154"/>
-      <c r="Y6" s="152" t="s">
+      <c r="W6" s="155"/>
+      <c r="X6" s="156"/>
+      <c r="Y6" s="154" t="s">
         <v>16</v>
       </c>
-      <c r="Z6" s="153"/>
-      <c r="AA6" s="154"/>
-      <c r="AB6" s="152" t="s">
+      <c r="Z6" s="155"/>
+      <c r="AA6" s="156"/>
+      <c r="AB6" s="154" t="s">
         <v>17</v>
       </c>
-      <c r="AC6" s="153"/>
-      <c r="AD6" s="154"/>
-      <c r="AE6" s="152" t="s">
+      <c r="AC6" s="155"/>
+      <c r="AD6" s="156"/>
+      <c r="AE6" s="154" t="s">
         <v>18</v>
       </c>
-      <c r="AF6" s="153"/>
-      <c r="AG6" s="154"/>
-      <c r="AH6" s="147" t="s">
+      <c r="AF6" s="155"/>
+      <c r="AG6" s="156"/>
+      <c r="AH6" s="151" t="s">
         <v>14</v>
       </c>
-      <c r="AI6" s="148"/>
-      <c r="AJ6" s="149"/>
-      <c r="AK6" s="147" t="s">
+      <c r="AI6" s="152"/>
+      <c r="AJ6" s="153"/>
+      <c r="AK6" s="151" t="s">
         <v>15</v>
       </c>
-      <c r="AL6" s="148"/>
-      <c r="AM6" s="149"/>
-      <c r="AN6" s="147" t="s">
+      <c r="AL6" s="152"/>
+      <c r="AM6" s="153"/>
+      <c r="AN6" s="151" t="s">
         <v>16</v>
       </c>
-      <c r="AO6" s="148"/>
-      <c r="AP6" s="149"/>
-      <c r="AQ6" s="147" t="s">
+      <c r="AO6" s="152"/>
+      <c r="AP6" s="153"/>
+      <c r="AQ6" s="151" t="s">
         <v>17</v>
       </c>
-      <c r="AR6" s="148"/>
-      <c r="AS6" s="149"/>
-      <c r="AT6" s="147" t="s">
+      <c r="AR6" s="152"/>
+      <c r="AS6" s="153"/>
+      <c r="AT6" s="151" t="s">
         <v>18</v>
       </c>
-      <c r="AU6" s="148"/>
-      <c r="AV6" s="149"/>
-      <c r="AW6" s="152" t="s">
+      <c r="AU6" s="152"/>
+      <c r="AV6" s="153"/>
+      <c r="AW6" s="154" t="s">
         <v>14</v>
       </c>
-      <c r="AX6" s="153"/>
-      <c r="AY6" s="154"/>
-      <c r="AZ6" s="152" t="s">
+      <c r="AX6" s="155"/>
+      <c r="AY6" s="156"/>
+      <c r="AZ6" s="154" t="s">
         <v>15</v>
       </c>
-      <c r="BA6" s="153"/>
-      <c r="BB6" s="154"/>
-      <c r="BC6" s="152" t="s">
+      <c r="BA6" s="155"/>
+      <c r="BB6" s="156"/>
+      <c r="BC6" s="154" t="s">
         <v>16</v>
       </c>
-      <c r="BD6" s="153"/>
-      <c r="BE6" s="154"/>
-      <c r="BF6" s="152" t="s">
+      <c r="BD6" s="155"/>
+      <c r="BE6" s="156"/>
+      <c r="BF6" s="154" t="s">
         <v>17</v>
       </c>
-      <c r="BG6" s="153"/>
-      <c r="BH6" s="154"/>
-      <c r="BI6" s="152" t="s">
+      <c r="BG6" s="155"/>
+      <c r="BH6" s="156"/>
+      <c r="BI6" s="154" t="s">
         <v>18</v>
       </c>
-      <c r="BJ6" s="153"/>
-      <c r="BK6" s="154"/>
-      <c r="BL6" s="147" t="s">
+      <c r="BJ6" s="155"/>
+      <c r="BK6" s="156"/>
+      <c r="BL6" s="151" t="s">
         <v>14</v>
       </c>
-      <c r="BM6" s="148"/>
-      <c r="BN6" s="149"/>
-      <c r="BO6" s="147" t="s">
+      <c r="BM6" s="152"/>
+      <c r="BN6" s="153"/>
+      <c r="BO6" s="151" t="s">
         <v>15</v>
       </c>
-      <c r="BP6" s="148"/>
-      <c r="BQ6" s="149"/>
-      <c r="BR6" s="147" t="s">
+      <c r="BP6" s="152"/>
+      <c r="BQ6" s="153"/>
+      <c r="BR6" s="151" t="s">
         <v>16</v>
       </c>
-      <c r="BS6" s="148"/>
-      <c r="BT6" s="149"/>
-      <c r="BU6" s="147" t="s">
+      <c r="BS6" s="152"/>
+      <c r="BT6" s="153"/>
+      <c r="BU6" s="151" t="s">
         <v>17</v>
       </c>
-      <c r="BV6" s="148"/>
-      <c r="BW6" s="149"/>
-      <c r="BX6" s="147" t="s">
+      <c r="BV6" s="152"/>
+      <c r="BW6" s="153"/>
+      <c r="BX6" s="151" t="s">
         <v>18</v>
       </c>
-      <c r="BY6" s="148"/>
-      <c r="BZ6" s="149"/>
-      <c r="CA6" s="150" t="s">
+      <c r="BY6" s="152"/>
+      <c r="BZ6" s="153"/>
+      <c r="CA6" s="160" t="s">
         <v>19</v>
       </c>
-      <c r="CB6" s="150" t="s">
+      <c r="CB6" s="160" t="s">
         <v>15</v>
       </c>
-      <c r="CC6" s="150" t="s">
+      <c r="CC6" s="160" t="s">
         <v>16</v>
       </c>
-      <c r="CD6" s="150" t="s">
+      <c r="CD6" s="160" t="s">
         <v>17</v>
       </c>
-      <c r="CE6" s="150" t="s">
+      <c r="CE6" s="160" t="s">
         <v>18</v>
       </c>
-      <c r="CF6" s="147" t="s">
+      <c r="CF6" s="151" t="s">
         <v>14</v>
       </c>
-      <c r="CG6" s="148"/>
-      <c r="CH6" s="149"/>
-      <c r="CI6" s="147" t="s">
+      <c r="CG6" s="152"/>
+      <c r="CH6" s="153"/>
+      <c r="CI6" s="151" t="s">
         <v>15</v>
       </c>
-      <c r="CJ6" s="148"/>
-      <c r="CK6" s="149"/>
-      <c r="CL6" s="147" t="s">
+      <c r="CJ6" s="152"/>
+      <c r="CK6" s="153"/>
+      <c r="CL6" s="151" t="s">
         <v>16</v>
       </c>
-      <c r="CM6" s="148"/>
-      <c r="CN6" s="149"/>
-      <c r="CO6" s="147" t="s">
+      <c r="CM6" s="152"/>
+      <c r="CN6" s="153"/>
+      <c r="CO6" s="151" t="s">
         <v>17</v>
       </c>
-      <c r="CP6" s="148"/>
-      <c r="CQ6" s="149"/>
-      <c r="CR6" s="147" t="s">
+      <c r="CP6" s="152"/>
+      <c r="CQ6" s="153"/>
+      <c r="CR6" s="151" t="s">
         <v>18</v>
       </c>
-      <c r="CS6" s="148"/>
-      <c r="CT6" s="149"/>
-      <c r="CU6" s="146" t="s">
+      <c r="CS6" s="152"/>
+      <c r="CT6" s="153"/>
+      <c r="CU6" s="149" t="s">
         <v>19</v>
       </c>
-      <c r="CV6" s="146" t="s">
+      <c r="CV6" s="149" t="s">
         <v>15</v>
       </c>
-      <c r="CW6" s="146" t="s">
+      <c r="CW6" s="149" t="s">
         <v>16</v>
       </c>
-      <c r="CX6" s="146" t="s">
+      <c r="CX6" s="149" t="s">
         <v>17</v>
       </c>
-      <c r="CY6" s="146" t="s">
+      <c r="CY6" s="149" t="s">
         <v>18</v>
       </c>
-      <c r="CZ6" s="158"/>
-      <c r="DA6" s="158"/>
-      <c r="DB6" s="158"/>
+      <c r="CZ6" s="150"/>
+      <c r="DA6" s="150"/>
+      <c r="DB6" s="150"/>
       <c r="DC6" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="DD6" s="158" t="s">
+      <c r="DD6" s="150" t="s">
         <v>20</v>
       </c>
-      <c r="DE6" s="158"/>
-      <c r="DF6" s="158"/>
+      <c r="DE6" s="150"/>
+      <c r="DF6" s="150"/>
     </row>
     <row r="7" spans="1:110" s="8" customFormat="1" ht="15">
       <c r="D7" s="11" t="s">
@@ -13782,15 +13967,15 @@
       <c r="BZ7" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="CA7" s="151"/>
-      <c r="CB7" s="151"/>
-      <c r="CC7" s="151" t="s">
+      <c r="CA7" s="161"/>
+      <c r="CB7" s="161"/>
+      <c r="CC7" s="161" t="s">
         <v>22</v>
       </c>
-      <c r="CD7" s="151" t="s">
+      <c r="CD7" s="161" t="s">
         <v>23</v>
       </c>
-      <c r="CE7" s="151" t="s">
+      <c r="CE7" s="161" t="s">
         <v>21</v>
       </c>
       <c r="CF7" s="11" t="s">
@@ -13838,15 +14023,15 @@
       <c r="CT7" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="CU7" s="146"/>
-      <c r="CV7" s="146"/>
-      <c r="CW7" s="146" t="s">
+      <c r="CU7" s="149"/>
+      <c r="CV7" s="149"/>
+      <c r="CW7" s="149" t="s">
         <v>22</v>
       </c>
-      <c r="CX7" s="146" t="s">
+      <c r="CX7" s="149" t="s">
         <v>23</v>
       </c>
-      <c r="CY7" s="146" t="s">
+      <c r="CY7" s="149" t="s">
         <v>21</v>
       </c>
       <c r="CZ7" s="17" t="s">
@@ -16605,6 +16790,40 @@
     </row>
   </sheetData>
   <mergeCells count="50">
+    <mergeCell ref="CV6:CV7"/>
+    <mergeCell ref="CW6:CW7"/>
+    <mergeCell ref="CX6:CX7"/>
+    <mergeCell ref="CY6:CY7"/>
+    <mergeCell ref="CF6:CH6"/>
+    <mergeCell ref="CI6:CK6"/>
+    <mergeCell ref="CL6:CN6"/>
+    <mergeCell ref="CO6:CQ6"/>
+    <mergeCell ref="CR6:CT6"/>
+    <mergeCell ref="CU6:CU7"/>
+    <mergeCell ref="CE6:CE7"/>
+    <mergeCell ref="BF6:BH6"/>
+    <mergeCell ref="BI6:BK6"/>
+    <mergeCell ref="BL6:BN6"/>
+    <mergeCell ref="BO6:BQ6"/>
+    <mergeCell ref="BR6:BT6"/>
+    <mergeCell ref="BU6:BW6"/>
+    <mergeCell ref="BX6:BZ6"/>
+    <mergeCell ref="CA6:CA7"/>
+    <mergeCell ref="CB6:CB7"/>
+    <mergeCell ref="CC6:CC7"/>
+    <mergeCell ref="CD6:CD7"/>
+    <mergeCell ref="BC6:BE6"/>
+    <mergeCell ref="V6:X6"/>
+    <mergeCell ref="Y6:AA6"/>
+    <mergeCell ref="AB6:AD6"/>
+    <mergeCell ref="AE6:AG6"/>
+    <mergeCell ref="AH6:AJ6"/>
+    <mergeCell ref="AK6:AM6"/>
+    <mergeCell ref="AN6:AP6"/>
+    <mergeCell ref="AQ6:AS6"/>
+    <mergeCell ref="AT6:AV6"/>
+    <mergeCell ref="AW6:AY6"/>
+    <mergeCell ref="AZ6:BB6"/>
     <mergeCell ref="CF5:CT5"/>
     <mergeCell ref="CU5:CY5"/>
     <mergeCell ref="CZ5:DB6"/>
@@ -16621,40 +16840,6 @@
     <mergeCell ref="AW5:BK5"/>
     <mergeCell ref="BL5:BZ5"/>
     <mergeCell ref="CA5:CE5"/>
-    <mergeCell ref="BC6:BE6"/>
-    <mergeCell ref="V6:X6"/>
-    <mergeCell ref="Y6:AA6"/>
-    <mergeCell ref="AB6:AD6"/>
-    <mergeCell ref="AE6:AG6"/>
-    <mergeCell ref="AH6:AJ6"/>
-    <mergeCell ref="AK6:AM6"/>
-    <mergeCell ref="AN6:AP6"/>
-    <mergeCell ref="AQ6:AS6"/>
-    <mergeCell ref="AT6:AV6"/>
-    <mergeCell ref="AW6:AY6"/>
-    <mergeCell ref="AZ6:BB6"/>
-    <mergeCell ref="CE6:CE7"/>
-    <mergeCell ref="BF6:BH6"/>
-    <mergeCell ref="BI6:BK6"/>
-    <mergeCell ref="BL6:BN6"/>
-    <mergeCell ref="BO6:BQ6"/>
-    <mergeCell ref="BR6:BT6"/>
-    <mergeCell ref="BU6:BW6"/>
-    <mergeCell ref="BX6:BZ6"/>
-    <mergeCell ref="CA6:CA7"/>
-    <mergeCell ref="CB6:CB7"/>
-    <mergeCell ref="CC6:CC7"/>
-    <mergeCell ref="CD6:CD7"/>
-    <mergeCell ref="CV6:CV7"/>
-    <mergeCell ref="CW6:CW7"/>
-    <mergeCell ref="CX6:CX7"/>
-    <mergeCell ref="CY6:CY7"/>
-    <mergeCell ref="CF6:CH6"/>
-    <mergeCell ref="CI6:CK6"/>
-    <mergeCell ref="CL6:CN6"/>
-    <mergeCell ref="CO6:CQ6"/>
-    <mergeCell ref="CR6:CT6"/>
-    <mergeCell ref="CU6:CU7"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -16969,8 +17154,8 @@
       </c>
     </row>
     <row r="4" spans="1:35">
-      <c r="A4" s="162"/>
-      <c r="B4" s="172"/>
+      <c r="A4" s="165"/>
+      <c r="B4" s="167"/>
       <c r="C4" s="40"/>
       <c r="D4" s="32"/>
       <c r="E4" s="32"/>
@@ -17005,8 +17190,8 @@
       <c r="AH4" s="32"/>
     </row>
     <row r="5" spans="1:35">
-      <c r="A5" s="163"/>
-      <c r="B5" s="166"/>
+      <c r="A5" s="176"/>
+      <c r="B5" s="162"/>
       <c r="C5" s="41"/>
       <c r="D5" s="30"/>
       <c r="E5" s="30"/>
@@ -17041,8 +17226,8 @@
       <c r="AH5" s="30"/>
     </row>
     <row r="6" spans="1:35">
-      <c r="A6" s="163"/>
-      <c r="B6" s="169"/>
+      <c r="A6" s="176"/>
+      <c r="B6" s="168"/>
       <c r="C6" s="42"/>
       <c r="D6" s="32"/>
       <c r="E6" s="32"/>
@@ -17077,8 +17262,8 @@
       <c r="AH6" s="30"/>
     </row>
     <row r="7" spans="1:35">
-      <c r="A7" s="163"/>
-      <c r="B7" s="172"/>
+      <c r="A7" s="176"/>
+      <c r="B7" s="167"/>
       <c r="C7" s="40"/>
       <c r="D7" s="30"/>
       <c r="E7" s="30"/>
@@ -17113,8 +17298,8 @@
       <c r="AH7" s="32"/>
     </row>
     <row r="8" spans="1:35">
-      <c r="A8" s="163"/>
-      <c r="B8" s="166"/>
+      <c r="A8" s="176"/>
+      <c r="B8" s="162"/>
       <c r="C8" s="41"/>
       <c r="D8" s="32"/>
       <c r="E8" s="32"/>
@@ -17149,8 +17334,8 @@
       <c r="AH8" s="30"/>
     </row>
     <row r="9" spans="1:35">
-      <c r="A9" s="163"/>
-      <c r="B9" s="169"/>
+      <c r="A9" s="176"/>
+      <c r="B9" s="168"/>
       <c r="C9" s="42"/>
       <c r="D9" s="30"/>
       <c r="E9" s="30"/>
@@ -17185,8 +17370,8 @@
       <c r="AH9" s="30"/>
     </row>
     <row r="10" spans="1:35">
-      <c r="A10" s="163"/>
-      <c r="B10" s="172"/>
+      <c r="A10" s="176"/>
+      <c r="B10" s="167"/>
       <c r="C10" s="40"/>
       <c r="D10" s="32"/>
       <c r="E10" s="32"/>
@@ -17221,8 +17406,8 @@
       <c r="AH10" s="32"/>
     </row>
     <row r="11" spans="1:35">
-      <c r="A11" s="163"/>
-      <c r="B11" s="166"/>
+      <c r="A11" s="176"/>
+      <c r="B11" s="162"/>
       <c r="C11" s="41"/>
       <c r="D11" s="30"/>
       <c r="E11" s="30"/>
@@ -17257,8 +17442,8 @@
       <c r="AH11" s="30"/>
     </row>
     <row r="12" spans="1:35">
-      <c r="A12" s="163"/>
-      <c r="B12" s="169"/>
+      <c r="A12" s="176"/>
+      <c r="B12" s="168"/>
       <c r="C12" s="42"/>
       <c r="D12" s="32"/>
       <c r="E12" s="32"/>
@@ -17293,8 +17478,8 @@
       <c r="AH12" s="30"/>
     </row>
     <row r="13" spans="1:35">
-      <c r="A13" s="163"/>
-      <c r="B13" s="172"/>
+      <c r="A13" s="176"/>
+      <c r="B13" s="167"/>
       <c r="C13" s="40"/>
       <c r="D13" s="30"/>
       <c r="E13" s="30"/>
@@ -17329,8 +17514,8 @@
       <c r="AH13" s="32"/>
     </row>
     <row r="14" spans="1:35">
-      <c r="A14" s="163"/>
-      <c r="B14" s="166"/>
+      <c r="A14" s="176"/>
+      <c r="B14" s="162"/>
       <c r="C14" s="41"/>
       <c r="D14" s="32"/>
       <c r="E14" s="32"/>
@@ -17365,8 +17550,8 @@
       <c r="AH14" s="30"/>
     </row>
     <row r="15" spans="1:35">
-      <c r="A15" s="163"/>
-      <c r="B15" s="169"/>
+      <c r="A15" s="176"/>
+      <c r="B15" s="168"/>
       <c r="C15" s="42"/>
       <c r="D15" s="30"/>
       <c r="E15" s="30"/>
@@ -17401,8 +17586,8 @@
       <c r="AH15" s="30"/>
     </row>
     <row r="16" spans="1:35">
-      <c r="A16" s="163"/>
-      <c r="B16" s="172"/>
+      <c r="A16" s="176"/>
+      <c r="B16" s="167"/>
       <c r="C16" s="40"/>
       <c r="D16" s="32"/>
       <c r="E16" s="32"/>
@@ -17437,8 +17622,8 @@
       <c r="AH16" s="32"/>
     </row>
     <row r="17" spans="1:34">
-      <c r="A17" s="163"/>
-      <c r="B17" s="166"/>
+      <c r="A17" s="176"/>
+      <c r="B17" s="162"/>
       <c r="C17" s="41"/>
       <c r="D17" s="30"/>
       <c r="E17" s="30"/>
@@ -17473,8 +17658,8 @@
       <c r="AH17" s="30"/>
     </row>
     <row r="18" spans="1:34">
-      <c r="A18" s="164"/>
-      <c r="B18" s="169"/>
+      <c r="A18" s="166"/>
+      <c r="B18" s="168"/>
       <c r="C18" s="42"/>
       <c r="D18" s="32"/>
       <c r="E18" s="32"/>
@@ -17509,8 +17694,8 @@
       <c r="AH18" s="30"/>
     </row>
     <row r="19" spans="1:34">
-      <c r="A19" s="165"/>
-      <c r="B19" s="166"/>
+      <c r="A19" s="163"/>
+      <c r="B19" s="162"/>
       <c r="C19" s="40"/>
       <c r="D19" s="32"/>
       <c r="E19" s="32"/>
@@ -17545,8 +17730,8 @@
       <c r="AH19" s="30"/>
     </row>
     <row r="20" spans="1:34">
-      <c r="A20" s="166"/>
-      <c r="B20" s="166"/>
+      <c r="A20" s="162"/>
+      <c r="B20" s="162"/>
       <c r="C20" s="41"/>
       <c r="D20" s="32"/>
       <c r="E20" s="32"/>
@@ -17581,8 +17766,8 @@
       <c r="AH20" s="30"/>
     </row>
     <row r="21" spans="1:34">
-      <c r="A21" s="167"/>
-      <c r="B21" s="166"/>
+      <c r="A21" s="164"/>
+      <c r="B21" s="162"/>
       <c r="C21" s="42"/>
       <c r="D21" s="32"/>
       <c r="E21" s="32"/>
@@ -17617,8 +17802,8 @@
       <c r="AH21" s="30"/>
     </row>
     <row r="22" spans="1:34">
-      <c r="A22" s="165"/>
-      <c r="B22" s="166"/>
+      <c r="A22" s="163"/>
+      <c r="B22" s="162"/>
       <c r="C22" s="40"/>
       <c r="D22" s="30"/>
       <c r="E22" s="30"/>
@@ -17653,8 +17838,8 @@
       <c r="AH22" s="32"/>
     </row>
     <row r="23" spans="1:34">
-      <c r="A23" s="166"/>
-      <c r="B23" s="166"/>
+      <c r="A23" s="162"/>
+      <c r="B23" s="162"/>
       <c r="C23" s="41"/>
       <c r="D23" s="32"/>
       <c r="E23" s="32"/>
@@ -17689,8 +17874,8 @@
       <c r="AH23" s="30"/>
     </row>
     <row r="24" spans="1:34">
-      <c r="A24" s="166"/>
-      <c r="B24" s="166"/>
+      <c r="A24" s="162"/>
+      <c r="B24" s="162"/>
       <c r="C24" s="42"/>
       <c r="D24" s="30"/>
       <c r="E24" s="30"/>
@@ -17725,8 +17910,8 @@
       <c r="AH24" s="30"/>
     </row>
     <row r="25" spans="1:34">
-      <c r="A25" s="166"/>
-      <c r="B25" s="166"/>
+      <c r="A25" s="162"/>
+      <c r="B25" s="162"/>
       <c r="C25" s="40"/>
       <c r="D25" s="32"/>
       <c r="E25" s="32"/>
@@ -17761,8 +17946,8 @@
       <c r="AH25" s="32"/>
     </row>
     <row r="26" spans="1:34">
-      <c r="A26" s="166"/>
-      <c r="B26" s="166"/>
+      <c r="A26" s="162"/>
+      <c r="B26" s="162"/>
       <c r="C26" s="41"/>
       <c r="D26" s="30"/>
       <c r="E26" s="30"/>
@@ -17797,8 +17982,8 @@
       <c r="AH26" s="30"/>
     </row>
     <row r="27" spans="1:34">
-      <c r="A27" s="166"/>
-      <c r="B27" s="166"/>
+      <c r="A27" s="162"/>
+      <c r="B27" s="162"/>
       <c r="C27" s="42"/>
       <c r="D27" s="32"/>
       <c r="E27" s="32"/>
@@ -17833,8 +18018,8 @@
       <c r="AH27" s="30"/>
     </row>
     <row r="28" spans="1:34">
-      <c r="A28" s="166"/>
-      <c r="B28" s="166"/>
+      <c r="A28" s="162"/>
+      <c r="B28" s="162"/>
       <c r="C28" s="40"/>
       <c r="D28" s="30"/>
       <c r="E28" s="30"/>
@@ -17869,8 +18054,8 @@
       <c r="AH28" s="32"/>
     </row>
     <row r="29" spans="1:34">
-      <c r="A29" s="166"/>
-      <c r="B29" s="166"/>
+      <c r="A29" s="162"/>
+      <c r="B29" s="162"/>
       <c r="C29" s="41"/>
       <c r="D29" s="32"/>
       <c r="E29" s="32"/>
@@ -17905,8 +18090,8 @@
       <c r="AH29" s="30"/>
     </row>
     <row r="30" spans="1:34">
-      <c r="A30" s="166"/>
-      <c r="B30" s="166"/>
+      <c r="A30" s="162"/>
+      <c r="B30" s="162"/>
       <c r="C30" s="42"/>
       <c r="D30" s="30"/>
       <c r="E30" s="30"/>
@@ -17941,8 +18126,8 @@
       <c r="AH30" s="30"/>
     </row>
     <row r="31" spans="1:34">
-      <c r="A31" s="166"/>
-      <c r="B31" s="166"/>
+      <c r="A31" s="162"/>
+      <c r="B31" s="162"/>
       <c r="C31" s="40"/>
       <c r="D31" s="32"/>
       <c r="E31" s="32"/>
@@ -17977,8 +18162,8 @@
       <c r="AH31" s="32"/>
     </row>
     <row r="32" spans="1:34">
-      <c r="A32" s="166"/>
-      <c r="B32" s="166"/>
+      <c r="A32" s="162"/>
+      <c r="B32" s="162"/>
       <c r="C32" s="41"/>
       <c r="D32" s="30"/>
       <c r="E32" s="30"/>
@@ -18013,8 +18198,8 @@
       <c r="AH32" s="30"/>
     </row>
     <row r="33" spans="1:34">
-      <c r="A33" s="166"/>
-      <c r="B33" s="166"/>
+      <c r="A33" s="162"/>
+      <c r="B33" s="162"/>
       <c r="C33" s="42"/>
       <c r="D33" s="32"/>
       <c r="E33" s="32"/>
@@ -18049,8 +18234,8 @@
       <c r="AH33" s="30"/>
     </row>
     <row r="34" spans="1:34">
-      <c r="A34" s="166"/>
-      <c r="B34" s="166"/>
+      <c r="A34" s="162"/>
+      <c r="B34" s="162"/>
       <c r="C34" s="40"/>
       <c r="D34" s="30"/>
       <c r="E34" s="30"/>
@@ -18085,8 +18270,8 @@
       <c r="AH34" s="32"/>
     </row>
     <row r="35" spans="1:34">
-      <c r="A35" s="166"/>
-      <c r="B35" s="166"/>
+      <c r="A35" s="162"/>
+      <c r="B35" s="162"/>
       <c r="C35" s="41"/>
       <c r="D35" s="32"/>
       <c r="E35" s="32"/>
@@ -18121,8 +18306,8 @@
       <c r="AH35" s="30"/>
     </row>
     <row r="36" spans="1:34">
-      <c r="A36" s="167"/>
-      <c r="B36" s="166"/>
+      <c r="A36" s="164"/>
+      <c r="B36" s="162"/>
       <c r="C36" s="42"/>
       <c r="D36" s="30"/>
       <c r="E36" s="30"/>
@@ -18157,8 +18342,8 @@
       <c r="AH36" s="30"/>
     </row>
     <row r="37" spans="1:34" ht="15.5" customHeight="1">
-      <c r="A37" s="165"/>
-      <c r="B37" s="166"/>
+      <c r="A37" s="163"/>
+      <c r="B37" s="162"/>
       <c r="C37" s="40"/>
       <c r="D37" s="32"/>
       <c r="E37" s="32"/>
@@ -18193,8 +18378,8 @@
       <c r="AH37" s="32"/>
     </row>
     <row r="38" spans="1:34">
-      <c r="A38" s="166"/>
-      <c r="B38" s="166"/>
+      <c r="A38" s="162"/>
+      <c r="B38" s="162"/>
       <c r="C38" s="41"/>
       <c r="D38" s="30"/>
       <c r="E38" s="30"/>
@@ -18229,8 +18414,8 @@
       <c r="AH38" s="30"/>
     </row>
     <row r="39" spans="1:34">
-      <c r="A39" s="166"/>
-      <c r="B39" s="166"/>
+      <c r="A39" s="162"/>
+      <c r="B39" s="162"/>
       <c r="C39" s="42"/>
       <c r="D39" s="32"/>
       <c r="E39" s="32"/>
@@ -18265,8 +18450,8 @@
       <c r="AH39" s="30"/>
     </row>
     <row r="40" spans="1:34">
-      <c r="A40" s="166"/>
-      <c r="B40" s="166"/>
+      <c r="A40" s="162"/>
+      <c r="B40" s="162"/>
       <c r="C40" s="40"/>
       <c r="D40" s="30"/>
       <c r="E40" s="30"/>
@@ -18301,8 +18486,8 @@
       <c r="AH40" s="32"/>
     </row>
     <row r="41" spans="1:34">
-      <c r="A41" s="166"/>
-      <c r="B41" s="166"/>
+      <c r="A41" s="162"/>
+      <c r="B41" s="162"/>
       <c r="C41" s="41"/>
       <c r="D41" s="32"/>
       <c r="E41" s="32"/>
@@ -18337,8 +18522,8 @@
       <c r="AH41" s="30"/>
     </row>
     <row r="42" spans="1:34">
-      <c r="A42" s="166"/>
-      <c r="B42" s="166"/>
+      <c r="A42" s="162"/>
+      <c r="B42" s="162"/>
       <c r="C42" s="42"/>
       <c r="D42" s="30"/>
       <c r="E42" s="30"/>
@@ -18373,8 +18558,8 @@
       <c r="AH42" s="30"/>
     </row>
     <row r="43" spans="1:34">
-      <c r="A43" s="166"/>
-      <c r="B43" s="166"/>
+      <c r="A43" s="162"/>
+      <c r="B43" s="162"/>
       <c r="C43" s="40"/>
       <c r="D43" s="32"/>
       <c r="E43" s="32"/>
@@ -18409,8 +18594,8 @@
       <c r="AH43" s="32"/>
     </row>
     <row r="44" spans="1:34">
-      <c r="A44" s="166"/>
-      <c r="B44" s="166"/>
+      <c r="A44" s="162"/>
+      <c r="B44" s="162"/>
       <c r="C44" s="41"/>
       <c r="D44" s="30"/>
       <c r="E44" s="30"/>
@@ -18445,8 +18630,8 @@
       <c r="AH44" s="30"/>
     </row>
     <row r="45" spans="1:34">
-      <c r="A45" s="166"/>
-      <c r="B45" s="166"/>
+      <c r="A45" s="162"/>
+      <c r="B45" s="162"/>
       <c r="C45" s="42"/>
       <c r="D45" s="32"/>
       <c r="E45" s="32"/>
@@ -18481,8 +18666,8 @@
       <c r="AH45" s="30"/>
     </row>
     <row r="46" spans="1:34">
-      <c r="A46" s="166"/>
-      <c r="B46" s="166"/>
+      <c r="A46" s="162"/>
+      <c r="B46" s="162"/>
       <c r="C46" s="40"/>
       <c r="D46" s="30"/>
       <c r="E46" s="30"/>
@@ -18517,8 +18702,8 @@
       <c r="AH46" s="32"/>
     </row>
     <row r="47" spans="1:34">
-      <c r="A47" s="166"/>
-      <c r="B47" s="166"/>
+      <c r="A47" s="162"/>
+      <c r="B47" s="162"/>
       <c r="C47" s="41"/>
       <c r="D47" s="32"/>
       <c r="E47" s="32"/>
@@ -18553,8 +18738,8 @@
       <c r="AH47" s="30"/>
     </row>
     <row r="48" spans="1:34">
-      <c r="A48" s="166"/>
-      <c r="B48" s="166"/>
+      <c r="A48" s="162"/>
+      <c r="B48" s="162"/>
       <c r="C48" s="42"/>
       <c r="D48" s="30"/>
       <c r="E48" s="30"/>
@@ -18589,8 +18774,8 @@
       <c r="AH48" s="30"/>
     </row>
     <row r="49" spans="1:34">
-      <c r="A49" s="166"/>
-      <c r="B49" s="166"/>
+      <c r="A49" s="162"/>
+      <c r="B49" s="162"/>
       <c r="C49" s="40"/>
       <c r="D49" s="32"/>
       <c r="E49" s="32"/>
@@ -18625,8 +18810,8 @@
       <c r="AH49" s="32"/>
     </row>
     <row r="50" spans="1:34">
-      <c r="A50" s="166"/>
-      <c r="B50" s="166"/>
+      <c r="A50" s="162"/>
+      <c r="B50" s="162"/>
       <c r="C50" s="41"/>
       <c r="D50" s="30"/>
       <c r="E50" s="30"/>
@@ -18661,8 +18846,8 @@
       <c r="AH50" s="30"/>
     </row>
     <row r="51" spans="1:34">
-      <c r="A51" s="167"/>
-      <c r="B51" s="166"/>
+      <c r="A51" s="164"/>
+      <c r="B51" s="162"/>
       <c r="C51" s="42"/>
       <c r="D51" s="32"/>
       <c r="E51" s="32"/>
@@ -18697,10 +18882,10 @@
       <c r="AH51" s="30"/>
     </row>
     <row r="52" spans="1:34" ht="15.5" customHeight="1">
-      <c r="A52" s="165" t="s">
+      <c r="A52" s="163" t="s">
         <v>6</v>
       </c>
-      <c r="B52" s="166" t="s">
+      <c r="B52" s="162" t="s">
         <v>14</v>
       </c>
       <c r="C52" s="40" t="s">
@@ -18791,8 +18976,8 @@
       </c>
     </row>
     <row r="53" spans="1:34">
-      <c r="A53" s="166"/>
-      <c r="B53" s="166"/>
+      <c r="A53" s="162"/>
+      <c r="B53" s="162"/>
       <c r="C53" s="41" t="s">
         <v>22</v>
       </c>
@@ -18881,8 +19066,8 @@
       </c>
     </row>
     <row r="54" spans="1:34">
-      <c r="A54" s="166"/>
-      <c r="B54" s="166"/>
+      <c r="A54" s="162"/>
+      <c r="B54" s="162"/>
       <c r="C54" s="42" t="s">
         <v>23</v>
       </c>
@@ -18971,8 +19156,8 @@
       </c>
     </row>
     <row r="55" spans="1:34">
-      <c r="A55" s="166"/>
-      <c r="B55" s="166" t="s">
+      <c r="A55" s="162"/>
+      <c r="B55" s="162" t="s">
         <v>15</v>
       </c>
       <c r="C55" s="40" t="s">
@@ -19063,8 +19248,8 @@
       </c>
     </row>
     <row r="56" spans="1:34">
-      <c r="A56" s="166"/>
-      <c r="B56" s="166"/>
+      <c r="A56" s="162"/>
+      <c r="B56" s="162"/>
       <c r="C56" s="41" t="s">
         <v>22</v>
       </c>
@@ -19153,8 +19338,8 @@
       </c>
     </row>
     <row r="57" spans="1:34">
-      <c r="A57" s="166"/>
-      <c r="B57" s="166"/>
+      <c r="A57" s="162"/>
+      <c r="B57" s="162"/>
       <c r="C57" s="42" t="s">
         <v>23</v>
       </c>
@@ -19242,8 +19427,8 @@
       </c>
     </row>
     <row r="58" spans="1:34">
-      <c r="A58" s="166"/>
-      <c r="B58" s="166" t="s">
+      <c r="A58" s="162"/>
+      <c r="B58" s="162" t="s">
         <v>16</v>
       </c>
       <c r="C58" s="40" t="s">
@@ -19334,8 +19519,8 @@
       </c>
     </row>
     <row r="59" spans="1:34">
-      <c r="A59" s="166"/>
-      <c r="B59" s="166"/>
+      <c r="A59" s="162"/>
+      <c r="B59" s="162"/>
       <c r="C59" s="41" t="s">
         <v>22</v>
       </c>
@@ -19424,8 +19609,8 @@
       </c>
     </row>
     <row r="60" spans="1:34">
-      <c r="A60" s="166"/>
-      <c r="B60" s="166"/>
+      <c r="A60" s="162"/>
+      <c r="B60" s="162"/>
       <c r="C60" s="42" t="s">
         <v>23</v>
       </c>
@@ -19514,8 +19699,8 @@
       </c>
     </row>
     <row r="61" spans="1:34">
-      <c r="A61" s="166"/>
-      <c r="B61" s="166" t="s">
+      <c r="A61" s="162"/>
+      <c r="B61" s="162" t="s">
         <v>17</v>
       </c>
       <c r="C61" s="40" t="s">
@@ -19606,8 +19791,8 @@
       </c>
     </row>
     <row r="62" spans="1:34">
-      <c r="A62" s="166"/>
-      <c r="B62" s="166"/>
+      <c r="A62" s="162"/>
+      <c r="B62" s="162"/>
       <c r="C62" s="41" t="s">
         <v>22</v>
       </c>
@@ -19696,8 +19881,8 @@
       </c>
     </row>
     <row r="63" spans="1:34">
-      <c r="A63" s="166"/>
-      <c r="B63" s="166"/>
+      <c r="A63" s="162"/>
+      <c r="B63" s="162"/>
       <c r="C63" s="42" t="s">
         <v>23</v>
       </c>
@@ -19786,8 +19971,8 @@
       </c>
     </row>
     <row r="64" spans="1:34">
-      <c r="A64" s="166"/>
-      <c r="B64" s="166" t="s">
+      <c r="A64" s="162"/>
+      <c r="B64" s="162" t="s">
         <v>18</v>
       </c>
       <c r="C64" s="40" t="s">
@@ -19878,8 +20063,8 @@
       </c>
     </row>
     <row r="65" spans="1:34">
-      <c r="A65" s="166"/>
-      <c r="B65" s="166"/>
+      <c r="A65" s="162"/>
+      <c r="B65" s="162"/>
       <c r="C65" s="41" t="s">
         <v>22</v>
       </c>
@@ -19968,8 +20153,8 @@
       </c>
     </row>
     <row r="66" spans="1:34">
-      <c r="A66" s="167"/>
-      <c r="B66" s="166"/>
+      <c r="A66" s="164"/>
+      <c r="B66" s="162"/>
       <c r="C66" s="42" t="s">
         <v>23</v>
       </c>
@@ -20058,8 +20243,8 @@
       </c>
     </row>
     <row r="67" spans="1:34" ht="15.5" customHeight="1">
-      <c r="A67" s="165"/>
-      <c r="B67" s="166"/>
+      <c r="A67" s="163"/>
+      <c r="B67" s="162"/>
       <c r="C67" s="40"/>
       <c r="D67" s="32"/>
       <c r="E67" s="32"/>
@@ -20094,8 +20279,8 @@
       <c r="AH67" s="32"/>
     </row>
     <row r="68" spans="1:34">
-      <c r="A68" s="166"/>
-      <c r="B68" s="166"/>
+      <c r="A68" s="162"/>
+      <c r="B68" s="162"/>
       <c r="C68" s="41"/>
       <c r="D68" s="30"/>
       <c r="E68" s="30"/>
@@ -20130,8 +20315,8 @@
       <c r="AH68" s="30"/>
     </row>
     <row r="69" spans="1:34">
-      <c r="A69" s="166"/>
-      <c r="B69" s="166"/>
+      <c r="A69" s="162"/>
+      <c r="B69" s="162"/>
       <c r="C69" s="42"/>
       <c r="D69" s="32"/>
       <c r="E69" s="32"/>
@@ -20166,8 +20351,8 @@
       <c r="AH69" s="30"/>
     </row>
     <row r="70" spans="1:34">
-      <c r="A70" s="166"/>
-      <c r="B70" s="166"/>
+      <c r="A70" s="162"/>
+      <c r="B70" s="162"/>
       <c r="C70" s="40"/>
       <c r="D70" s="30"/>
       <c r="E70" s="30"/>
@@ -20202,8 +20387,8 @@
       <c r="AH70" s="32"/>
     </row>
     <row r="71" spans="1:34">
-      <c r="A71" s="166"/>
-      <c r="B71" s="166"/>
+      <c r="A71" s="162"/>
+      <c r="B71" s="162"/>
       <c r="C71" s="41"/>
       <c r="D71" s="32"/>
       <c r="E71" s="32"/>
@@ -20238,8 +20423,8 @@
       <c r="AH71" s="30"/>
     </row>
     <row r="72" spans="1:34">
-      <c r="A72" s="166"/>
-      <c r="B72" s="166"/>
+      <c r="A72" s="162"/>
+      <c r="B72" s="162"/>
       <c r="C72" s="42"/>
       <c r="D72" s="30"/>
       <c r="E72" s="30"/>
@@ -20274,8 +20459,8 @@
       <c r="AH72" s="30"/>
     </row>
     <row r="73" spans="1:34">
-      <c r="A73" s="166"/>
-      <c r="B73" s="166"/>
+      <c r="A73" s="162"/>
+      <c r="B73" s="162"/>
       <c r="C73" s="40"/>
       <c r="D73" s="32"/>
       <c r="E73" s="32"/>
@@ -20310,8 +20495,8 @@
       <c r="AH73" s="32"/>
     </row>
     <row r="74" spans="1:34">
-      <c r="A74" s="166"/>
-      <c r="B74" s="166"/>
+      <c r="A74" s="162"/>
+      <c r="B74" s="162"/>
       <c r="C74" s="41"/>
       <c r="D74" s="30"/>
       <c r="E74" s="30"/>
@@ -20346,8 +20531,8 @@
       <c r="AH74" s="30"/>
     </row>
     <row r="75" spans="1:34">
-      <c r="A75" s="166"/>
-      <c r="B75" s="166"/>
+      <c r="A75" s="162"/>
+      <c r="B75" s="162"/>
       <c r="C75" s="42"/>
       <c r="D75" s="32"/>
       <c r="E75" s="32"/>
@@ -20382,8 +20567,8 @@
       <c r="AH75" s="30"/>
     </row>
     <row r="76" spans="1:34">
-      <c r="A76" s="166"/>
-      <c r="B76" s="166"/>
+      <c r="A76" s="162"/>
+      <c r="B76" s="162"/>
       <c r="C76" s="40"/>
       <c r="D76" s="30"/>
       <c r="E76" s="30"/>
@@ -20418,8 +20603,8 @@
       <c r="AH76" s="32"/>
     </row>
     <row r="77" spans="1:34">
-      <c r="A77" s="166"/>
-      <c r="B77" s="166"/>
+      <c r="A77" s="162"/>
+      <c r="B77" s="162"/>
       <c r="C77" s="41"/>
       <c r="D77" s="32"/>
       <c r="E77" s="32"/>
@@ -20454,8 +20639,8 @@
       <c r="AH77" s="30"/>
     </row>
     <row r="78" spans="1:34">
-      <c r="A78" s="166"/>
-      <c r="B78" s="166"/>
+      <c r="A78" s="162"/>
+      <c r="B78" s="162"/>
       <c r="C78" s="42"/>
       <c r="D78" s="30"/>
       <c r="E78" s="30"/>
@@ -20490,8 +20675,8 @@
       <c r="AH78" s="30"/>
     </row>
     <row r="79" spans="1:34">
-      <c r="A79" s="166"/>
-      <c r="B79" s="166"/>
+      <c r="A79" s="162"/>
+      <c r="B79" s="162"/>
       <c r="C79" s="40"/>
       <c r="D79" s="32"/>
       <c r="E79" s="32"/>
@@ -20526,8 +20711,8 @@
       <c r="AH79" s="32"/>
     </row>
     <row r="80" spans="1:34">
-      <c r="A80" s="166"/>
-      <c r="B80" s="166"/>
+      <c r="A80" s="162"/>
+      <c r="B80" s="162"/>
       <c r="C80" s="41"/>
       <c r="D80" s="30"/>
       <c r="E80" s="30"/>
@@ -20562,8 +20747,8 @@
       <c r="AH80" s="30"/>
     </row>
     <row r="81" spans="1:34">
-      <c r="A81" s="167"/>
-      <c r="B81" s="167"/>
+      <c r="A81" s="164"/>
+      <c r="B81" s="164"/>
       <c r="C81" s="42"/>
       <c r="D81" s="32"/>
       <c r="E81" s="32"/>
@@ -20598,9 +20783,9 @@
       <c r="AH81" s="30"/>
     </row>
     <row r="82" spans="1:34">
-      <c r="A82" s="168"/>
-      <c r="B82" s="162"/>
-      <c r="C82" s="164"/>
+      <c r="A82" s="170"/>
+      <c r="B82" s="165"/>
+      <c r="C82" s="166"/>
       <c r="D82" s="30"/>
       <c r="E82" s="30"/>
       <c r="F82" s="30"/>
@@ -20634,9 +20819,9 @@
       <c r="AH82" s="33"/>
     </row>
     <row r="83" spans="1:34">
-      <c r="A83" s="169"/>
-      <c r="B83" s="162"/>
-      <c r="C83" s="164"/>
+      <c r="A83" s="168"/>
+      <c r="B83" s="165"/>
+      <c r="C83" s="166"/>
       <c r="D83" s="32"/>
       <c r="E83" s="32"/>
       <c r="F83" s="32"/>
@@ -20670,9 +20855,9 @@
       <c r="AH83" s="33"/>
     </row>
     <row r="84" spans="1:34">
-      <c r="A84" s="169"/>
-      <c r="B84" s="162"/>
-      <c r="C84" s="164"/>
+      <c r="A84" s="168"/>
+      <c r="B84" s="165"/>
+      <c r="C84" s="166"/>
       <c r="D84" s="30"/>
       <c r="E84" s="30"/>
       <c r="F84" s="30"/>
@@ -20706,7 +20891,7 @@
       <c r="AH84" s="33"/>
     </row>
     <row r="85" spans="1:34">
-      <c r="A85" s="169"/>
+      <c r="A85" s="168"/>
       <c r="B85" s="96"/>
       <c r="C85" s="97"/>
       <c r="D85" s="32"/>
@@ -20742,7 +20927,7 @@
       <c r="AH85" s="33"/>
     </row>
     <row r="86" spans="1:34">
-      <c r="A86" s="170"/>
+      <c r="A86" s="172"/>
       <c r="B86" s="96"/>
       <c r="C86" s="97"/>
       <c r="D86" s="30"/>
@@ -20778,8 +20963,8 @@
       <c r="AH86" s="33"/>
     </row>
     <row r="87" spans="1:34">
-      <c r="A87" s="165"/>
-      <c r="B87" s="166"/>
+      <c r="A87" s="163"/>
+      <c r="B87" s="162"/>
       <c r="C87" s="40"/>
       <c r="D87" s="32"/>
       <c r="E87" s="32"/>
@@ -20814,8 +20999,8 @@
       <c r="AH87" s="33"/>
     </row>
     <row r="88" spans="1:34">
-      <c r="A88" s="166"/>
-      <c r="B88" s="166"/>
+      <c r="A88" s="162"/>
+      <c r="B88" s="162"/>
       <c r="C88" s="41"/>
       <c r="D88" s="30"/>
       <c r="E88" s="30"/>
@@ -20850,8 +21035,8 @@
       <c r="AH88" s="34"/>
     </row>
     <row r="89" spans="1:34">
-      <c r="A89" s="166"/>
-      <c r="B89" s="166"/>
+      <c r="A89" s="162"/>
+      <c r="B89" s="162"/>
       <c r="C89" s="42"/>
       <c r="D89" s="32"/>
       <c r="E89" s="32"/>
@@ -20886,8 +21071,8 @@
       <c r="AH89" s="34"/>
     </row>
     <row r="90" spans="1:34">
-      <c r="A90" s="166"/>
-      <c r="B90" s="166"/>
+      <c r="A90" s="162"/>
+      <c r="B90" s="162"/>
       <c r="C90" s="40"/>
       <c r="D90" s="30"/>
       <c r="E90" s="30"/>
@@ -20922,8 +21107,8 @@
       <c r="AH90" s="33"/>
     </row>
     <row r="91" spans="1:34">
-      <c r="A91" s="166"/>
-      <c r="B91" s="166"/>
+      <c r="A91" s="162"/>
+      <c r="B91" s="162"/>
       <c r="C91" s="41"/>
       <c r="D91" s="32"/>
       <c r="E91" s="32"/>
@@ -20958,8 +21143,8 @@
       <c r="AH91" s="34"/>
     </row>
     <row r="92" spans="1:34">
-      <c r="A92" s="166"/>
-      <c r="B92" s="166"/>
+      <c r="A92" s="162"/>
+      <c r="B92" s="162"/>
       <c r="C92" s="42"/>
       <c r="D92" s="30"/>
       <c r="E92" s="30"/>
@@ -20994,8 +21179,8 @@
       <c r="AH92" s="34"/>
     </row>
     <row r="93" spans="1:34">
-      <c r="A93" s="166"/>
-      <c r="B93" s="166"/>
+      <c r="A93" s="162"/>
+      <c r="B93" s="162"/>
       <c r="C93" s="40"/>
       <c r="D93" s="32"/>
       <c r="E93" s="32"/>
@@ -21030,8 +21215,8 @@
       <c r="AH93" s="33"/>
     </row>
     <row r="94" spans="1:34">
-      <c r="A94" s="166"/>
-      <c r="B94" s="166"/>
+      <c r="A94" s="162"/>
+      <c r="B94" s="162"/>
       <c r="C94" s="41"/>
       <c r="D94" s="30"/>
       <c r="E94" s="30"/>
@@ -21066,8 +21251,8 @@
       <c r="AH94" s="34"/>
     </row>
     <row r="95" spans="1:34">
-      <c r="A95" s="166"/>
-      <c r="B95" s="166"/>
+      <c r="A95" s="162"/>
+      <c r="B95" s="162"/>
       <c r="C95" s="42"/>
       <c r="D95" s="32"/>
       <c r="E95" s="32"/>
@@ -21102,8 +21287,8 @@
       <c r="AH95" s="34"/>
     </row>
     <row r="96" spans="1:34">
-      <c r="A96" s="166"/>
-      <c r="B96" s="166"/>
+      <c r="A96" s="162"/>
+      <c r="B96" s="162"/>
       <c r="C96" s="40"/>
       <c r="D96" s="30"/>
       <c r="E96" s="30"/>
@@ -21138,8 +21323,8 @@
       <c r="AH96" s="33"/>
     </row>
     <row r="97" spans="1:34">
-      <c r="A97" s="166"/>
-      <c r="B97" s="166"/>
+      <c r="A97" s="162"/>
+      <c r="B97" s="162"/>
       <c r="C97" s="41"/>
       <c r="D97" s="32"/>
       <c r="E97" s="32"/>
@@ -21174,8 +21359,8 @@
       <c r="AH97" s="34"/>
     </row>
     <row r="98" spans="1:34">
-      <c r="A98" s="166"/>
-      <c r="B98" s="166"/>
+      <c r="A98" s="162"/>
+      <c r="B98" s="162"/>
       <c r="C98" s="42"/>
       <c r="D98" s="30"/>
       <c r="E98" s="30"/>
@@ -21210,8 +21395,8 @@
       <c r="AH98" s="34"/>
     </row>
     <row r="99" spans="1:34">
-      <c r="A99" s="166"/>
-      <c r="B99" s="166"/>
+      <c r="A99" s="162"/>
+      <c r="B99" s="162"/>
       <c r="C99" s="40"/>
       <c r="D99" s="32"/>
       <c r="E99" s="32"/>
@@ -21246,8 +21431,8 @@
       <c r="AH99" s="33"/>
     </row>
     <row r="100" spans="1:34">
-      <c r="A100" s="166"/>
-      <c r="B100" s="166"/>
+      <c r="A100" s="162"/>
+      <c r="B100" s="162"/>
       <c r="C100" s="41"/>
       <c r="D100" s="30"/>
       <c r="E100" s="30"/>
@@ -21282,8 +21467,8 @@
       <c r="AH100" s="34"/>
     </row>
     <row r="101" spans="1:34">
-      <c r="A101" s="167"/>
-      <c r="B101" s="167"/>
+      <c r="A101" s="164"/>
+      <c r="B101" s="164"/>
       <c r="C101" s="42"/>
       <c r="D101" s="32"/>
       <c r="E101" s="32"/>
@@ -21318,9 +21503,9 @@
       <c r="AH101" s="34"/>
     </row>
     <row r="102" spans="1:34">
-      <c r="A102" s="174"/>
-      <c r="B102" s="162"/>
-      <c r="C102" s="164"/>
+      <c r="A102" s="173"/>
+      <c r="B102" s="165"/>
+      <c r="C102" s="166"/>
       <c r="D102" s="30"/>
       <c r="E102" s="30"/>
       <c r="F102" s="30"/>
@@ -21354,9 +21539,9 @@
       <c r="AH102" s="33"/>
     </row>
     <row r="103" spans="1:34">
-      <c r="A103" s="175"/>
-      <c r="B103" s="162"/>
-      <c r="C103" s="164"/>
+      <c r="A103" s="174"/>
+      <c r="B103" s="165"/>
+      <c r="C103" s="166"/>
       <c r="D103" s="32"/>
       <c r="E103" s="32"/>
       <c r="F103" s="32"/>
@@ -21390,9 +21575,9 @@
       <c r="AH103" s="33"/>
     </row>
     <row r="104" spans="1:34">
-      <c r="A104" s="175"/>
-      <c r="B104" s="162"/>
-      <c r="C104" s="164"/>
+      <c r="A104" s="174"/>
+      <c r="B104" s="165"/>
+      <c r="C104" s="166"/>
       <c r="D104" s="30"/>
       <c r="E104" s="30"/>
       <c r="F104" s="30"/>
@@ -21426,9 +21611,9 @@
       <c r="AH104" s="33"/>
     </row>
     <row r="105" spans="1:34">
-      <c r="A105" s="175"/>
-      <c r="B105" s="162"/>
-      <c r="C105" s="164"/>
+      <c r="A105" s="174"/>
+      <c r="B105" s="165"/>
+      <c r="C105" s="166"/>
       <c r="D105" s="32"/>
       <c r="E105" s="32"/>
       <c r="F105" s="32"/>
@@ -21462,9 +21647,9 @@
       <c r="AH105" s="33"/>
     </row>
     <row r="106" spans="1:34">
-      <c r="A106" s="176"/>
-      <c r="B106" s="162"/>
-      <c r="C106" s="164"/>
+      <c r="A106" s="175"/>
+      <c r="B106" s="165"/>
+      <c r="C106" s="166"/>
       <c r="D106" s="30"/>
       <c r="E106" s="30"/>
       <c r="F106" s="30"/>
@@ -21498,8 +21683,8 @@
       <c r="AH106" s="33"/>
     </row>
     <row r="107" spans="1:34" ht="15.5" customHeight="1">
-      <c r="A107" s="171"/>
-      <c r="B107" s="168"/>
+      <c r="A107" s="169"/>
+      <c r="B107" s="170"/>
       <c r="C107" s="43"/>
       <c r="D107" s="32"/>
       <c r="E107" s="32"/>
@@ -21534,8 +21719,8 @@
       <c r="AH107" s="32"/>
     </row>
     <row r="108" spans="1:34">
-      <c r="A108" s="172"/>
-      <c r="B108" s="169"/>
+      <c r="A108" s="167"/>
+      <c r="B108" s="168"/>
       <c r="C108" s="44"/>
       <c r="D108" s="30"/>
       <c r="E108" s="30"/>
@@ -21570,8 +21755,8 @@
       <c r="AH108" s="30"/>
     </row>
     <row r="109" spans="1:34">
-      <c r="A109" s="173"/>
-      <c r="B109" s="170"/>
+      <c r="A109" s="171"/>
+      <c r="B109" s="172"/>
       <c r="C109" s="44"/>
       <c r="D109" s="32"/>
       <c r="E109" s="32"/>
@@ -21642,8 +21827,8 @@
       <c r="AH110" s="129"/>
     </row>
     <row r="111" spans="1:34" ht="15.5" customHeight="1">
-      <c r="A111" s="171"/>
-      <c r="B111" s="168"/>
+      <c r="A111" s="169"/>
+      <c r="B111" s="170"/>
       <c r="C111" s="43"/>
       <c r="D111" s="32"/>
       <c r="E111" s="32"/>
@@ -21678,8 +21863,8 @@
       <c r="AH111" s="32"/>
     </row>
     <row r="112" spans="1:34">
-      <c r="A112" s="172"/>
-      <c r="B112" s="169"/>
+      <c r="A112" s="167"/>
+      <c r="B112" s="168"/>
       <c r="C112" s="44"/>
       <c r="D112" s="30"/>
       <c r="E112" s="30"/>
@@ -21714,8 +21899,8 @@
       <c r="AH112" s="30"/>
     </row>
     <row r="113" spans="1:34">
-      <c r="A113" s="172"/>
-      <c r="B113" s="169"/>
+      <c r="A113" s="167"/>
+      <c r="B113" s="168"/>
       <c r="C113" s="44"/>
       <c r="D113" s="32"/>
       <c r="E113" s="32"/>
@@ -21759,7 +21944,7 @@
       <c r="AE115" s="33"/>
     </row>
     <row r="117" spans="1:34" ht="27.5" customHeight="1">
-      <c r="A117" s="144"/>
+      <c r="A117" s="143"/>
       <c r="B117" s="137"/>
       <c r="Z117" s="131"/>
       <c r="AA117" s="131"/>
@@ -21767,7 +21952,7 @@
       <c r="AC117" s="131"/>
     </row>
     <row r="118" spans="1:34">
-      <c r="A118" s="144"/>
+      <c r="A118" s="143"/>
       <c r="B118" s="137"/>
       <c r="Z118" s="131"/>
       <c r="AA118" s="131"/>
@@ -21775,7 +21960,7 @@
       <c r="AC118" s="131"/>
     </row>
     <row r="119" spans="1:34">
-      <c r="A119" s="144"/>
+      <c r="A119" s="143"/>
       <c r="B119" s="137"/>
       <c r="Z119" s="131"/>
       <c r="AA119" s="131"/>
@@ -21783,7 +21968,7 @@
       <c r="AC119" s="131"/>
     </row>
     <row r="120" spans="1:34">
-      <c r="A120" s="144"/>
+      <c r="A120" s="143"/>
       <c r="B120" s="137"/>
       <c r="Z120" s="131"/>
       <c r="AA120" s="131"/>
@@ -21791,7 +21976,7 @@
       <c r="AC120" s="131"/>
     </row>
     <row r="121" spans="1:34">
-      <c r="A121" s="144"/>
+      <c r="A121" s="143"/>
       <c r="B121" s="137"/>
       <c r="Z121" s="131"/>
       <c r="AA121" s="131"/>
@@ -21799,7 +21984,7 @@
       <c r="AC121" s="131"/>
     </row>
     <row r="122" spans="1:34">
-      <c r="A122" s="144"/>
+      <c r="A122" s="143"/>
       <c r="B122" s="137"/>
       <c r="Z122" s="131"/>
       <c r="AA122" s="131"/>
@@ -21807,7 +21992,7 @@
       <c r="AC122" s="131"/>
     </row>
     <row r="123" spans="1:34">
-      <c r="A123" s="144"/>
+      <c r="A123" s="143"/>
       <c r="B123" s="137"/>
       <c r="Z123" s="131"/>
       <c r="AA123" s="131"/>
@@ -21815,7 +22000,7 @@
       <c r="AC123" s="131"/>
     </row>
     <row r="124" spans="1:34">
-      <c r="A124" s="144"/>
+      <c r="A124" s="143"/>
       <c r="B124" s="137"/>
       <c r="Z124" s="131"/>
       <c r="AA124" s="131"/>
@@ -21823,7 +22008,7 @@
       <c r="AC124" s="131"/>
     </row>
     <row r="125" spans="1:34">
-      <c r="A125" s="144"/>
+      <c r="A125" s="143"/>
       <c r="B125" s="137"/>
       <c r="Z125" s="131"/>
       <c r="AA125" s="131"/>
@@ -21831,20 +22016,20 @@
       <c r="AC125" s="131"/>
     </row>
     <row r="126" spans="1:34">
-      <c r="A126" s="144"/>
+      <c r="A126" s="143"/>
       <c r="B126" s="137"/>
       <c r="C126" s="43"/>
     </row>
     <row r="127" spans="1:34">
-      <c r="A127" s="144"/>
+      <c r="A127" s="143"/>
       <c r="C127" s="44"/>
     </row>
     <row r="128" spans="1:34">
-      <c r="A128" s="144"/>
+      <c r="A128" s="143"/>
       <c r="C128" s="44"/>
     </row>
     <row r="129" spans="1:35">
-      <c r="A129" s="144" t="s">
+      <c r="A129" s="143" t="s">
         <v>394</v>
       </c>
       <c r="B129" s="137" t="s">
@@ -21858,19 +22043,19 @@
       </c>
     </row>
     <row r="130" spans="1:35">
-      <c r="A130" s="144"/>
+      <c r="A130" s="143"/>
       <c r="C130" s="44" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="131" spans="1:35">
-      <c r="A131" s="144"/>
+      <c r="A131" s="143"/>
       <c r="C131" s="44" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="132" spans="1:35">
-      <c r="A132" s="144" t="s">
+      <c r="A132" s="143" t="s">
         <v>396</v>
       </c>
       <c r="B132" s="137" t="s">
@@ -21886,7 +22071,7 @@
       <c r="AI132" s="32"/>
     </row>
     <row r="133" spans="1:35">
-      <c r="A133" s="144"/>
+      <c r="A133" s="143"/>
       <c r="C133" s="44" t="s">
         <v>22</v>
       </c>
@@ -21896,7 +22081,7 @@
       </c>
     </row>
     <row r="134" spans="1:35">
-      <c r="A134" s="144"/>
+      <c r="A134" s="143"/>
       <c r="C134" s="44" t="s">
         <v>23</v>
       </c>
@@ -21906,7 +22091,7 @@
       </c>
     </row>
     <row r="135" spans="1:35">
-      <c r="A135" s="144" t="s">
+      <c r="A135" s="143" t="s">
         <v>398</v>
       </c>
       <c r="B135" s="137" t="s">
@@ -21921,7 +22106,7 @@
       </c>
     </row>
     <row r="136" spans="1:35">
-      <c r="A136" s="144"/>
+      <c r="A136" s="143"/>
       <c r="C136" s="44" t="s">
         <v>22</v>
       </c>
@@ -21931,7 +22116,7 @@
       </c>
     </row>
     <row r="137" spans="1:35">
-      <c r="A137" s="144"/>
+      <c r="A137" s="143"/>
       <c r="C137" s="44" t="s">
         <v>23</v>
       </c>
@@ -21942,6 +22127,47 @@
     </row>
   </sheetData>
   <mergeCells count="57">
+    <mergeCell ref="A135:A137"/>
+    <mergeCell ref="A132:A134"/>
+    <mergeCell ref="A117:A119"/>
+    <mergeCell ref="A120:A122"/>
+    <mergeCell ref="A123:A125"/>
+    <mergeCell ref="A129:A131"/>
+    <mergeCell ref="A126:A128"/>
+    <mergeCell ref="A4:A18"/>
+    <mergeCell ref="A22:A36"/>
+    <mergeCell ref="A37:A51"/>
+    <mergeCell ref="A52:A66"/>
+    <mergeCell ref="A82:A86"/>
+    <mergeCell ref="A87:A101"/>
+    <mergeCell ref="A107:B109"/>
+    <mergeCell ref="A111:B113"/>
+    <mergeCell ref="A102:A106"/>
+    <mergeCell ref="B102:C102"/>
+    <mergeCell ref="B103:C103"/>
+    <mergeCell ref="B104:C104"/>
+    <mergeCell ref="B105:C105"/>
+    <mergeCell ref="B106:C106"/>
+    <mergeCell ref="B96:B98"/>
+    <mergeCell ref="B99:B101"/>
+    <mergeCell ref="B4:B6"/>
+    <mergeCell ref="B7:B9"/>
+    <mergeCell ref="B10:B12"/>
+    <mergeCell ref="B13:B15"/>
+    <mergeCell ref="B16:B18"/>
+    <mergeCell ref="B22:B24"/>
+    <mergeCell ref="B25:B27"/>
+    <mergeCell ref="B28:B30"/>
+    <mergeCell ref="B31:B33"/>
+    <mergeCell ref="B34:B36"/>
+    <mergeCell ref="B58:B60"/>
+    <mergeCell ref="B61:B63"/>
+    <mergeCell ref="B64:B66"/>
+    <mergeCell ref="B37:B39"/>
+    <mergeCell ref="B40:B42"/>
+    <mergeCell ref="B43:B45"/>
+    <mergeCell ref="B46:B48"/>
+    <mergeCell ref="B49:B51"/>
     <mergeCell ref="B19:B21"/>
     <mergeCell ref="A19:A21"/>
     <mergeCell ref="B87:B89"/>
@@ -21958,47 +22184,6 @@
     <mergeCell ref="B79:B81"/>
     <mergeCell ref="B52:B54"/>
     <mergeCell ref="B55:B57"/>
-    <mergeCell ref="B58:B60"/>
-    <mergeCell ref="B61:B63"/>
-    <mergeCell ref="B64:B66"/>
-    <mergeCell ref="B37:B39"/>
-    <mergeCell ref="B40:B42"/>
-    <mergeCell ref="B43:B45"/>
-    <mergeCell ref="B46:B48"/>
-    <mergeCell ref="B49:B51"/>
-    <mergeCell ref="B22:B24"/>
-    <mergeCell ref="B25:B27"/>
-    <mergeCell ref="B28:B30"/>
-    <mergeCell ref="B31:B33"/>
-    <mergeCell ref="B34:B36"/>
-    <mergeCell ref="B4:B6"/>
-    <mergeCell ref="B7:B9"/>
-    <mergeCell ref="B10:B12"/>
-    <mergeCell ref="B13:B15"/>
-    <mergeCell ref="B16:B18"/>
-    <mergeCell ref="A87:A101"/>
-    <mergeCell ref="A107:B109"/>
-    <mergeCell ref="A111:B113"/>
-    <mergeCell ref="A102:A106"/>
-    <mergeCell ref="B102:C102"/>
-    <mergeCell ref="B103:C103"/>
-    <mergeCell ref="B104:C104"/>
-    <mergeCell ref="B105:C105"/>
-    <mergeCell ref="B106:C106"/>
-    <mergeCell ref="B96:B98"/>
-    <mergeCell ref="B99:B101"/>
-    <mergeCell ref="A4:A18"/>
-    <mergeCell ref="A22:A36"/>
-    <mergeCell ref="A37:A51"/>
-    <mergeCell ref="A52:A66"/>
-    <mergeCell ref="A82:A86"/>
-    <mergeCell ref="A135:A137"/>
-    <mergeCell ref="A132:A134"/>
-    <mergeCell ref="A117:A119"/>
-    <mergeCell ref="A120:A122"/>
-    <mergeCell ref="A123:A125"/>
-    <mergeCell ref="A129:A131"/>
-    <mergeCell ref="A126:A128"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -22368,7 +22553,7 @@
       <c r="AH4" s="28"/>
     </row>
     <row r="5" spans="1:36">
-      <c r="A5" s="143"/>
+      <c r="A5" s="145"/>
       <c r="B5" s="53"/>
       <c r="C5" s="45"/>
       <c r="D5" s="29"/>
@@ -22404,7 +22589,7 @@
       <c r="AH5" s="29"/>
     </row>
     <row r="6" spans="1:36">
-      <c r="A6" s="143"/>
+      <c r="A6" s="145"/>
       <c r="B6" s="53"/>
       <c r="C6" s="46"/>
       <c r="D6" s="30"/>
@@ -22440,7 +22625,7 @@
       <c r="AH6" s="30"/>
     </row>
     <row r="7" spans="1:36">
-      <c r="A7" s="143"/>
+      <c r="A7" s="145"/>
       <c r="B7" s="53"/>
       <c r="C7" s="46"/>
       <c r="D7" s="30"/>
@@ -22476,8 +22661,8 @@
       <c r="AH7" s="30"/>
     </row>
     <row r="8" spans="1:36">
-      <c r="A8" s="143"/>
-      <c r="B8" s="172"/>
+      <c r="A8" s="145"/>
+      <c r="B8" s="167"/>
       <c r="C8" s="40"/>
       <c r="D8" s="32"/>
       <c r="E8" s="32"/>
@@ -22512,8 +22697,8 @@
       <c r="AH8" s="32"/>
     </row>
     <row r="9" spans="1:36">
-      <c r="A9" s="143"/>
-      <c r="B9" s="166"/>
+      <c r="A9" s="145"/>
+      <c r="B9" s="162"/>
       <c r="C9" s="41"/>
       <c r="D9" s="30"/>
       <c r="E9" s="30"/>
@@ -22548,8 +22733,8 @@
       <c r="AH9" s="30"/>
     </row>
     <row r="10" spans="1:36">
-      <c r="A10" s="143"/>
-      <c r="B10" s="169"/>
+      <c r="A10" s="145"/>
+      <c r="B10" s="168"/>
       <c r="C10" s="42"/>
       <c r="D10" s="32"/>
       <c r="E10" s="32"/>
@@ -22584,8 +22769,8 @@
       <c r="AH10" s="30"/>
     </row>
     <row r="11" spans="1:36">
-      <c r="A11" s="143"/>
-      <c r="B11" s="172"/>
+      <c r="A11" s="145"/>
+      <c r="B11" s="167"/>
       <c r="C11" s="40"/>
       <c r="D11" s="30"/>
       <c r="E11" s="30"/>
@@ -22620,8 +22805,8 @@
       <c r="AH11" s="32"/>
     </row>
     <row r="12" spans="1:36">
-      <c r="A12" s="143"/>
-      <c r="B12" s="166"/>
+      <c r="A12" s="145"/>
+      <c r="B12" s="162"/>
       <c r="C12" s="41"/>
       <c r="D12" s="32"/>
       <c r="E12" s="32"/>
@@ -22656,8 +22841,8 @@
       <c r="AH12" s="30"/>
     </row>
     <row r="13" spans="1:36">
-      <c r="A13" s="143"/>
-      <c r="B13" s="169"/>
+      <c r="A13" s="145"/>
+      <c r="B13" s="168"/>
       <c r="C13" s="42"/>
       <c r="D13" s="30"/>
       <c r="E13" s="30"/>
@@ -22692,7 +22877,7 @@
       <c r="AH13" s="30"/>
     </row>
     <row r="14" spans="1:36">
-      <c r="A14" s="143"/>
+      <c r="A14" s="145"/>
       <c r="B14" s="177"/>
       <c r="C14" s="40"/>
       <c r="D14" s="32"/>
@@ -22728,7 +22913,7 @@
       <c r="AH14" s="32"/>
     </row>
     <row r="15" spans="1:36">
-      <c r="A15" s="143"/>
+      <c r="A15" s="145"/>
       <c r="B15" s="178"/>
       <c r="C15" s="41"/>
       <c r="D15" s="30"/>
@@ -22764,7 +22949,7 @@
       <c r="AH15" s="30"/>
     </row>
     <row r="16" spans="1:36">
-      <c r="A16" s="143"/>
+      <c r="A16" s="145"/>
       <c r="B16" s="179"/>
       <c r="C16" s="42"/>
       <c r="D16" s="32"/>
@@ -22800,56 +22985,56 @@
       <c r="AH16" s="30"/>
     </row>
     <row r="17" spans="1:31">
-      <c r="A17" s="143"/>
-      <c r="B17" s="172"/>
+      <c r="A17" s="145"/>
+      <c r="B17" s="167"/>
       <c r="C17" s="40"/>
       <c r="AB17" s="32"/>
       <c r="AE17" s="32"/>
     </row>
     <row r="18" spans="1:31">
-      <c r="A18" s="143"/>
-      <c r="B18" s="166"/>
+      <c r="A18" s="145"/>
+      <c r="B18" s="162"/>
       <c r="C18" s="41"/>
       <c r="AB18" s="32"/>
       <c r="AE18" s="32"/>
     </row>
     <row r="19" spans="1:31">
-      <c r="A19" s="143"/>
-      <c r="B19" s="169"/>
+      <c r="A19" s="145"/>
+      <c r="B19" s="168"/>
       <c r="C19" s="42"/>
       <c r="AB19" s="32"/>
       <c r="AE19" s="32"/>
     </row>
     <row r="20" spans="1:31">
-      <c r="A20" s="143"/>
-      <c r="B20" s="172"/>
+      <c r="A20" s="145"/>
+      <c r="B20" s="167"/>
       <c r="C20" s="40"/>
       <c r="AB20" s="32"/>
       <c r="AE20" s="32"/>
     </row>
     <row r="21" spans="1:31">
-      <c r="A21" s="143"/>
-      <c r="B21" s="166"/>
+      <c r="A21" s="145"/>
+      <c r="B21" s="162"/>
       <c r="C21" s="41"/>
       <c r="AB21" s="32"/>
       <c r="AE21" s="32"/>
     </row>
     <row r="22" spans="1:31">
-      <c r="A22" s="143"/>
-      <c r="B22" s="169"/>
+      <c r="A22" s="145"/>
+      <c r="B22" s="168"/>
       <c r="C22" s="42"/>
       <c r="AB22" s="32"/>
       <c r="AE22" s="32"/>
     </row>
     <row r="23" spans="1:31">
-      <c r="A23" s="143"/>
+      <c r="A23" s="145"/>
       <c r="B23" s="177"/>
       <c r="C23" s="41"/>
       <c r="AB23" s="32"/>
       <c r="AE23" s="32"/>
     </row>
     <row r="24" spans="1:31">
-      <c r="A24" s="143"/>
+      <c r="A24" s="145"/>
       <c r="B24" s="178"/>
       <c r="C24" s="41"/>
       <c r="X24" s="32"/>
@@ -22857,7 +23042,7 @@
       <c r="AE24" s="32"/>
     </row>
     <row r="25" spans="1:31">
-      <c r="A25" s="143"/>
+      <c r="A25" s="145"/>
       <c r="B25" s="179"/>
       <c r="C25" s="41"/>
       <c r="X25" s="32"/>
@@ -22865,92 +23050,92 @@
       <c r="AE25" s="32"/>
     </row>
     <row r="26" spans="1:31">
-      <c r="A26" s="143"/>
-      <c r="B26" s="172"/>
+      <c r="A26" s="145"/>
+      <c r="B26" s="167"/>
       <c r="C26" s="40"/>
       <c r="X26" s="32"/>
       <c r="AB26" s="32"/>
       <c r="AE26" s="32"/>
     </row>
     <row r="27" spans="1:31">
-      <c r="A27" s="143"/>
-      <c r="B27" s="166"/>
+      <c r="A27" s="145"/>
+      <c r="B27" s="162"/>
       <c r="C27" s="41"/>
       <c r="X27" s="32"/>
       <c r="AB27" s="54"/>
       <c r="AE27" s="32"/>
     </row>
     <row r="28" spans="1:31">
-      <c r="A28" s="143"/>
-      <c r="B28" s="169"/>
+      <c r="A28" s="145"/>
+      <c r="B28" s="168"/>
       <c r="C28" s="42"/>
       <c r="X28" s="32"/>
       <c r="AE28" s="32"/>
     </row>
     <row r="29" spans="1:31">
-      <c r="A29" s="143"/>
-      <c r="B29" s="172"/>
+      <c r="A29" s="145"/>
+      <c r="B29" s="167"/>
       <c r="C29" s="40"/>
       <c r="X29" s="32"/>
       <c r="AE29" s="32"/>
     </row>
     <row r="30" spans="1:31">
-      <c r="A30" s="143"/>
-      <c r="B30" s="166"/>
+      <c r="A30" s="145"/>
+      <c r="B30" s="162"/>
       <c r="C30" s="41"/>
       <c r="X30" s="32"/>
       <c r="AE30" s="32"/>
     </row>
     <row r="31" spans="1:31">
-      <c r="A31" s="143"/>
-      <c r="B31" s="169"/>
+      <c r="A31" s="145"/>
+      <c r="B31" s="168"/>
       <c r="C31" s="42"/>
       <c r="X31" s="32"/>
       <c r="AE31" s="32"/>
     </row>
     <row r="32" spans="1:31">
-      <c r="A32" s="143"/>
-      <c r="B32" s="172"/>
+      <c r="A32" s="145"/>
+      <c r="B32" s="167"/>
       <c r="C32" s="40"/>
       <c r="X32" s="32"/>
       <c r="AE32" s="32"/>
     </row>
     <row r="33" spans="1:36">
-      <c r="A33" s="143"/>
-      <c r="B33" s="166"/>
+      <c r="A33" s="145"/>
+      <c r="B33" s="162"/>
       <c r="C33" s="41"/>
       <c r="X33" s="32"/>
       <c r="AE33" s="32"/>
     </row>
     <row r="34" spans="1:36">
-      <c r="A34" s="143"/>
-      <c r="B34" s="169"/>
+      <c r="A34" s="145"/>
+      <c r="B34" s="168"/>
       <c r="C34" s="42"/>
       <c r="X34" s="32"/>
       <c r="AE34" s="32"/>
     </row>
     <row r="35" spans="1:36">
-      <c r="A35" s="166"/>
+      <c r="A35" s="162"/>
       <c r="B35" s="177"/>
       <c r="C35" s="40"/>
       <c r="X35" s="32"/>
       <c r="AE35" s="32"/>
     </row>
     <row r="36" spans="1:36">
-      <c r="A36" s="166"/>
+      <c r="A36" s="162"/>
       <c r="B36" s="178"/>
       <c r="C36" s="41"/>
       <c r="X36" s="32"/>
       <c r="AE36" s="32"/>
     </row>
     <row r="37" spans="1:36">
-      <c r="A37" s="166"/>
+      <c r="A37" s="162"/>
       <c r="B37" s="179"/>
       <c r="C37" s="42"/>
       <c r="AE37" s="32"/>
     </row>
     <row r="38" spans="1:36">
-      <c r="A38" s="166" t="s">
+      <c r="A38" s="162" t="s">
         <v>390</v>
       </c>
       <c r="B38" s="177" t="s">
@@ -22964,7 +23149,7 @@
       </c>
     </row>
     <row r="39" spans="1:36">
-      <c r="A39" s="166"/>
+      <c r="A39" s="162"/>
       <c r="B39" s="178"/>
       <c r="C39" s="41" t="s">
         <v>22</v>
@@ -22974,7 +23159,7 @@
       </c>
     </row>
     <row r="40" spans="1:36">
-      <c r="A40" s="166"/>
+      <c r="A40" s="162"/>
       <c r="B40" s="179"/>
       <c r="C40" s="42" t="s">
         <v>23</v>
@@ -22984,7 +23169,7 @@
       </c>
     </row>
     <row r="41" spans="1:36">
-      <c r="A41" s="166" t="s">
+      <c r="A41" s="162" t="s">
         <v>395</v>
       </c>
       <c r="B41" s="177" t="s">
@@ -23005,12 +23190,9 @@
       <c r="AE41" s="32">
         <v>12.3</v>
       </c>
-      <c r="AJ41">
-        <v>15.7</v>
-      </c>
     </row>
     <row r="42" spans="1:36">
-      <c r="A42" s="166"/>
+      <c r="A42" s="162"/>
       <c r="B42" s="178"/>
       <c r="C42" s="41" t="s">
         <v>22</v>
@@ -23024,12 +23206,9 @@
       <c r="AE42" s="32">
         <v>7.8</v>
       </c>
-      <c r="AJ42">
-        <v>10</v>
-      </c>
     </row>
     <row r="43" spans="1:36">
-      <c r="A43" s="166"/>
+      <c r="A43" s="162"/>
       <c r="B43" s="179"/>
       <c r="C43" s="42" t="s">
         <v>23</v>
@@ -23043,12 +23222,9 @@
       <c r="AE43" s="32">
         <v>18.899999999999999</v>
       </c>
-      <c r="AJ43">
-        <v>21.4</v>
-      </c>
     </row>
     <row r="44" spans="1:36">
-      <c r="A44" s="166" t="s">
+      <c r="A44" s="162" t="s">
         <v>400</v>
       </c>
       <c r="B44" s="177" t="s">
@@ -23071,7 +23247,7 @@
       </c>
     </row>
     <row r="45" spans="1:36">
-      <c r="A45" s="166"/>
+      <c r="A45" s="162"/>
       <c r="B45" s="178"/>
       <c r="C45" s="41" t="s">
         <v>22</v>
@@ -23087,7 +23263,7 @@
       </c>
     </row>
     <row r="46" spans="1:36">
-      <c r="A46" s="166"/>
+      <c r="A46" s="162"/>
       <c r="B46" s="179"/>
       <c r="C46" s="42" t="s">
         <v>23</v>
@@ -23103,7 +23279,7 @@
       </c>
     </row>
     <row r="47" spans="1:36" ht="30">
-      <c r="A47" s="169" t="s">
+      <c r="A47" s="168" t="s">
         <v>382</v>
       </c>
       <c r="B47" s="135" t="s">
@@ -23118,7 +23294,7 @@
       <c r="AE47" s="32"/>
     </row>
     <row r="48" spans="1:36" ht="30">
-      <c r="A48" s="169"/>
+      <c r="A48" s="168"/>
       <c r="B48" s="135" t="s">
         <v>102</v>
       </c>
@@ -23130,19 +23306,82 @@
       </c>
       <c r="AE48" s="32"/>
     </row>
-    <row r="52" spans="31:31">
+    <row r="49" spans="1:36">
+      <c r="A49" s="162" t="s">
+        <v>427</v>
+      </c>
+      <c r="B49" s="177" t="s">
+        <v>389</v>
+      </c>
+      <c r="C49" s="40" t="s">
+        <v>21</v>
+      </c>
+      <c r="X49">
+        <v>2.1</v>
+      </c>
+      <c r="AA49">
+        <v>8.1999999999999993</v>
+      </c>
+      <c r="AB49">
+        <v>16.100000000000001</v>
+      </c>
+      <c r="AE49" s="32">
+        <v>12.3</v>
+      </c>
+      <c r="AJ49">
+        <v>15.7</v>
+      </c>
+    </row>
+    <row r="50" spans="1:36">
+      <c r="A50" s="162"/>
+      <c r="B50" s="178"/>
+      <c r="C50" s="41" t="s">
+        <v>22</v>
+      </c>
+      <c r="AA50">
+        <v>3.2</v>
+      </c>
+      <c r="AB50">
+        <v>8.8000000000000007</v>
+      </c>
+      <c r="AE50" s="32">
+        <v>7.8</v>
+      </c>
+      <c r="AJ50">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="51" spans="1:36">
+      <c r="A51" s="162"/>
+      <c r="B51" s="179"/>
+      <c r="C51" s="42" t="s">
+        <v>23</v>
+      </c>
+      <c r="AA51">
+        <v>18.2</v>
+      </c>
+      <c r="AB51">
+        <v>27.4</v>
+      </c>
+      <c r="AE51" s="32">
+        <v>18.899999999999999</v>
+      </c>
+      <c r="AJ51">
+        <v>21.4</v>
+      </c>
+    </row>
+    <row r="52" spans="1:36">
       <c r="AE52" s="32"/>
     </row>
   </sheetData>
-  <mergeCells count="22">
-    <mergeCell ref="B41:B43"/>
-    <mergeCell ref="A38:A40"/>
-    <mergeCell ref="A41:A43"/>
-    <mergeCell ref="A47:A48"/>
-    <mergeCell ref="B35:B37"/>
-    <mergeCell ref="A35:A37"/>
-    <mergeCell ref="A44:A46"/>
-    <mergeCell ref="B44:B46"/>
+  <mergeCells count="24">
+    <mergeCell ref="A49:A51"/>
+    <mergeCell ref="B49:B51"/>
+    <mergeCell ref="A5:A7"/>
+    <mergeCell ref="B8:B10"/>
+    <mergeCell ref="B11:B13"/>
+    <mergeCell ref="B14:B16"/>
+    <mergeCell ref="A8:A16"/>
     <mergeCell ref="B23:B25"/>
     <mergeCell ref="B38:B40"/>
     <mergeCell ref="B29:B31"/>
@@ -23152,11 +23391,14 @@
     <mergeCell ref="B17:B19"/>
     <mergeCell ref="B20:B22"/>
     <mergeCell ref="B26:B28"/>
-    <mergeCell ref="A5:A7"/>
-    <mergeCell ref="B8:B10"/>
-    <mergeCell ref="B11:B13"/>
-    <mergeCell ref="B14:B16"/>
-    <mergeCell ref="A8:A16"/>
+    <mergeCell ref="B41:B43"/>
+    <mergeCell ref="A38:A40"/>
+    <mergeCell ref="A41:A43"/>
+    <mergeCell ref="A47:A48"/>
+    <mergeCell ref="B35:B37"/>
+    <mergeCell ref="A35:A37"/>
+    <mergeCell ref="A44:A46"/>
+    <mergeCell ref="B44:B46"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -24211,15 +24453,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8">
-      <c r="A1" s="191" t="s">
+      <c r="A1" s="206" t="s">
         <v>233</v>
       </c>
       <c r="B1" s="73"/>
-      <c r="C1" s="191" t="s">
+      <c r="C1" s="206" t="s">
         <v>235</v>
       </c>
       <c r="D1" s="73"/>
-      <c r="E1" s="191" t="s">
+      <c r="E1" s="206" t="s">
         <v>237</v>
       </c>
       <c r="F1" s="73"/>
@@ -24229,15 +24471,15 @@
       <c r="H1" s="73"/>
     </row>
     <row r="2" spans="1:8" ht="27" thickBot="1">
-      <c r="A2" s="192"/>
+      <c r="A2" s="207"/>
       <c r="B2" s="74" t="s">
         <v>234</v>
       </c>
-      <c r="C2" s="192"/>
+      <c r="C2" s="207"/>
       <c r="D2" s="74" t="s">
         <v>236</v>
       </c>
-      <c r="E2" s="192"/>
+      <c r="E2" s="207"/>
       <c r="F2" s="74" t="s">
         <v>238</v>
       </c>
@@ -24266,7 +24508,7 @@
       <c r="C4" s="79"/>
       <c r="D4" s="79"/>
       <c r="E4" s="79"/>
-      <c r="F4" s="189" t="s">
+      <c r="F4" s="196" t="s">
         <v>244</v>
       </c>
       <c r="G4" s="79"/>
@@ -24288,7 +24530,7 @@
       <c r="E5" s="80">
         <v>0</v>
       </c>
-      <c r="F5" s="190"/>
+      <c r="F5" s="198"/>
       <c r="G5" s="80" t="s">
         <v>245</v>
       </c>
@@ -24302,7 +24544,7 @@
       <c r="C6" s="79"/>
       <c r="D6" s="79"/>
       <c r="E6" s="79"/>
-      <c r="F6" s="189" t="s">
+      <c r="F6" s="196" t="s">
         <v>244</v>
       </c>
       <c r="G6" s="79"/>
@@ -24324,7 +24566,7 @@
       <c r="E7" s="80">
         <v>0</v>
       </c>
-      <c r="F7" s="190"/>
+      <c r="F7" s="198"/>
       <c r="G7" s="80" t="s">
         <v>245</v>
       </c>
@@ -24338,7 +24580,7 @@
       <c r="C8" s="79"/>
       <c r="D8" s="79"/>
       <c r="E8" s="79"/>
-      <c r="F8" s="189" t="s">
+      <c r="F8" s="196" t="s">
         <v>244</v>
       </c>
       <c r="G8" s="79"/>
@@ -24360,7 +24602,7 @@
       <c r="E9" s="80">
         <v>0</v>
       </c>
-      <c r="F9" s="190"/>
+      <c r="F9" s="198"/>
       <c r="G9" s="80" t="s">
         <v>245</v>
       </c>
@@ -24370,28 +24612,28 @@
     </row>
     <row r="10" spans="1:8" ht="24" customHeight="1" thickBot="1">
       <c r="A10" s="76"/>
-      <c r="B10" s="193" t="s">
+      <c r="B10" s="199" t="s">
         <v>249</v>
       </c>
-      <c r="C10" s="194"/>
-      <c r="D10" s="194"/>
-      <c r="E10" s="194"/>
-      <c r="F10" s="194"/>
-      <c r="G10" s="194"/>
-      <c r="H10" s="195"/>
+      <c r="C10" s="200"/>
+      <c r="D10" s="200"/>
+      <c r="E10" s="200"/>
+      <c r="F10" s="200"/>
+      <c r="G10" s="200"/>
+      <c r="H10" s="201"/>
     </row>
     <row r="11" spans="1:8">
       <c r="A11" s="82"/>
-      <c r="B11" s="189" t="s">
+      <c r="B11" s="196" t="s">
         <v>250</v>
       </c>
-      <c r="C11" s="189" t="s">
+      <c r="C11" s="196" t="s">
         <v>251</v>
       </c>
-      <c r="D11" s="189" t="s">
+      <c r="D11" s="196" t="s">
         <v>252</v>
       </c>
-      <c r="E11" s="189" t="s">
+      <c r="E11" s="196" t="s">
         <v>253</v>
       </c>
       <c r="F11" s="83"/>
@@ -24402,10 +24644,10 @@
       <c r="A12" s="78">
         <v>1</v>
       </c>
-      <c r="B12" s="190"/>
-      <c r="C12" s="190"/>
-      <c r="D12" s="190"/>
-      <c r="E12" s="190"/>
+      <c r="B12" s="198"/>
+      <c r="C12" s="198"/>
+      <c r="D12" s="198"/>
+      <c r="E12" s="198"/>
       <c r="F12" s="80" t="s">
         <v>254</v>
       </c>
@@ -24418,7 +24660,7 @@
     </row>
     <row r="13" spans="1:8">
       <c r="A13" s="82"/>
-      <c r="B13" s="189" t="s">
+      <c r="B13" s="196" t="s">
         <v>257</v>
       </c>
       <c r="C13" s="81" t="s">
@@ -24438,7 +24680,7 @@
       <c r="A14" s="84">
         <v>2</v>
       </c>
-      <c r="B14" s="196"/>
+      <c r="B14" s="197"/>
       <c r="C14" s="81" t="s">
         <v>259</v>
       </c>
@@ -24460,7 +24702,7 @@
     </row>
     <row r="15" spans="1:8" ht="17" thickBot="1">
       <c r="A15" s="85"/>
-      <c r="B15" s="190"/>
+      <c r="B15" s="198"/>
       <c r="C15" s="86"/>
       <c r="D15" s="80" t="s">
         <v>262</v>
@@ -24474,25 +24716,25 @@
     </row>
     <row r="16" spans="1:8" s="37" customFormat="1">
       <c r="A16" s="102"/>
-      <c r="B16" s="197" t="s">
+      <c r="B16" s="189" t="s">
         <v>265</v>
       </c>
-      <c r="C16" s="199">
+      <c r="C16" s="204">
         <v>0.5</v>
       </c>
-      <c r="D16" s="199">
+      <c r="D16" s="204">
         <v>0.7</v>
       </c>
-      <c r="E16" s="199">
+      <c r="E16" s="204">
         <v>0.9</v>
       </c>
-      <c r="F16" s="197" t="s">
+      <c r="F16" s="189" t="s">
         <v>254</v>
       </c>
-      <c r="G16" s="197" t="s">
+      <c r="G16" s="189" t="s">
         <v>266</v>
       </c>
-      <c r="H16" s="197" t="s">
+      <c r="H16" s="189" t="s">
         <v>256</v>
       </c>
     </row>
@@ -24500,35 +24742,35 @@
       <c r="A17" s="99">
         <v>3</v>
       </c>
-      <c r="B17" s="198"/>
-      <c r="C17" s="200"/>
-      <c r="D17" s="200"/>
-      <c r="E17" s="200"/>
-      <c r="F17" s="198"/>
-      <c r="G17" s="198"/>
-      <c r="H17" s="198"/>
+      <c r="B17" s="190"/>
+      <c r="C17" s="205"/>
+      <c r="D17" s="205"/>
+      <c r="E17" s="205"/>
+      <c r="F17" s="190"/>
+      <c r="G17" s="190"/>
+      <c r="H17" s="190"/>
     </row>
     <row r="18" spans="1:8">
       <c r="A18" s="82"/>
-      <c r="B18" s="189" t="s">
+      <c r="B18" s="196" t="s">
         <v>267</v>
       </c>
-      <c r="C18" s="189" t="s">
+      <c r="C18" s="196" t="s">
         <v>268</v>
       </c>
-      <c r="D18" s="189" t="s">
+      <c r="D18" s="196" t="s">
         <v>245</v>
       </c>
-      <c r="E18" s="189" t="s">
+      <c r="E18" s="196" t="s">
         <v>245</v>
       </c>
-      <c r="F18" s="189" t="s">
+      <c r="F18" s="196" t="s">
         <v>269</v>
       </c>
-      <c r="G18" s="189" t="s">
+      <c r="G18" s="196" t="s">
         <v>255</v>
       </c>
-      <c r="H18" s="189" t="s">
+      <c r="H18" s="196" t="s">
         <v>270</v>
       </c>
     </row>
@@ -24536,13 +24778,13 @@
       <c r="A19" s="78">
         <v>4</v>
       </c>
-      <c r="B19" s="190"/>
-      <c r="C19" s="190"/>
-      <c r="D19" s="190"/>
-      <c r="E19" s="190"/>
-      <c r="F19" s="190"/>
-      <c r="G19" s="190"/>
-      <c r="H19" s="190"/>
+      <c r="B19" s="198"/>
+      <c r="C19" s="198"/>
+      <c r="D19" s="198"/>
+      <c r="E19" s="198"/>
+      <c r="F19" s="198"/>
+      <c r="G19" s="198"/>
+      <c r="H19" s="198"/>
     </row>
     <row r="20" spans="1:8" ht="27" thickBot="1">
       <c r="A20" s="78">
@@ -24598,25 +24840,25 @@
     </row>
     <row r="22" spans="1:8" ht="17" thickBot="1">
       <c r="A22" s="88"/>
-      <c r="B22" s="193" t="s">
+      <c r="B22" s="199" t="s">
         <v>276</v>
       </c>
-      <c r="C22" s="194"/>
-      <c r="D22" s="194"/>
-      <c r="E22" s="194"/>
-      <c r="F22" s="194"/>
-      <c r="G22" s="194"/>
-      <c r="H22" s="195"/>
+      <c r="C22" s="200"/>
+      <c r="D22" s="200"/>
+      <c r="E22" s="200"/>
+      <c r="F22" s="200"/>
+      <c r="G22" s="200"/>
+      <c r="H22" s="201"/>
     </row>
     <row r="23" spans="1:8">
       <c r="A23" s="89"/>
-      <c r="B23" s="189" t="s">
+      <c r="B23" s="196" t="s">
         <v>277</v>
       </c>
       <c r="C23" s="79"/>
       <c r="D23" s="90"/>
       <c r="E23" s="79"/>
-      <c r="F23" s="189" t="s">
+      <c r="F23" s="196" t="s">
         <v>281</v>
       </c>
       <c r="G23" s="90"/>
@@ -24626,7 +24868,7 @@
       <c r="A24" s="78">
         <v>1</v>
       </c>
-      <c r="B24" s="190"/>
+      <c r="B24" s="198"/>
       <c r="C24" s="80" t="s">
         <v>278</v>
       </c>
@@ -24636,7 +24878,7 @@
       <c r="E24" s="80" t="s">
         <v>280</v>
       </c>
-      <c r="F24" s="190"/>
+      <c r="F24" s="198"/>
       <c r="G24" s="80" t="s">
         <v>282</v>
       </c>
@@ -24646,25 +24888,25 @@
     </row>
     <row r="25" spans="1:8" s="37" customFormat="1">
       <c r="A25" s="98"/>
-      <c r="B25" s="197" t="s">
+      <c r="B25" s="189" t="s">
         <v>284</v>
       </c>
-      <c r="C25" s="201">
+      <c r="C25" s="202">
         <v>2765</v>
       </c>
-      <c r="D25" s="197" t="s">
+      <c r="D25" s="189" t="s">
         <v>285</v>
       </c>
-      <c r="E25" s="197" t="s">
+      <c r="E25" s="189" t="s">
         <v>46</v>
       </c>
-      <c r="F25" s="197" t="s">
+      <c r="F25" s="189" t="s">
         <v>286</v>
       </c>
-      <c r="G25" s="197" t="s">
+      <c r="G25" s="189" t="s">
         <v>272</v>
       </c>
-      <c r="H25" s="197" t="s">
+      <c r="H25" s="189" t="s">
         <v>287</v>
       </c>
     </row>
@@ -24672,23 +24914,23 @@
       <c r="A26" s="99">
         <v>2</v>
       </c>
-      <c r="B26" s="198"/>
-      <c r="C26" s="202"/>
-      <c r="D26" s="198"/>
-      <c r="E26" s="198"/>
-      <c r="F26" s="198"/>
-      <c r="G26" s="198"/>
-      <c r="H26" s="198"/>
+      <c r="B26" s="190"/>
+      <c r="C26" s="203"/>
+      <c r="D26" s="190"/>
+      <c r="E26" s="190"/>
+      <c r="F26" s="190"/>
+      <c r="G26" s="190"/>
+      <c r="H26" s="190"/>
     </row>
     <row r="27" spans="1:8">
       <c r="A27" s="82"/>
-      <c r="B27" s="189" t="s">
+      <c r="B27" s="196" t="s">
         <v>288</v>
       </c>
       <c r="C27" s="79"/>
       <c r="D27" s="79"/>
       <c r="E27" s="79"/>
-      <c r="F27" s="189" t="s">
+      <c r="F27" s="196" t="s">
         <v>289</v>
       </c>
       <c r="G27" s="79"/>
@@ -24698,7 +24940,7 @@
       <c r="A28" s="78">
         <v>3</v>
       </c>
-      <c r="B28" s="190"/>
+      <c r="B28" s="198"/>
       <c r="C28" s="91">
         <v>3.5999999999999997E-2</v>
       </c>
@@ -24708,7 +24950,7 @@
       <c r="E28" s="92">
         <v>0.95</v>
       </c>
-      <c r="F28" s="190"/>
+      <c r="F28" s="198"/>
       <c r="G28" s="80" t="s">
         <v>272</v>
       </c>
@@ -24718,13 +24960,13 @@
     </row>
     <row r="29" spans="1:8">
       <c r="A29" s="77"/>
-      <c r="B29" s="189" t="s">
+      <c r="B29" s="196" t="s">
         <v>290</v>
       </c>
       <c r="C29" s="79"/>
       <c r="D29" s="79"/>
       <c r="E29" s="79"/>
-      <c r="F29" s="189" t="s">
+      <c r="F29" s="196" t="s">
         <v>289</v>
       </c>
       <c r="G29" s="79"/>
@@ -24734,7 +24976,7 @@
       <c r="A30" s="78">
         <v>4</v>
       </c>
-      <c r="B30" s="190"/>
+      <c r="B30" s="198"/>
       <c r="C30" s="92">
         <v>0.79</v>
       </c>
@@ -24744,7 +24986,7 @@
       <c r="E30" s="92">
         <v>0.95</v>
       </c>
-      <c r="F30" s="190"/>
+      <c r="F30" s="198"/>
       <c r="G30" s="80" t="s">
         <v>272</v>
       </c>
@@ -24818,7 +25060,7 @@
     </row>
     <row r="34" spans="1:8" s="37" customFormat="1">
       <c r="A34" s="98"/>
-      <c r="B34" s="197" t="s">
+      <c r="B34" s="189" t="s">
         <v>300</v>
       </c>
       <c r="C34" s="100" t="s">
@@ -24830,13 +25072,13 @@
       <c r="E34" s="100" t="s">
         <v>301</v>
       </c>
-      <c r="F34" s="197" t="s">
+      <c r="F34" s="189" t="s">
         <v>303</v>
       </c>
-      <c r="G34" s="197" t="s">
+      <c r="G34" s="189" t="s">
         <v>304</v>
       </c>
-      <c r="H34" s="197" t="s">
+      <c r="H34" s="189" t="s">
         <v>305</v>
       </c>
     </row>
@@ -24844,7 +25086,7 @@
       <c r="A35" s="99">
         <v>7</v>
       </c>
-      <c r="B35" s="198"/>
+      <c r="B35" s="190"/>
       <c r="C35" s="101" t="s">
         <v>302</v>
       </c>
@@ -24854,13 +25096,13 @@
       <c r="E35" s="101" t="s">
         <v>302</v>
       </c>
-      <c r="F35" s="198"/>
-      <c r="G35" s="198"/>
-      <c r="H35" s="198"/>
+      <c r="F35" s="190"/>
+      <c r="G35" s="190"/>
+      <c r="H35" s="190"/>
     </row>
     <row r="36" spans="1:8" s="37" customFormat="1">
       <c r="A36" s="98"/>
-      <c r="B36" s="197" t="s">
+      <c r="B36" s="189" t="s">
         <v>306</v>
       </c>
       <c r="C36" s="100" t="s">
@@ -24874,7 +25116,7 @@
       </c>
       <c r="F36" s="103"/>
       <c r="G36" s="103"/>
-      <c r="H36" s="197" t="s">
+      <c r="H36" s="189" t="s">
         <v>305</v>
       </c>
     </row>
@@ -24882,7 +25124,7 @@
       <c r="A37" s="99">
         <v>8</v>
       </c>
-      <c r="B37" s="198"/>
+      <c r="B37" s="190"/>
       <c r="C37" s="101" t="s">
         <v>308</v>
       </c>
@@ -24898,11 +25140,11 @@
       <c r="G37" s="101" t="s">
         <v>304</v>
       </c>
-      <c r="H37" s="198"/>
+      <c r="H37" s="190"/>
     </row>
     <row r="38" spans="1:8" s="37" customFormat="1">
       <c r="A38" s="102"/>
-      <c r="B38" s="205" t="s">
+      <c r="B38" s="191" t="s">
         <v>313</v>
       </c>
       <c r="C38" s="100" t="s">
@@ -24922,7 +25164,7 @@
       <c r="A39" s="104">
         <v>9</v>
       </c>
-      <c r="B39" s="206"/>
+      <c r="B39" s="192"/>
       <c r="C39" s="100" t="s">
         <v>315</v>
       </c>
@@ -24944,7 +25186,7 @@
     </row>
     <row r="40" spans="1:8" s="37" customFormat="1" ht="17" thickBot="1">
       <c r="A40" s="105"/>
-      <c r="B40" s="207"/>
+      <c r="B40" s="193"/>
       <c r="C40" s="101" t="s">
         <v>316</v>
       </c>
@@ -24959,10 +25201,10 @@
       <c r="H40" s="106"/>
     </row>
     <row r="41" spans="1:8">
-      <c r="A41" s="203">
+      <c r="A41" s="194">
         <v>10</v>
       </c>
-      <c r="B41" s="189" t="s">
+      <c r="B41" s="196" t="s">
         <v>321</v>
       </c>
       <c r="C41" s="81" t="s">
@@ -24974,19 +25216,19 @@
       <c r="E41" s="81" t="s">
         <v>326</v>
       </c>
-      <c r="F41" s="189" t="s">
+      <c r="F41" s="196" t="s">
         <v>303</v>
       </c>
-      <c r="G41" s="189" t="s">
+      <c r="G41" s="196" t="s">
         <v>304</v>
       </c>
-      <c r="H41" s="189" t="s">
+      <c r="H41" s="196" t="s">
         <v>305</v>
       </c>
     </row>
     <row r="42" spans="1:8" ht="26">
-      <c r="A42" s="204"/>
-      <c r="B42" s="196"/>
+      <c r="A42" s="195"/>
+      <c r="B42" s="197"/>
       <c r="C42" s="81" t="s">
         <v>323</v>
       </c>
@@ -24996,9 +25238,9 @@
       <c r="E42" s="81" t="s">
         <v>327</v>
       </c>
-      <c r="F42" s="196"/>
-      <c r="G42" s="196"/>
-      <c r="H42" s="196"/>
+      <c r="F42" s="197"/>
+      <c r="G42" s="197"/>
+      <c r="H42" s="197"/>
     </row>
     <row r="43" spans="1:8">
       <c r="A43" s="107">
@@ -25560,22 +25802,32 @@
     </row>
   </sheetData>
   <mergeCells count="52">
-    <mergeCell ref="G34:G35"/>
-    <mergeCell ref="H34:H35"/>
-    <mergeCell ref="B36:B37"/>
-    <mergeCell ref="H36:H37"/>
-    <mergeCell ref="B38:B40"/>
-    <mergeCell ref="A41:A42"/>
-    <mergeCell ref="B41:B42"/>
-    <mergeCell ref="F41:F42"/>
-    <mergeCell ref="G41:G42"/>
-    <mergeCell ref="H41:H42"/>
-    <mergeCell ref="B27:B28"/>
-    <mergeCell ref="F27:F28"/>
-    <mergeCell ref="B29:B30"/>
-    <mergeCell ref="F29:F30"/>
-    <mergeCell ref="B34:B35"/>
-    <mergeCell ref="F34:F35"/>
+    <mergeCell ref="F6:F7"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="C1:C2"/>
+    <mergeCell ref="E1:E2"/>
+    <mergeCell ref="F4:F5"/>
+    <mergeCell ref="F8:F9"/>
+    <mergeCell ref="B10:H10"/>
+    <mergeCell ref="B11:B12"/>
+    <mergeCell ref="C11:C12"/>
+    <mergeCell ref="D11:D12"/>
+    <mergeCell ref="E11:E12"/>
+    <mergeCell ref="B13:B15"/>
+    <mergeCell ref="B16:B17"/>
+    <mergeCell ref="C16:C17"/>
+    <mergeCell ref="D16:D17"/>
+    <mergeCell ref="E16:E17"/>
+    <mergeCell ref="G16:G17"/>
+    <mergeCell ref="H16:H17"/>
+    <mergeCell ref="B18:B19"/>
+    <mergeCell ref="C18:C19"/>
+    <mergeCell ref="D18:D19"/>
+    <mergeCell ref="E18:E19"/>
+    <mergeCell ref="F18:F19"/>
+    <mergeCell ref="G18:G19"/>
+    <mergeCell ref="H18:H19"/>
+    <mergeCell ref="F16:F17"/>
     <mergeCell ref="B22:H22"/>
     <mergeCell ref="B23:B24"/>
     <mergeCell ref="F23:F24"/>
@@ -25586,32 +25838,22 @@
     <mergeCell ref="F25:F26"/>
     <mergeCell ref="G25:G26"/>
     <mergeCell ref="H25:H26"/>
-    <mergeCell ref="G16:G17"/>
-    <mergeCell ref="H16:H17"/>
-    <mergeCell ref="B18:B19"/>
-    <mergeCell ref="C18:C19"/>
-    <mergeCell ref="D18:D19"/>
-    <mergeCell ref="E18:E19"/>
-    <mergeCell ref="F18:F19"/>
-    <mergeCell ref="G18:G19"/>
-    <mergeCell ref="H18:H19"/>
-    <mergeCell ref="F16:F17"/>
-    <mergeCell ref="B13:B15"/>
-    <mergeCell ref="B16:B17"/>
-    <mergeCell ref="C16:C17"/>
-    <mergeCell ref="D16:D17"/>
-    <mergeCell ref="E16:E17"/>
-    <mergeCell ref="F8:F9"/>
-    <mergeCell ref="B10:H10"/>
-    <mergeCell ref="B11:B12"/>
-    <mergeCell ref="C11:C12"/>
-    <mergeCell ref="D11:D12"/>
-    <mergeCell ref="E11:E12"/>
-    <mergeCell ref="F6:F7"/>
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="C1:C2"/>
-    <mergeCell ref="E1:E2"/>
-    <mergeCell ref="F4:F5"/>
+    <mergeCell ref="B27:B28"/>
+    <mergeCell ref="F27:F28"/>
+    <mergeCell ref="B29:B30"/>
+    <mergeCell ref="F29:F30"/>
+    <mergeCell ref="B34:B35"/>
+    <mergeCell ref="F34:F35"/>
+    <mergeCell ref="A41:A42"/>
+    <mergeCell ref="B41:B42"/>
+    <mergeCell ref="F41:F42"/>
+    <mergeCell ref="G41:G42"/>
+    <mergeCell ref="H41:H42"/>
+    <mergeCell ref="G34:G35"/>
+    <mergeCell ref="H34:H35"/>
+    <mergeCell ref="B36:B37"/>
+    <mergeCell ref="H36:H37"/>
+    <mergeCell ref="B38:B40"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -25629,26 +25871,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="9ef0ecd9-0ead-4309-8654-c6fc6a0aeea6">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="68eaa246-66f5-4d4b-bc2d-4cd6ec79d795" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100714250AEEB2AC4409DE69A29E07D1293" ma:contentTypeVersion="12" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="2c479027f39f79bf5fe77e0c13ff8fe0">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="9ef0ecd9-0ead-4309-8654-c6fc6a0aeea6" xmlns:ns3="68eaa246-66f5-4d4b-bc2d-4cd6ec79d795" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0ac27669cc00f86f1897f89f498d9d9b" ns2:_="" ns3:_="">
     <xsd:import namespace="9ef0ecd9-0ead-4309-8654-c6fc6a0aeea6"/>
@@ -25851,32 +26073,27 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{317F62B1-8FBE-489E-AF5B-00C050AC7470}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="9ef0ecd9-0ead-4309-8654-c6fc6a0aeea6"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="68eaa246-66f5-4d4b-bc2d-4cd6ec79d795"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{83D1394D-06CD-4C52-A98B-8D3C2B511CE9}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="9ef0ecd9-0ead-4309-8654-c6fc6a0aeea6">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="68eaa246-66f5-4d4b-bc2d-4cd6ec79d795" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CA56E987-09E7-4B23-987F-390DA95286EF}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -25893,4 +26110,29 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{83D1394D-06CD-4C52-A98B-8D3C2B511CE9}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{317F62B1-8FBE-489E-AF5B-00C050AC7470}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="68eaa246-66f5-4d4b-bc2d-4cd6ec79d795"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="9ef0ecd9-0ead-4309-8654-c6fc6a0aeea6"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>